<commit_message>
Update GPU prices and charts - 2026-06-12 05:45:22
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="8">
   <si>
     <t>Date</t>
   </si>
@@ -46,6 +46,9 @@
   </si>
   <si>
     <t>2026-06-11</t>
+  </si>
+  <si>
+    <t>2026-06-12</t>
   </si>
 </sst>
 </file>
@@ -162,9 +165,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>100991</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>89336</xdr:rowOff>
+      <xdr:rowOff>100913</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -182,7 +185,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8025791" cy="4347011"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -205,9 +208,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>100991</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>89336</xdr:rowOff>
+      <xdr:rowOff>100913</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -225,7 +228,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8025791" cy="4347011"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -248,9 +251,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>100991</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>89336</xdr:rowOff>
+      <xdr:rowOff>100913</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -268,7 +271,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8025791" cy="4347011"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -291,9 +294,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>93957</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>89336</xdr:rowOff>
+      <xdr:rowOff>100913</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -311,7 +314,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8018757" cy="4347011"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -336,7 +339,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>206501</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>32482</xdr:rowOff>
+      <xdr:rowOff>22957</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -377,9 +380,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>100991</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>89336</xdr:rowOff>
+      <xdr:rowOff>100913</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -397,7 +400,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8025791" cy="4347011"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -420,9 +423,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>100991</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>89336</xdr:rowOff>
+      <xdr:rowOff>100913</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -440,7 +443,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8025791" cy="4347011"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -463,9 +466,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>100991</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>89336</xdr:rowOff>
+      <xdr:rowOff>100913</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -483,7 +486,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8025791" cy="4347011"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -506,9 +509,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>100991</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>89336</xdr:rowOff>
+      <xdr:rowOff>100913</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -526,7 +529,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8025791" cy="4347011"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -549,9 +552,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>100991</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>89336</xdr:rowOff>
+      <xdr:rowOff>100913</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -569,7 +572,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8025791" cy="4347011"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -592,9 +595,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>100991</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>89336</xdr:rowOff>
+      <xdr:rowOff>100913</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -612,7 +615,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8025791" cy="4347011"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -637,7 +640,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>206501</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>32482</xdr:rowOff>
+      <xdr:rowOff>22957</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -952,7 +955,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1004,6 +1007,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="5" spans="1:3" ht="16" customHeight="1">
+      <c r="A5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="3">
+        <v>7.5</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1012,7 +1026,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1064,6 +1078,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="5" spans="1:3" ht="16" customHeight="1">
+      <c r="A5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="3">
+        <v>1.99</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1072,7 +1097,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1124,6 +1149,17 @@
         <v>1.43</v>
       </c>
     </row>
+    <row r="5" spans="1:3" ht="16" customHeight="1">
+      <c r="A5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="3">
+        <v>0.88</v>
+      </c>
+      <c r="C5" s="3">
+        <v>1.43</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1132,7 +1168,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1184,6 +1220,17 @@
         <v>0.91</v>
       </c>
     </row>
+    <row r="5" spans="1:3" ht="16" customHeight="1">
+      <c r="A5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="3">
+        <v>0.91</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1192,7 +1239,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1244,6 +1291,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="5" spans="1:3" ht="16" customHeight="1">
+      <c r="A5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1252,7 +1310,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1304,6 +1362,17 @@
         <v>4.38</v>
       </c>
     </row>
+    <row r="5" spans="1:3" ht="16" customHeight="1">
+      <c r="A5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="3">
+        <v>6.99</v>
+      </c>
+      <c r="C5" s="3">
+        <v>4.38</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1312,7 +1381,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1364,6 +1433,17 @@
         <v>3.6</v>
       </c>
     </row>
+    <row r="5" spans="1:3" ht="16" customHeight="1">
+      <c r="A5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="3">
+        <v>3.44</v>
+      </c>
+      <c r="C5" s="3">
+        <v>4.24</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1372,7 +1452,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1424,6 +1504,17 @@
         <v>3.75</v>
       </c>
     </row>
+    <row r="5" spans="1:3" ht="16" customHeight="1">
+      <c r="A5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C5" s="3">
+        <v>3.75</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1432,7 +1523,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1484,6 +1575,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="5" spans="1:3" ht="16" customHeight="1">
+      <c r="A5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="3">
+        <v>1.99</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1492,7 +1594,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1544,6 +1646,17 @@
         <v>2.67</v>
       </c>
     </row>
+    <row r="5" spans="1:3" ht="16" customHeight="1">
+      <c r="A5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="3">
+        <v>2.4</v>
+      </c>
+      <c r="C5" s="3">
+        <v>2.33</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1552,7 +1665,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1604,6 +1717,17 @@
         <v>3.07</v>
       </c>
     </row>
+    <row r="5" spans="1:3" ht="16" customHeight="1">
+      <c r="A5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1612,7 +1736,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1664,6 +1788,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="5" spans="1:3" ht="16" customHeight="1">
+      <c r="A5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-06-13 12:24:35
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="9">
   <si>
     <t>Date</t>
   </si>
@@ -49,6 +49,9 @@
   </si>
   <si>
     <t>2026-06-12</t>
+  </si>
+  <si>
+    <t>2026-06-13</t>
   </si>
 </sst>
 </file>
@@ -167,7 +170,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>100913</xdr:rowOff>
+      <xdr:rowOff>91388</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -210,7 +213,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>100913</xdr:rowOff>
+      <xdr:rowOff>91388</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -253,7 +256,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>100913</xdr:rowOff>
+      <xdr:rowOff>91388</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -296,7 +299,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>100913</xdr:rowOff>
+      <xdr:rowOff>91388</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -339,7 +342,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>206501</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>22957</xdr:rowOff>
+      <xdr:rowOff>13432</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -382,7 +385,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>100913</xdr:rowOff>
+      <xdr:rowOff>91388</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -425,7 +428,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>100913</xdr:rowOff>
+      <xdr:rowOff>91388</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -468,7 +471,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>100913</xdr:rowOff>
+      <xdr:rowOff>91388</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -511,7 +514,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>100913</xdr:rowOff>
+      <xdr:rowOff>91388</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -554,7 +557,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>100913</xdr:rowOff>
+      <xdr:rowOff>91388</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -597,7 +600,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>100913</xdr:rowOff>
+      <xdr:rowOff>91388</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -640,7 +643,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>206501</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>22957</xdr:rowOff>
+      <xdr:rowOff>13432</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -955,7 +958,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1018,6 +1021,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="6" spans="1:3" ht="16" customHeight="1">
+      <c r="A6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1026,7 +1040,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1089,6 +1103,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="6" spans="1:3" ht="16" customHeight="1">
+      <c r="A6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1097,7 +1122,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1160,6 +1185,17 @@
         <v>1.43</v>
       </c>
     </row>
+    <row r="6" spans="1:3" ht="16" customHeight="1">
+      <c r="A6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1168,7 +1204,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1231,6 +1267,17 @@
         <v>0.91</v>
       </c>
     </row>
+    <row r="6" spans="1:3" ht="16" customHeight="1">
+      <c r="A6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1239,7 +1286,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1302,6 +1349,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="6" spans="1:3" ht="16" customHeight="1">
+      <c r="A6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1310,7 +1368,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1373,6 +1431,17 @@
         <v>4.38</v>
       </c>
     </row>
+    <row r="6" spans="1:3" ht="16" customHeight="1">
+      <c r="A6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1381,7 +1450,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1444,6 +1513,17 @@
         <v>4.24</v>
       </c>
     </row>
+    <row r="6" spans="1:3" ht="16" customHeight="1">
+      <c r="A6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1452,7 +1532,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1515,6 +1595,17 @@
         <v>3.75</v>
       </c>
     </row>
+    <row r="6" spans="1:3" ht="16" customHeight="1">
+      <c r="A6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1523,7 +1614,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1586,6 +1677,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="6" spans="1:3" ht="16" customHeight="1">
+      <c r="A6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1594,7 +1696,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1657,6 +1759,17 @@
         <v>2.33</v>
       </c>
     </row>
+    <row r="6" spans="1:3" ht="16" customHeight="1">
+      <c r="A6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1665,7 +1778,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1728,6 +1841,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="6" spans="1:3" ht="16" customHeight="1">
+      <c r="A6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1736,7 +1860,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1799,6 +1923,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="6" spans="1:3" ht="16" customHeight="1">
+      <c r="A6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-06-14 07:15:29
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="10">
   <si>
     <t>Date</t>
   </si>
@@ -52,6 +52,9 @@
   </si>
   <si>
     <t>2026-06-13</t>
+  </si>
+  <si>
+    <t>2026-06-14</t>
   </si>
 </sst>
 </file>
@@ -170,7 +173,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>91388</xdr:rowOff>
+      <xdr:rowOff>81863</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -213,7 +216,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>91388</xdr:rowOff>
+      <xdr:rowOff>81863</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -256,7 +259,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>91388</xdr:rowOff>
+      <xdr:rowOff>81863</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -299,7 +302,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>91388</xdr:rowOff>
+      <xdr:rowOff>81863</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -342,7 +345,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>206501</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>13432</xdr:rowOff>
+      <xdr:rowOff>3907</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -385,7 +388,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>91388</xdr:rowOff>
+      <xdr:rowOff>81863</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -428,7 +431,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>91388</xdr:rowOff>
+      <xdr:rowOff>81863</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -471,7 +474,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>91388</xdr:rowOff>
+      <xdr:rowOff>81863</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -514,7 +517,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>91388</xdr:rowOff>
+      <xdr:rowOff>81863</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -557,7 +560,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>91388</xdr:rowOff>
+      <xdr:rowOff>81863</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -600,7 +603,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>91388</xdr:rowOff>
+      <xdr:rowOff>81863</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -643,7 +646,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>206501</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>13432</xdr:rowOff>
+      <xdr:rowOff>3907</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -958,7 +961,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1032,6 +1035,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="7" spans="1:3" ht="16" customHeight="1">
+      <c r="A7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1040,7 +1054,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1114,6 +1128,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="7" spans="1:3" ht="16" customHeight="1">
+      <c r="A7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1122,7 +1147,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1196,6 +1221,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="7" spans="1:3" ht="16" customHeight="1">
+      <c r="A7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1204,7 +1240,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1278,6 +1314,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="7" spans="1:3" ht="16" customHeight="1">
+      <c r="A7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1286,7 +1333,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1360,6 +1407,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="7" spans="1:3" ht="16" customHeight="1">
+      <c r="A7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1368,7 +1426,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1442,6 +1500,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="7" spans="1:3" ht="16" customHeight="1">
+      <c r="A7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1450,7 +1519,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1524,6 +1593,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="7" spans="1:3" ht="16" customHeight="1">
+      <c r="A7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1532,7 +1612,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1606,6 +1686,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="7" spans="1:3" ht="16" customHeight="1">
+      <c r="A7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1614,7 +1705,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1688,6 +1779,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="7" spans="1:3" ht="16" customHeight="1">
+      <c r="A7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1696,7 +1798,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1770,6 +1872,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="7" spans="1:3" ht="16" customHeight="1">
+      <c r="A7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1778,7 +1891,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1852,6 +1965,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="7" spans="1:3" ht="16" customHeight="1">
+      <c r="A7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1860,7 +1984,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1934,6 +2058,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="7" spans="1:3" ht="16" customHeight="1">
+      <c r="A7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-06-15 08:48:11
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="11">
   <si>
     <t>Date</t>
   </si>
@@ -55,6 +55,9 @@
   </si>
   <si>
     <t>2026-06-14</t>
+  </si>
+  <si>
+    <t>2026-06-15</t>
   </si>
 </sst>
 </file>
@@ -173,7 +176,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>81863</xdr:rowOff>
+      <xdr:rowOff>72338</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -216,7 +219,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>81863</xdr:rowOff>
+      <xdr:rowOff>72338</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -259,7 +262,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>81863</xdr:rowOff>
+      <xdr:rowOff>72338</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -302,7 +305,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>81863</xdr:rowOff>
+      <xdr:rowOff>72338</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -344,8 +347,8 @@
     <xdr:to>
       <xdr:col>17</xdr:col>
       <xdr:colOff>206501</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>3907</xdr:rowOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>184882</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -388,7 +391,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>81863</xdr:rowOff>
+      <xdr:rowOff>72338</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -431,7 +434,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>81863</xdr:rowOff>
+      <xdr:rowOff>72338</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -474,7 +477,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>81863</xdr:rowOff>
+      <xdr:rowOff>72338</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -517,7 +520,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>81863</xdr:rowOff>
+      <xdr:rowOff>72338</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -560,7 +563,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>81863</xdr:rowOff>
+      <xdr:rowOff>72338</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -603,7 +606,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>81863</xdr:rowOff>
+      <xdr:rowOff>72338</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -645,8 +648,8 @@
     <xdr:to>
       <xdr:col>17</xdr:col>
       <xdr:colOff>206501</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>3907</xdr:rowOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>184882</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -961,7 +964,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1046,6 +1049,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="8" spans="1:3" ht="16" customHeight="1">
+      <c r="A8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1054,7 +1068,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1139,6 +1153,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="8" spans="1:3" ht="16" customHeight="1">
+      <c r="A8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1147,7 +1172,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1232,6 +1257,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="8" spans="1:3" ht="16" customHeight="1">
+      <c r="A8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1240,7 +1276,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1325,6 +1361,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="8" spans="1:3" ht="16" customHeight="1">
+      <c r="A8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1333,7 +1380,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1418,6 +1465,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="8" spans="1:3" ht="16" customHeight="1">
+      <c r="A8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1426,7 +1484,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1511,6 +1569,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="8" spans="1:3" ht="16" customHeight="1">
+      <c r="A8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1519,7 +1588,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1604,6 +1673,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="8" spans="1:3" ht="16" customHeight="1">
+      <c r="A8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1612,7 +1692,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1697,6 +1777,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="8" spans="1:3" ht="16" customHeight="1">
+      <c r="A8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1705,7 +1796,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1790,6 +1881,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="8" spans="1:3" ht="16" customHeight="1">
+      <c r="A8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1798,7 +1900,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1883,6 +1985,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="8" spans="1:3" ht="16" customHeight="1">
+      <c r="A8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1891,7 +2004,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1976,6 +2089,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="8" spans="1:3" ht="16" customHeight="1">
+      <c r="A8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1984,7 +2108,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2069,6 +2193,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="8" spans="1:3" ht="16" customHeight="1">
+      <c r="A8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-06-16 08:38:33
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="12">
   <si>
     <t>Date</t>
   </si>
@@ -58,6 +58,9 @@
   </si>
   <si>
     <t>2026-06-15</t>
+  </si>
+  <si>
+    <t>2026-06-16</t>
   </si>
 </sst>
 </file>
@@ -176,7 +179,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>72338</xdr:rowOff>
+      <xdr:rowOff>62813</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -219,7 +222,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>72338</xdr:rowOff>
+      <xdr:rowOff>62813</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -262,7 +265,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>72338</xdr:rowOff>
+      <xdr:rowOff>62813</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -305,7 +308,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>72338</xdr:rowOff>
+      <xdr:rowOff>62813</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -348,7 +351,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>206501</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>184882</xdr:rowOff>
+      <xdr:rowOff>175357</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -391,7 +394,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>72338</xdr:rowOff>
+      <xdr:rowOff>62813</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -434,7 +437,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>72338</xdr:rowOff>
+      <xdr:rowOff>62813</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -477,7 +480,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>72338</xdr:rowOff>
+      <xdr:rowOff>62813</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -520,7 +523,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>72338</xdr:rowOff>
+      <xdr:rowOff>62813</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -563,7 +566,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>72338</xdr:rowOff>
+      <xdr:rowOff>62813</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -606,7 +609,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>72338</xdr:rowOff>
+      <xdr:rowOff>62813</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -649,7 +652,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>206501</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>184882</xdr:rowOff>
+      <xdr:rowOff>175357</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -964,7 +967,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1060,6 +1063,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="9" spans="1:3" ht="16" customHeight="1">
+      <c r="A9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1068,7 +1082,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1164,6 +1178,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="9" spans="1:3" ht="16" customHeight="1">
+      <c r="A9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1172,7 +1197,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1268,6 +1293,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="9" spans="1:3" ht="16" customHeight="1">
+      <c r="A9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1276,7 +1312,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1372,6 +1408,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="9" spans="1:3" ht="16" customHeight="1">
+      <c r="A9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1380,7 +1427,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1476,6 +1523,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="9" spans="1:3" ht="16" customHeight="1">
+      <c r="A9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1484,7 +1542,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1580,6 +1638,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="9" spans="1:3" ht="16" customHeight="1">
+      <c r="A9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1588,7 +1657,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1684,6 +1753,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="9" spans="1:3" ht="16" customHeight="1">
+      <c r="A9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1692,7 +1772,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1788,6 +1868,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="9" spans="1:3" ht="16" customHeight="1">
+      <c r="A9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1796,7 +1887,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1892,6 +1983,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="9" spans="1:3" ht="16" customHeight="1">
+      <c r="A9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1900,7 +2002,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1996,6 +2098,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="9" spans="1:3" ht="16" customHeight="1">
+      <c r="A9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2004,7 +2117,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2100,6 +2213,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="9" spans="1:3" ht="16" customHeight="1">
+      <c r="A9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2108,7 +2232,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2204,6 +2328,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="9" spans="1:3" ht="16" customHeight="1">
+      <c r="A9" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-06-17 08:21:25
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="13">
   <si>
     <t>Date</t>
   </si>
@@ -61,6 +61,9 @@
   </si>
   <si>
     <t>2026-06-16</t>
+  </si>
+  <si>
+    <t>2026-06-17</t>
   </si>
 </sst>
 </file>
@@ -179,7 +182,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>62813</xdr:rowOff>
+      <xdr:rowOff>53288</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -222,7 +225,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>62813</xdr:rowOff>
+      <xdr:rowOff>53288</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -265,7 +268,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>62813</xdr:rowOff>
+      <xdr:rowOff>53288</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -308,7 +311,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>62813</xdr:rowOff>
+      <xdr:rowOff>53288</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -351,7 +354,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>206501</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>175357</xdr:rowOff>
+      <xdr:rowOff>165832</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -394,7 +397,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>62813</xdr:rowOff>
+      <xdr:rowOff>53288</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -437,7 +440,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>62813</xdr:rowOff>
+      <xdr:rowOff>53288</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -480,7 +483,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>62813</xdr:rowOff>
+      <xdr:rowOff>53288</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -523,7 +526,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>62813</xdr:rowOff>
+      <xdr:rowOff>53288</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -566,7 +569,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>62813</xdr:rowOff>
+      <xdr:rowOff>53288</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -609,7 +612,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>62813</xdr:rowOff>
+      <xdr:rowOff>53288</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -652,7 +655,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>206501</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>175357</xdr:rowOff>
+      <xdr:rowOff>165832</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -967,7 +970,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1074,6 +1077,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="10" spans="1:3" ht="16" customHeight="1">
+      <c r="A10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1082,7 +1096,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1189,6 +1203,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="10" spans="1:3" ht="16" customHeight="1">
+      <c r="A10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1197,7 +1222,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1304,6 +1329,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="10" spans="1:3" ht="16" customHeight="1">
+      <c r="A10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1312,7 +1348,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1419,6 +1455,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="10" spans="1:3" ht="16" customHeight="1">
+      <c r="A10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1427,7 +1474,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1534,6 +1581,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="10" spans="1:3" ht="16" customHeight="1">
+      <c r="A10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1542,7 +1600,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1649,6 +1707,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="10" spans="1:3" ht="16" customHeight="1">
+      <c r="A10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1657,7 +1726,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1764,6 +1833,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="10" spans="1:3" ht="16" customHeight="1">
+      <c r="A10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1772,7 +1852,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1879,6 +1959,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="10" spans="1:3" ht="16" customHeight="1">
+      <c r="A10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1887,7 +1978,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1994,6 +2085,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="10" spans="1:3" ht="16" customHeight="1">
+      <c r="A10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2002,7 +2104,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2109,6 +2211,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="10" spans="1:3" ht="16" customHeight="1">
+      <c r="A10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2117,7 +2230,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2224,6 +2337,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="10" spans="1:3" ht="16" customHeight="1">
+      <c r="A10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2232,7 +2356,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2339,6 +2463,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="10" spans="1:3" ht="16" customHeight="1">
+      <c r="A10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-06-18 13:56:50
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="14">
   <si>
     <t>Date</t>
   </si>
@@ -64,6 +64,9 @@
   </si>
   <si>
     <t>2026-06-17</t>
+  </si>
+  <si>
+    <t>2026-06-18</t>
   </si>
 </sst>
 </file>
@@ -182,7 +185,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>53288</xdr:rowOff>
+      <xdr:rowOff>43763</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -225,7 +228,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>53288</xdr:rowOff>
+      <xdr:rowOff>43763</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -268,7 +271,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>53288</xdr:rowOff>
+      <xdr:rowOff>43763</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -311,7 +314,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>53288</xdr:rowOff>
+      <xdr:rowOff>43763</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -354,7 +357,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>206501</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>165832</xdr:rowOff>
+      <xdr:rowOff>156307</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -397,7 +400,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>53288</xdr:rowOff>
+      <xdr:rowOff>43763</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -440,7 +443,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>53288</xdr:rowOff>
+      <xdr:rowOff>43763</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -483,7 +486,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>53288</xdr:rowOff>
+      <xdr:rowOff>43763</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -526,7 +529,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>53288</xdr:rowOff>
+      <xdr:rowOff>43763</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -569,7 +572,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>53288</xdr:rowOff>
+      <xdr:rowOff>43763</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -612,7 +615,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>53288</xdr:rowOff>
+      <xdr:rowOff>43763</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -655,7 +658,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>206501</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>165832</xdr:rowOff>
+      <xdr:rowOff>156307</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -970,7 +973,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1088,6 +1091,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="11" spans="1:3" ht="16" customHeight="1">
+      <c r="A11" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1096,7 +1110,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1214,6 +1228,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="11" spans="1:3" ht="16" customHeight="1">
+      <c r="A11" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1222,7 +1247,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1340,6 +1365,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="11" spans="1:3" ht="16" customHeight="1">
+      <c r="A11" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1348,7 +1384,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1466,6 +1502,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="11" spans="1:3" ht="16" customHeight="1">
+      <c r="A11" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1474,7 +1521,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1592,6 +1639,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="11" spans="1:3" ht="16" customHeight="1">
+      <c r="A11" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1600,7 +1658,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1718,6 +1776,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="11" spans="1:3" ht="16" customHeight="1">
+      <c r="A11" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1726,7 +1795,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1844,6 +1913,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="11" spans="1:3" ht="16" customHeight="1">
+      <c r="A11" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1852,7 +1932,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1970,6 +2050,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="11" spans="1:3" ht="16" customHeight="1">
+      <c r="A11" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1978,7 +2069,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2096,6 +2187,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="11" spans="1:3" ht="16" customHeight="1">
+      <c r="A11" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2104,7 +2206,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2222,6 +2324,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="11" spans="1:3" ht="16" customHeight="1">
+      <c r="A11" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2230,7 +2343,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2348,6 +2461,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="11" spans="1:3" ht="16" customHeight="1">
+      <c r="A11" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2356,7 +2480,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2474,6 +2598,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="11" spans="1:3" ht="16" customHeight="1">
+      <c r="A11" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-06-19 13:59:09
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="15">
   <si>
     <t>Date</t>
   </si>
@@ -67,6 +67,9 @@
   </si>
   <si>
     <t>2026-06-18</t>
+  </si>
+  <si>
+    <t>2026-06-19</t>
   </si>
 </sst>
 </file>
@@ -185,7 +188,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>43763</xdr:rowOff>
+      <xdr:rowOff>34238</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -228,7 +231,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>43763</xdr:rowOff>
+      <xdr:rowOff>34238</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -271,7 +274,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>43763</xdr:rowOff>
+      <xdr:rowOff>34238</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -314,7 +317,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>43763</xdr:rowOff>
+      <xdr:rowOff>34238</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -357,7 +360,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>206501</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>156307</xdr:rowOff>
+      <xdr:rowOff>146782</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -400,7 +403,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>43763</xdr:rowOff>
+      <xdr:rowOff>34238</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -443,7 +446,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>43763</xdr:rowOff>
+      <xdr:rowOff>34238</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -486,7 +489,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>43763</xdr:rowOff>
+      <xdr:rowOff>34238</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -529,7 +532,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>43763</xdr:rowOff>
+      <xdr:rowOff>34238</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -572,7 +575,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>43763</xdr:rowOff>
+      <xdr:rowOff>34238</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -615,7 +618,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>43763</xdr:rowOff>
+      <xdr:rowOff>34238</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -658,7 +661,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>206501</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>156307</xdr:rowOff>
+      <xdr:rowOff>146782</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -973,7 +976,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1102,6 +1105,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="12" spans="1:3" ht="16" customHeight="1">
+      <c r="A12" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1110,7 +1124,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1239,6 +1253,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="12" spans="1:3" ht="16" customHeight="1">
+      <c r="A12" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1247,7 +1272,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1376,6 +1401,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="12" spans="1:3" ht="16" customHeight="1">
+      <c r="A12" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1384,7 +1420,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1513,6 +1549,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="12" spans="1:3" ht="16" customHeight="1">
+      <c r="A12" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1521,7 +1568,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1650,6 +1697,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="12" spans="1:3" ht="16" customHeight="1">
+      <c r="A12" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1658,7 +1716,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1787,6 +1845,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="12" spans="1:3" ht="16" customHeight="1">
+      <c r="A12" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1795,7 +1864,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1924,6 +1993,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="12" spans="1:3" ht="16" customHeight="1">
+      <c r="A12" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1932,7 +2012,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2061,6 +2141,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="12" spans="1:3" ht="16" customHeight="1">
+      <c r="A12" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2069,7 +2160,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2198,6 +2289,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="12" spans="1:3" ht="16" customHeight="1">
+      <c r="A12" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2206,7 +2308,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2335,6 +2437,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="12" spans="1:3" ht="16" customHeight="1">
+      <c r="A12" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2343,7 +2456,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2472,6 +2585,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="12" spans="1:3" ht="16" customHeight="1">
+      <c r="A12" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2480,7 +2604,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2609,6 +2733,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="12" spans="1:3" ht="16" customHeight="1">
+      <c r="A12" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-06-20 12:23:41
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="412" uniqueCount="16">
   <si>
     <t>Date</t>
   </si>
@@ -70,6 +70,9 @@
   </si>
   <si>
     <t>2026-06-19</t>
+  </si>
+  <si>
+    <t>2026-06-20</t>
   </si>
 </sst>
 </file>
@@ -188,7 +191,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>34238</xdr:rowOff>
+      <xdr:rowOff>24713</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -231,7 +234,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>34238</xdr:rowOff>
+      <xdr:rowOff>24713</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -274,7 +277,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>34238</xdr:rowOff>
+      <xdr:rowOff>24713</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -317,7 +320,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>34238</xdr:rowOff>
+      <xdr:rowOff>24713</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -360,7 +363,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>206501</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>146782</xdr:rowOff>
+      <xdr:rowOff>137257</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -403,7 +406,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>34238</xdr:rowOff>
+      <xdr:rowOff>24713</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -446,7 +449,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>34238</xdr:rowOff>
+      <xdr:rowOff>24713</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -489,7 +492,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>34238</xdr:rowOff>
+      <xdr:rowOff>24713</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -532,7 +535,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>34238</xdr:rowOff>
+      <xdr:rowOff>24713</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -575,7 +578,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>34238</xdr:rowOff>
+      <xdr:rowOff>24713</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -618,7 +621,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>34238</xdr:rowOff>
+      <xdr:rowOff>24713</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -661,7 +664,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>206501</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>146782</xdr:rowOff>
+      <xdr:rowOff>137257</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -976,7 +979,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1116,6 +1119,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="13" spans="1:3" ht="16" customHeight="1">
+      <c r="A13" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1124,7 +1138,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1264,6 +1278,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="13" spans="1:3" ht="16" customHeight="1">
+      <c r="A13" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1272,7 +1297,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1412,6 +1437,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="13" spans="1:3" ht="16" customHeight="1">
+      <c r="A13" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1420,7 +1456,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1560,6 +1596,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="13" spans="1:3" ht="16" customHeight="1">
+      <c r="A13" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1568,7 +1615,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1708,6 +1755,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="13" spans="1:3" ht="16" customHeight="1">
+      <c r="A13" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1716,7 +1774,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1856,6 +1914,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="13" spans="1:3" ht="16" customHeight="1">
+      <c r="A13" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1864,7 +1933,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2004,6 +2073,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="13" spans="1:3" ht="16" customHeight="1">
+      <c r="A13" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2012,7 +2092,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2152,6 +2232,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="13" spans="1:3" ht="16" customHeight="1">
+      <c r="A13" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2160,7 +2251,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2300,6 +2391,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="13" spans="1:3" ht="16" customHeight="1">
+      <c r="A13" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2308,7 +2410,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2448,6 +2550,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="13" spans="1:3" ht="16" customHeight="1">
+      <c r="A13" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2456,7 +2569,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2596,6 +2709,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="13" spans="1:3" ht="16" customHeight="1">
+      <c r="A13" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2604,7 +2728,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2744,6 +2868,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="13" spans="1:3" ht="16" customHeight="1">
+      <c r="A13" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-06-21 13:01:35
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="412" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="17">
   <si>
     <t>Date</t>
   </si>
@@ -73,6 +73,9 @@
   </si>
   <si>
     <t>2026-06-20</t>
+  </si>
+  <si>
+    <t>2026-06-21</t>
   </si>
 </sst>
 </file>
@@ -191,7 +194,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>24713</xdr:rowOff>
+      <xdr:rowOff>15188</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -234,7 +237,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>24713</xdr:rowOff>
+      <xdr:rowOff>15188</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -277,7 +280,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>24713</xdr:rowOff>
+      <xdr:rowOff>15188</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -320,7 +323,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>24713</xdr:rowOff>
+      <xdr:rowOff>15188</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -363,7 +366,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>206501</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>137257</xdr:rowOff>
+      <xdr:rowOff>127732</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -406,7 +409,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>24713</xdr:rowOff>
+      <xdr:rowOff>15188</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -449,7 +452,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>24713</xdr:rowOff>
+      <xdr:rowOff>15188</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -492,7 +495,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>24713</xdr:rowOff>
+      <xdr:rowOff>15188</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -535,7 +538,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>24713</xdr:rowOff>
+      <xdr:rowOff>15188</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -578,7 +581,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>24713</xdr:rowOff>
+      <xdr:rowOff>15188</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -621,7 +624,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>24713</xdr:rowOff>
+      <xdr:rowOff>15188</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -664,7 +667,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>206501</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>137257</xdr:rowOff>
+      <xdr:rowOff>127732</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -979,7 +982,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1130,6 +1133,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="14" spans="1:3" ht="16" customHeight="1">
+      <c r="A14" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1138,7 +1152,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1289,6 +1303,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="14" spans="1:3" ht="16" customHeight="1">
+      <c r="A14" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1297,7 +1322,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1448,6 +1473,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="14" spans="1:3" ht="16" customHeight="1">
+      <c r="A14" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1456,7 +1492,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1607,6 +1643,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="14" spans="1:3" ht="16" customHeight="1">
+      <c r="A14" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1615,7 +1662,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1766,6 +1813,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="14" spans="1:3" ht="16" customHeight="1">
+      <c r="A14" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1774,7 +1832,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1925,6 +1983,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="14" spans="1:3" ht="16" customHeight="1">
+      <c r="A14" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1933,7 +2002,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2084,6 +2153,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="14" spans="1:3" ht="16" customHeight="1">
+      <c r="A14" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2092,7 +2172,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2243,6 +2323,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="14" spans="1:3" ht="16" customHeight="1">
+      <c r="A14" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2251,7 +2342,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2402,6 +2493,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="14" spans="1:3" ht="16" customHeight="1">
+      <c r="A14" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2410,7 +2512,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2561,6 +2663,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="14" spans="1:3" ht="16" customHeight="1">
+      <c r="A14" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2569,7 +2682,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2720,6 +2833,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="14" spans="1:3" ht="16" customHeight="1">
+      <c r="A14" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2728,7 +2852,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2879,6 +3003,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="14" spans="1:3" ht="16" customHeight="1">
+      <c r="A14" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-06-22 15:48:05
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="18">
   <si>
     <t>Date</t>
   </si>
@@ -76,6 +76,9 @@
   </si>
   <si>
     <t>2026-06-21</t>
+  </si>
+  <si>
+    <t>2026-06-22</t>
   </si>
 </sst>
 </file>
@@ -194,7 +197,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>15188</xdr:rowOff>
+      <xdr:rowOff>5663</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -237,7 +240,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>15188</xdr:rowOff>
+      <xdr:rowOff>5663</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -280,7 +283,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>15188</xdr:rowOff>
+      <xdr:rowOff>5663</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -323,7 +326,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>15188</xdr:rowOff>
+      <xdr:rowOff>5663</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -366,7 +369,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>206501</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>127732</xdr:rowOff>
+      <xdr:rowOff>118207</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -409,7 +412,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>15188</xdr:rowOff>
+      <xdr:rowOff>5663</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -452,7 +455,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>15188</xdr:rowOff>
+      <xdr:rowOff>5663</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -495,7 +498,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>15188</xdr:rowOff>
+      <xdr:rowOff>5663</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -538,7 +541,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>15188</xdr:rowOff>
+      <xdr:rowOff>5663</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -581,7 +584,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>15188</xdr:rowOff>
+      <xdr:rowOff>5663</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -624,7 +627,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>15188</xdr:rowOff>
+      <xdr:rowOff>5663</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -667,7 +670,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>206501</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>127732</xdr:rowOff>
+      <xdr:rowOff>118207</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -982,7 +985,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1144,6 +1147,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="15" spans="1:3" ht="16" customHeight="1">
+      <c r="A15" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1152,7 +1166,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1314,6 +1328,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="15" spans="1:3" ht="16" customHeight="1">
+      <c r="A15" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1322,7 +1347,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1484,6 +1509,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="15" spans="1:3" ht="16" customHeight="1">
+      <c r="A15" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1492,7 +1528,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1654,6 +1690,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="15" spans="1:3" ht="16" customHeight="1">
+      <c r="A15" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1662,7 +1709,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1824,6 +1871,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="15" spans="1:3" ht="16" customHeight="1">
+      <c r="A15" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1832,7 +1890,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1994,6 +2052,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="15" spans="1:3" ht="16" customHeight="1">
+      <c r="A15" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2002,7 +2071,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2164,6 +2233,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="15" spans="1:3" ht="16" customHeight="1">
+      <c r="A15" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2172,7 +2252,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2334,6 +2414,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="15" spans="1:3" ht="16" customHeight="1">
+      <c r="A15" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2342,7 +2433,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2504,6 +2595,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="15" spans="1:3" ht="16" customHeight="1">
+      <c r="A15" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2512,7 +2614,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2674,6 +2776,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="15" spans="1:3" ht="16" customHeight="1">
+      <c r="A15" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2682,7 +2795,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2844,6 +2957,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="15" spans="1:3" ht="16" customHeight="1">
+      <c r="A15" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2852,7 +2976,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3014,6 +3138,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="15" spans="1:3" ht="16" customHeight="1">
+      <c r="A15" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-06-23 13:37:28
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="520" uniqueCount="19">
   <si>
     <t>Date</t>
   </si>
@@ -79,6 +79,9 @@
   </si>
   <si>
     <t>2026-06-22</t>
+  </si>
+  <si>
+    <t>2026-06-23</t>
   </si>
 </sst>
 </file>
@@ -196,8 +199,8 @@
     <xdr:to>
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>5663</xdr:rowOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>186638</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -239,8 +242,8 @@
     <xdr:to>
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>5663</xdr:rowOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>186638</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -282,8 +285,8 @@
     <xdr:to>
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>5663</xdr:rowOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>186638</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -325,8 +328,8 @@
     <xdr:to>
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>5663</xdr:rowOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>186638</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -369,7 +372,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>206501</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>118207</xdr:rowOff>
+      <xdr:rowOff>108682</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -411,8 +414,8 @@
     <xdr:to>
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>5663</xdr:rowOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>186638</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -454,8 +457,8 @@
     <xdr:to>
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>5663</xdr:rowOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>186638</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -497,8 +500,8 @@
     <xdr:to>
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>5663</xdr:rowOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>186638</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -540,8 +543,8 @@
     <xdr:to>
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>5663</xdr:rowOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>186638</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -583,8 +586,8 @@
     <xdr:to>
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>5663</xdr:rowOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>186638</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -626,8 +629,8 @@
     <xdr:to>
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>5663</xdr:rowOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>186638</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -670,7 +673,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>206501</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>118207</xdr:rowOff>
+      <xdr:rowOff>108682</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -985,7 +988,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1158,6 +1161,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="16" spans="1:3" ht="16" customHeight="1">
+      <c r="A16" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1166,7 +1180,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1339,6 +1353,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="16" spans="1:3" ht="16" customHeight="1">
+      <c r="A16" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1347,7 +1372,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1520,6 +1545,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="16" spans="1:3" ht="16" customHeight="1">
+      <c r="A16" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1528,7 +1564,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1701,6 +1737,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="16" spans="1:3" ht="16" customHeight="1">
+      <c r="A16" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1709,7 +1756,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1882,6 +1929,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="16" spans="1:3" ht="16" customHeight="1">
+      <c r="A16" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1890,7 +1948,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2063,6 +2121,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="16" spans="1:3" ht="16" customHeight="1">
+      <c r="A16" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2071,7 +2140,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2244,6 +2313,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="16" spans="1:3" ht="16" customHeight="1">
+      <c r="A16" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2252,7 +2332,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2425,6 +2505,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="16" spans="1:3" ht="16" customHeight="1">
+      <c r="A16" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2433,7 +2524,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2606,6 +2697,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="16" spans="1:3" ht="16" customHeight="1">
+      <c r="A16" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2614,7 +2716,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2787,6 +2889,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="16" spans="1:3" ht="16" customHeight="1">
+      <c r="A16" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2795,7 +2908,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2968,6 +3081,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="16" spans="1:3" ht="16" customHeight="1">
+      <c r="A16" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2976,7 +3100,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3149,6 +3273,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="16" spans="1:3" ht="16" customHeight="1">
+      <c r="A16" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-06-24 13:11:21
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="520" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="556" uniqueCount="20">
   <si>
     <t>Date</t>
   </si>
@@ -82,6 +82,9 @@
   </si>
   <si>
     <t>2026-06-23</t>
+  </si>
+  <si>
+    <t>2026-06-24</t>
   </si>
 </sst>
 </file>
@@ -200,7 +203,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>186638</xdr:rowOff>
+      <xdr:rowOff>177113</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -243,7 +246,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>186638</xdr:rowOff>
+      <xdr:rowOff>177113</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -286,7 +289,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>186638</xdr:rowOff>
+      <xdr:rowOff>177113</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -329,7 +332,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>186638</xdr:rowOff>
+      <xdr:rowOff>177113</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -372,7 +375,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>206501</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>108682</xdr:rowOff>
+      <xdr:rowOff>99157</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -415,7 +418,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>186638</xdr:rowOff>
+      <xdr:rowOff>177113</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -458,7 +461,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>186638</xdr:rowOff>
+      <xdr:rowOff>177113</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -501,7 +504,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>186638</xdr:rowOff>
+      <xdr:rowOff>177113</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -544,7 +547,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>186638</xdr:rowOff>
+      <xdr:rowOff>177113</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -587,7 +590,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>186638</xdr:rowOff>
+      <xdr:rowOff>177113</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -630,7 +633,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>186638</xdr:rowOff>
+      <xdr:rowOff>177113</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -673,7 +676,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>206501</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>108682</xdr:rowOff>
+      <xdr:rowOff>99157</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -988,7 +991,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1172,6 +1175,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="17" spans="1:3" ht="16" customHeight="1">
+      <c r="A17" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1180,7 +1194,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1364,6 +1378,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="17" spans="1:3" ht="16" customHeight="1">
+      <c r="A17" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1372,7 +1397,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1556,6 +1581,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="17" spans="1:3" ht="16" customHeight="1">
+      <c r="A17" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1564,7 +1600,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1748,6 +1784,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="17" spans="1:3" ht="16" customHeight="1">
+      <c r="A17" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1756,7 +1803,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1940,6 +1987,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="17" spans="1:3" ht="16" customHeight="1">
+      <c r="A17" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1948,7 +2006,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2132,6 +2190,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="17" spans="1:3" ht="16" customHeight="1">
+      <c r="A17" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2140,7 +2209,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2324,6 +2393,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="17" spans="1:3" ht="16" customHeight="1">
+      <c r="A17" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2332,7 +2412,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2516,6 +2596,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="17" spans="1:3" ht="16" customHeight="1">
+      <c r="A17" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2524,7 +2615,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2708,6 +2799,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="17" spans="1:3" ht="16" customHeight="1">
+      <c r="A17" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2716,7 +2818,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2900,6 +3002,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="17" spans="1:3" ht="16" customHeight="1">
+      <c r="A17" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2908,7 +3021,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3092,6 +3205,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="17" spans="1:3" ht="16" customHeight="1">
+      <c r="A17" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3100,7 +3224,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3284,6 +3408,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="17" spans="1:3" ht="16" customHeight="1">
+      <c r="A17" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-06-25 13:10:24
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="556" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="21">
   <si>
     <t>Date</t>
   </si>
@@ -85,6 +85,9 @@
   </si>
   <si>
     <t>2026-06-24</t>
+  </si>
+  <si>
+    <t>2026-06-25</t>
   </si>
 </sst>
 </file>
@@ -203,7 +206,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>177113</xdr:rowOff>
+      <xdr:rowOff>167588</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -246,7 +249,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>177113</xdr:rowOff>
+      <xdr:rowOff>167588</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -289,7 +292,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>177113</xdr:rowOff>
+      <xdr:rowOff>167588</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -332,7 +335,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>177113</xdr:rowOff>
+      <xdr:rowOff>167588</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -375,7 +378,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>206501</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>99157</xdr:rowOff>
+      <xdr:rowOff>89632</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -418,7 +421,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>177113</xdr:rowOff>
+      <xdr:rowOff>167588</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -461,7 +464,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>177113</xdr:rowOff>
+      <xdr:rowOff>167588</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -504,7 +507,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>177113</xdr:rowOff>
+      <xdr:rowOff>167588</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -547,7 +550,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>177113</xdr:rowOff>
+      <xdr:rowOff>167588</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -590,7 +593,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>177113</xdr:rowOff>
+      <xdr:rowOff>167588</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -633,7 +636,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>177113</xdr:rowOff>
+      <xdr:rowOff>167588</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -676,7 +679,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>206501</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>99157</xdr:rowOff>
+      <xdr:rowOff>89632</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -991,7 +994,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1186,6 +1189,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="18" spans="1:3" ht="16" customHeight="1">
+      <c r="A18" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1194,7 +1208,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1389,6 +1403,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="18" spans="1:3" ht="16" customHeight="1">
+      <c r="A18" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1397,7 +1422,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1592,6 +1617,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="18" spans="1:3" ht="16" customHeight="1">
+      <c r="A18" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1600,7 +1636,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1795,6 +1831,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="18" spans="1:3" ht="16" customHeight="1">
+      <c r="A18" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1803,7 +1850,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1998,6 +2045,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="18" spans="1:3" ht="16" customHeight="1">
+      <c r="A18" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2006,7 +2064,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2201,6 +2259,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="18" spans="1:3" ht="16" customHeight="1">
+      <c r="A18" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2209,7 +2278,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2404,6 +2473,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="18" spans="1:3" ht="16" customHeight="1">
+      <c r="A18" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2412,7 +2492,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2607,6 +2687,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="18" spans="1:3" ht="16" customHeight="1">
+      <c r="A18" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2615,7 +2706,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2810,6 +2901,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="18" spans="1:3" ht="16" customHeight="1">
+      <c r="A18" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2818,7 +2920,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3013,6 +3115,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="18" spans="1:3" ht="16" customHeight="1">
+      <c r="A18" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3021,7 +3134,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3216,6 +3329,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="18" spans="1:3" ht="16" customHeight="1">
+      <c r="A18" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3224,7 +3348,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3419,6 +3543,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="18" spans="1:3" ht="16" customHeight="1">
+      <c r="A18" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-06-26 13:02:50
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="628" uniqueCount="22">
   <si>
     <t>Date</t>
   </si>
@@ -88,6 +88,9 @@
   </si>
   <si>
     <t>2026-06-25</t>
+  </si>
+  <si>
+    <t>2026-06-26</t>
   </si>
 </sst>
 </file>
@@ -206,7 +209,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>167588</xdr:rowOff>
+      <xdr:rowOff>158063</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -249,7 +252,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>167588</xdr:rowOff>
+      <xdr:rowOff>158063</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -292,7 +295,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>167588</xdr:rowOff>
+      <xdr:rowOff>158063</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -335,7 +338,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>167588</xdr:rowOff>
+      <xdr:rowOff>158063</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -378,7 +381,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>206501</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>89632</xdr:rowOff>
+      <xdr:rowOff>80107</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -421,7 +424,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>167588</xdr:rowOff>
+      <xdr:rowOff>158063</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -464,7 +467,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>167588</xdr:rowOff>
+      <xdr:rowOff>158063</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -507,7 +510,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>167588</xdr:rowOff>
+      <xdr:rowOff>158063</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -550,7 +553,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>167588</xdr:rowOff>
+      <xdr:rowOff>158063</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -593,7 +596,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>167588</xdr:rowOff>
+      <xdr:rowOff>158063</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -636,7 +639,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>167588</xdr:rowOff>
+      <xdr:rowOff>158063</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -679,7 +682,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>206501</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>89632</xdr:rowOff>
+      <xdr:rowOff>80107</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -994,7 +997,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1200,6 +1203,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="19" spans="1:3" ht="16" customHeight="1">
+      <c r="A19" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1208,7 +1222,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1414,6 +1428,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="19" spans="1:3" ht="16" customHeight="1">
+      <c r="A19" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1422,7 +1447,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1628,6 +1653,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="19" spans="1:3" ht="16" customHeight="1">
+      <c r="A19" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1636,7 +1672,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1842,6 +1878,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="19" spans="1:3" ht="16" customHeight="1">
+      <c r="A19" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1850,7 +1897,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2056,6 +2103,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="19" spans="1:3" ht="16" customHeight="1">
+      <c r="A19" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2064,7 +2122,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2270,6 +2328,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="19" spans="1:3" ht="16" customHeight="1">
+      <c r="A19" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2278,7 +2347,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2484,6 +2553,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="19" spans="1:3" ht="16" customHeight="1">
+      <c r="A19" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2492,7 +2572,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2698,6 +2778,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="19" spans="1:3" ht="16" customHeight="1">
+      <c r="A19" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2706,7 +2797,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2912,6 +3003,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="19" spans="1:3" ht="16" customHeight="1">
+      <c r="A19" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2920,7 +3022,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3126,6 +3228,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="19" spans="1:3" ht="16" customHeight="1">
+      <c r="A19" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3134,7 +3247,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3340,6 +3453,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="19" spans="1:3" ht="16" customHeight="1">
+      <c r="A19" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3348,7 +3472,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3554,6 +3678,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="19" spans="1:3" ht="16" customHeight="1">
+      <c r="A19" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-06-27 12:05:45
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="628" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="664" uniqueCount="23">
   <si>
     <t>Date</t>
   </si>
@@ -91,6 +91,9 @@
   </si>
   <si>
     <t>2026-06-26</t>
+  </si>
+  <si>
+    <t>2026-06-27</t>
   </si>
 </sst>
 </file>
@@ -209,7 +212,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>158063</xdr:rowOff>
+      <xdr:rowOff>148538</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -252,7 +255,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>158063</xdr:rowOff>
+      <xdr:rowOff>148538</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -295,7 +298,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>158063</xdr:rowOff>
+      <xdr:rowOff>148538</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -338,7 +341,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>158063</xdr:rowOff>
+      <xdr:rowOff>148538</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -381,7 +384,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>206501</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>80107</xdr:rowOff>
+      <xdr:rowOff>70582</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -424,7 +427,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>158063</xdr:rowOff>
+      <xdr:rowOff>148538</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -467,7 +470,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>158063</xdr:rowOff>
+      <xdr:rowOff>148538</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -510,7 +513,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>158063</xdr:rowOff>
+      <xdr:rowOff>148538</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -553,7 +556,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>158063</xdr:rowOff>
+      <xdr:rowOff>148538</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -596,7 +599,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>158063</xdr:rowOff>
+      <xdr:rowOff>148538</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -639,7 +642,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>158063</xdr:rowOff>
+      <xdr:rowOff>148538</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -682,7 +685,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>206501</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>80107</xdr:rowOff>
+      <xdr:rowOff>70582</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -997,7 +1000,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1214,6 +1217,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="20" spans="1:3" ht="16" customHeight="1">
+      <c r="A20" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1222,7 +1236,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1439,6 +1453,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="20" spans="1:3" ht="16" customHeight="1">
+      <c r="A20" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1447,7 +1472,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1664,6 +1689,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="20" spans="1:3" ht="16" customHeight="1">
+      <c r="A20" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1672,7 +1708,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1889,6 +1925,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="20" spans="1:3" ht="16" customHeight="1">
+      <c r="A20" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1897,7 +1944,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2114,6 +2161,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="20" spans="1:3" ht="16" customHeight="1">
+      <c r="A20" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2122,7 +2180,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2339,6 +2397,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="20" spans="1:3" ht="16" customHeight="1">
+      <c r="A20" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2347,7 +2416,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2564,6 +2633,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="20" spans="1:3" ht="16" customHeight="1">
+      <c r="A20" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2572,7 +2652,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2789,6 +2869,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="20" spans="1:3" ht="16" customHeight="1">
+      <c r="A20" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2797,7 +2888,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3014,6 +3105,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="20" spans="1:3" ht="16" customHeight="1">
+      <c r="A20" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3022,7 +3124,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3239,6 +3341,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="20" spans="1:3" ht="16" customHeight="1">
+      <c r="A20" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3247,7 +3360,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3464,6 +3577,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="20" spans="1:3" ht="16" customHeight="1">
+      <c r="A20" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3472,7 +3596,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3689,6 +3813,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="20" spans="1:3" ht="16" customHeight="1">
+      <c r="A20" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-06-28 12:12:39
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="664" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="700" uniqueCount="24">
   <si>
     <t>Date</t>
   </si>
@@ -94,6 +94,9 @@
   </si>
   <si>
     <t>2026-06-27</t>
+  </si>
+  <si>
+    <t>2026-06-28</t>
   </si>
 </sst>
 </file>
@@ -212,7 +215,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>148538</xdr:rowOff>
+      <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -255,7 +258,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>148538</xdr:rowOff>
+      <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -298,7 +301,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>148538</xdr:rowOff>
+      <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -341,7 +344,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>148538</xdr:rowOff>
+      <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -384,7 +387,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>206501</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>70582</xdr:rowOff>
+      <xdr:rowOff>61057</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -427,7 +430,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>148538</xdr:rowOff>
+      <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -470,7 +473,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>148538</xdr:rowOff>
+      <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -513,7 +516,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>148538</xdr:rowOff>
+      <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -556,7 +559,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>148538</xdr:rowOff>
+      <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -599,7 +602,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>148538</xdr:rowOff>
+      <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -642,7 +645,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>148538</xdr:rowOff>
+      <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -685,7 +688,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>206501</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>70582</xdr:rowOff>
+      <xdr:rowOff>61057</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1000,7 +1003,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1228,6 +1231,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="21" spans="1:3" ht="16" customHeight="1">
+      <c r="A21" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1236,7 +1250,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1464,6 +1478,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="21" spans="1:3" ht="16" customHeight="1">
+      <c r="A21" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1472,7 +1497,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1700,6 +1725,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="21" spans="1:3" ht="16" customHeight="1">
+      <c r="A21" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1708,7 +1744,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1936,6 +1972,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="21" spans="1:3" ht="16" customHeight="1">
+      <c r="A21" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1944,7 +1991,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2172,6 +2219,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="21" spans="1:3" ht="16" customHeight="1">
+      <c r="A21" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2180,7 +2238,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2408,6 +2466,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="21" spans="1:3" ht="16" customHeight="1">
+      <c r="A21" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2416,7 +2485,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2644,6 +2713,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="21" spans="1:3" ht="16" customHeight="1">
+      <c r="A21" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2652,7 +2732,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2880,6 +2960,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="21" spans="1:3" ht="16" customHeight="1">
+      <c r="A21" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2888,7 +2979,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3116,6 +3207,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="21" spans="1:3" ht="16" customHeight="1">
+      <c r="A21" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3124,7 +3226,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3352,6 +3454,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="21" spans="1:3" ht="16" customHeight="1">
+      <c r="A21" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3360,7 +3473,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3588,6 +3701,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="21" spans="1:3" ht="16" customHeight="1">
+      <c r="A21" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3596,7 +3720,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3824,6 +3948,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="21" spans="1:3" ht="16" customHeight="1">
+      <c r="A21" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-06-29 14:41:59
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="700" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="736" uniqueCount="25">
   <si>
     <t>Date</t>
   </si>
@@ -97,6 +97,9 @@
   </si>
   <si>
     <t>2026-06-28</t>
+  </si>
+  <si>
+    <t>2026-06-29</t>
   </si>
 </sst>
 </file>
@@ -387,7 +390,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>206501</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>61057</xdr:rowOff>
+      <xdr:rowOff>51532</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -688,7 +691,7 @@
       <xdr:col>17</xdr:col>
       <xdr:colOff>206501</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>61057</xdr:rowOff>
+      <xdr:rowOff>51532</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1003,7 +1006,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1242,6 +1245,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="22" spans="1:3" ht="16" customHeight="1">
+      <c r="A22" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1250,7 +1264,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1489,6 +1503,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="22" spans="1:3" ht="16" customHeight="1">
+      <c r="A22" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1497,7 +1522,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1736,6 +1761,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="22" spans="1:3" ht="16" customHeight="1">
+      <c r="A22" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1744,7 +1780,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1983,6 +2019,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="22" spans="1:3" ht="16" customHeight="1">
+      <c r="A22" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1991,7 +2038,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2230,6 +2277,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="22" spans="1:3" ht="16" customHeight="1">
+      <c r="A22" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2238,7 +2296,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2477,6 +2535,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="22" spans="1:3" ht="16" customHeight="1">
+      <c r="A22" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2485,7 +2554,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2724,6 +2793,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="22" spans="1:3" ht="16" customHeight="1">
+      <c r="A22" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2732,7 +2812,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2971,6 +3051,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="22" spans="1:3" ht="16" customHeight="1">
+      <c r="A22" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2979,7 +3070,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3218,6 +3309,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="22" spans="1:3" ht="16" customHeight="1">
+      <c r="A22" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3226,7 +3328,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3465,6 +3567,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="22" spans="1:3" ht="16" customHeight="1">
+      <c r="A22" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3473,7 +3586,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3712,6 +3825,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="22" spans="1:3" ht="16" customHeight="1">
+      <c r="A22" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3720,7 +3844,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3959,6 +4083,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="22" spans="1:3" ht="16" customHeight="1">
+      <c r="A22" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-06-30 13:03:47
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="736" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="772" uniqueCount="26">
   <si>
     <t>Date</t>
   </si>
@@ -100,6 +100,9 @@
   </si>
   <si>
     <t>2026-06-29</t>
+  </si>
+  <si>
+    <t>2026-06-30</t>
   </si>
 </sst>
 </file>
@@ -1006,7 +1009,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1256,6 +1259,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="23" spans="1:3" ht="16" customHeight="1">
+      <c r="A23" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1264,7 +1278,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1514,6 +1528,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="23" spans="1:3" ht="16" customHeight="1">
+      <c r="A23" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1522,7 +1547,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1772,6 +1797,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="23" spans="1:3" ht="16" customHeight="1">
+      <c r="A23" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1780,7 +1816,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2030,6 +2066,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="23" spans="1:3" ht="16" customHeight="1">
+      <c r="A23" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2038,7 +2085,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2288,6 +2335,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="23" spans="1:3" ht="16" customHeight="1">
+      <c r="A23" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2296,7 +2354,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2546,6 +2604,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="23" spans="1:3" ht="16" customHeight="1">
+      <c r="A23" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2554,7 +2623,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2804,6 +2873,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="23" spans="1:3" ht="16" customHeight="1">
+      <c r="A23" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2812,7 +2892,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3062,6 +3142,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="23" spans="1:3" ht="16" customHeight="1">
+      <c r="A23" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3070,7 +3161,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3320,6 +3411,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="23" spans="1:3" ht="16" customHeight="1">
+      <c r="A23" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3328,7 +3430,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3578,6 +3680,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="23" spans="1:3" ht="16" customHeight="1">
+      <c r="A23" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3586,7 +3699,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3836,6 +3949,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="23" spans="1:3" ht="16" customHeight="1">
+      <c r="A23" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3844,7 +3968,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4094,6 +4218,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="23" spans="1:3" ht="16" customHeight="1">
+      <c r="A23" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-07-01 13:31:26
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="772" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="808" uniqueCount="27">
   <si>
     <t>Date</t>
   </si>
@@ -103,6 +103,9 @@
   </si>
   <si>
     <t>2026-06-30</t>
+  </si>
+  <si>
+    <t>2026-07-01</t>
   </si>
 </sst>
 </file>
@@ -1009,7 +1012,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1270,6 +1273,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="24" spans="1:3" ht="16" customHeight="1">
+      <c r="A24" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1278,7 +1292,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1539,6 +1553,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="24" spans="1:3" ht="16" customHeight="1">
+      <c r="A24" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1547,7 +1572,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1808,6 +1833,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="24" spans="1:3" ht="16" customHeight="1">
+      <c r="A24" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1816,7 +1852,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2077,6 +2113,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="24" spans="1:3" ht="16" customHeight="1">
+      <c r="A24" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2085,7 +2132,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2346,6 +2393,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="24" spans="1:3" ht="16" customHeight="1">
+      <c r="A24" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2354,7 +2412,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2615,6 +2673,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="24" spans="1:3" ht="16" customHeight="1">
+      <c r="A24" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2623,7 +2692,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2884,6 +2953,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="24" spans="1:3" ht="16" customHeight="1">
+      <c r="A24" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2892,7 +2972,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3153,6 +3233,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="24" spans="1:3" ht="16" customHeight="1">
+      <c r="A24" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3161,7 +3252,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3422,6 +3513,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="24" spans="1:3" ht="16" customHeight="1">
+      <c r="A24" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3430,7 +3532,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3691,6 +3793,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="24" spans="1:3" ht="16" customHeight="1">
+      <c r="A24" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3699,7 +3812,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3960,6 +4073,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="24" spans="1:3" ht="16" customHeight="1">
+      <c r="A24" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3968,7 +4092,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4229,6 +4353,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="24" spans="1:3" ht="16" customHeight="1">
+      <c r="A24" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-07-02 12:53:41
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="808" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="844" uniqueCount="28">
   <si>
     <t>Date</t>
   </si>
@@ -106,6 +106,9 @@
   </si>
   <si>
     <t>2026-07-01</t>
+  </si>
+  <si>
+    <t>2026-07-02</t>
   </si>
 </sst>
 </file>
@@ -1012,7 +1015,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1284,6 +1287,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="25" spans="1:3" ht="16" customHeight="1">
+      <c r="A25" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1292,7 +1306,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1564,6 +1578,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="25" spans="1:3" ht="16" customHeight="1">
+      <c r="A25" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1572,7 +1597,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1844,6 +1869,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="25" spans="1:3" ht="16" customHeight="1">
+      <c r="A25" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1852,7 +1888,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2124,6 +2160,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="25" spans="1:3" ht="16" customHeight="1">
+      <c r="A25" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2132,7 +2179,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2404,6 +2451,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="25" spans="1:3" ht="16" customHeight="1">
+      <c r="A25" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2412,7 +2470,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2684,6 +2742,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="25" spans="1:3" ht="16" customHeight="1">
+      <c r="A25" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2692,7 +2761,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2964,6 +3033,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="25" spans="1:3" ht="16" customHeight="1">
+      <c r="A25" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2972,7 +3052,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3244,6 +3324,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="25" spans="1:3" ht="16" customHeight="1">
+      <c r="A25" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3252,7 +3343,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3524,6 +3615,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="25" spans="1:3" ht="16" customHeight="1">
+      <c r="A25" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3532,7 +3634,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3804,6 +3906,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="25" spans="1:3" ht="16" customHeight="1">
+      <c r="A25" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3812,7 +3925,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4084,6 +4197,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="25" spans="1:3" ht="16" customHeight="1">
+      <c r="A25" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4092,7 +4216,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4364,6 +4488,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="25" spans="1:3" ht="16" customHeight="1">
+      <c r="A25" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-07-03 12:52:08
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="844" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="880" uniqueCount="29">
   <si>
     <t>Date</t>
   </si>
@@ -109,6 +109,9 @@
   </si>
   <si>
     <t>2026-07-02</t>
+  </si>
+  <si>
+    <t>2026-07-03</t>
   </si>
 </sst>
 </file>
@@ -225,7 +228,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -245,7 +248,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -268,7 +271,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -288,7 +291,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -311,7 +314,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -331,7 +334,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -354,7 +357,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -374,7 +377,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -440,7 +443,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -460,7 +463,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -483,7 +486,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -503,7 +506,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -526,7 +529,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -546,7 +549,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -569,7 +572,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -589,7 +592,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -612,7 +615,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -632,7 +635,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -655,7 +658,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -675,7 +678,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1015,7 +1018,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1298,6 +1301,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="26" spans="1:3" ht="16" customHeight="1">
+      <c r="A26" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1306,7 +1320,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1589,6 +1603,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="26" spans="1:3" ht="16" customHeight="1">
+      <c r="A26" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1597,7 +1622,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1880,6 +1905,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="26" spans="1:3" ht="16" customHeight="1">
+      <c r="A26" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1888,7 +1924,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2171,6 +2207,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="26" spans="1:3" ht="16" customHeight="1">
+      <c r="A26" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2179,7 +2226,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2462,6 +2509,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="26" spans="1:3" ht="16" customHeight="1">
+      <c r="A26" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2470,7 +2528,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2753,6 +2811,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="26" spans="1:3" ht="16" customHeight="1">
+      <c r="A26" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2761,7 +2830,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3044,6 +3113,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="26" spans="1:3" ht="16" customHeight="1">
+      <c r="A26" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3052,7 +3132,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3335,6 +3415,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="26" spans="1:3" ht="16" customHeight="1">
+      <c r="A26" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3343,7 +3434,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3626,6 +3717,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="26" spans="1:3" ht="16" customHeight="1">
+      <c r="A26" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3634,7 +3736,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3917,6 +4019,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="26" spans="1:3" ht="16" customHeight="1">
+      <c r="A26" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3925,7 +4038,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4208,6 +4321,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="26" spans="1:3" ht="16" customHeight="1">
+      <c r="A26" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4216,7 +4340,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4499,6 +4623,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="26" spans="1:3" ht="16" customHeight="1">
+      <c r="A26" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-07-04 12:01:30
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="880" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="916" uniqueCount="30">
   <si>
     <t>Date</t>
   </si>
@@ -112,6 +112,9 @@
   </si>
   <si>
     <t>2026-07-03</t>
+  </si>
+  <si>
+    <t>2026-07-04</t>
   </si>
 </sst>
 </file>
@@ -228,7 +231,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -248,7 +251,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -271,7 +274,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -291,7 +294,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -314,7 +317,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -334,7 +337,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -357,7 +360,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -377,7 +380,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -443,7 +446,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -463,7 +466,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -486,7 +489,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -506,7 +509,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -529,7 +532,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -549,7 +552,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -572,7 +575,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -592,7 +595,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -615,7 +618,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -635,7 +638,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -658,7 +661,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -678,7 +681,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1018,7 +1021,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1312,6 +1315,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="27" spans="1:3" ht="16" customHeight="1">
+      <c r="A27" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1320,7 +1334,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1614,6 +1628,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="27" spans="1:3" ht="16" customHeight="1">
+      <c r="A27" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1622,7 +1647,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1916,6 +1941,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="27" spans="1:3" ht="16" customHeight="1">
+      <c r="A27" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1924,7 +1960,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2218,6 +2254,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="27" spans="1:3" ht="16" customHeight="1">
+      <c r="A27" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2226,7 +2273,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2520,6 +2567,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="27" spans="1:3" ht="16" customHeight="1">
+      <c r="A27" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2528,7 +2586,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2822,6 +2880,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="27" spans="1:3" ht="16" customHeight="1">
+      <c r="A27" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2830,7 +2899,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3124,6 +3193,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="27" spans="1:3" ht="16" customHeight="1">
+      <c r="A27" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3132,7 +3212,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3426,6 +3506,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="27" spans="1:3" ht="16" customHeight="1">
+      <c r="A27" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3434,7 +3525,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3728,6 +3819,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="27" spans="1:3" ht="16" customHeight="1">
+      <c r="A27" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3736,7 +3838,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4030,6 +4132,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="27" spans="1:3" ht="16" customHeight="1">
+      <c r="A27" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4038,7 +4151,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4332,6 +4445,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="27" spans="1:3" ht="16" customHeight="1">
+      <c r="A27" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4340,7 +4464,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4634,6 +4758,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="27" spans="1:3" ht="16" customHeight="1">
+      <c r="A27" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-07-05 12:09:14
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="916" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="952" uniqueCount="31">
   <si>
     <t>Date</t>
   </si>
@@ -115,6 +115,9 @@
   </si>
   <si>
     <t>2026-07-04</t>
+  </si>
+  <si>
+    <t>2026-07-05</t>
   </si>
 </sst>
 </file>
@@ -1021,7 +1024,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1326,6 +1329,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="28" spans="1:3" ht="16" customHeight="1">
+      <c r="A28" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1334,7 +1348,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1639,6 +1653,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="28" spans="1:3" ht="16" customHeight="1">
+      <c r="A28" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1647,7 +1672,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1952,6 +1977,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="28" spans="1:3" ht="16" customHeight="1">
+      <c r="A28" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1960,7 +1996,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2265,6 +2301,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="28" spans="1:3" ht="16" customHeight="1">
+      <c r="A28" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2273,7 +2320,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2578,6 +2625,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="28" spans="1:3" ht="16" customHeight="1">
+      <c r="A28" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2586,7 +2644,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2891,6 +2949,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="28" spans="1:3" ht="16" customHeight="1">
+      <c r="A28" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2899,7 +2968,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3204,6 +3273,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="28" spans="1:3" ht="16" customHeight="1">
+      <c r="A28" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3212,7 +3292,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3517,6 +3597,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="28" spans="1:3" ht="16" customHeight="1">
+      <c r="A28" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3525,7 +3616,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3830,6 +3921,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="28" spans="1:3" ht="16" customHeight="1">
+      <c r="A28" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3838,7 +3940,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4143,6 +4245,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="28" spans="1:3" ht="16" customHeight="1">
+      <c r="A28" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4151,7 +4264,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4456,6 +4569,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="28" spans="1:3" ht="16" customHeight="1">
+      <c r="A28" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4464,7 +4588,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4769,6 +4893,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="28" spans="1:3" ht="16" customHeight="1">
+      <c r="A28" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-07-06 14:23:04
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="952" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="988" uniqueCount="32">
   <si>
     <t>Date</t>
   </si>
@@ -118,6 +118,9 @@
   </si>
   <si>
     <t>2026-07-05</t>
+  </si>
+  <si>
+    <t>2026-07-06</t>
   </si>
 </sst>
 </file>
@@ -234,7 +237,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -254,7 +257,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -277,7 +280,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -297,7 +300,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -320,7 +323,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -340,7 +343,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -363,7 +366,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -383,7 +386,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -449,7 +452,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -469,7 +472,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -492,7 +495,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -512,7 +515,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -535,7 +538,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -555,7 +558,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -578,7 +581,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -598,7 +601,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -621,7 +624,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -641,7 +644,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -664,7 +667,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -684,7 +687,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1024,7 +1027,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1340,6 +1343,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="29" spans="1:3" ht="16" customHeight="1">
+      <c r="A29" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1348,7 +1362,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1664,6 +1678,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="29" spans="1:3" ht="16" customHeight="1">
+      <c r="A29" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1672,7 +1697,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1988,6 +2013,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="29" spans="1:3" ht="16" customHeight="1">
+      <c r="A29" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1996,7 +2032,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2312,6 +2348,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="29" spans="1:3" ht="16" customHeight="1">
+      <c r="A29" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2320,7 +2367,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2636,6 +2683,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="29" spans="1:3" ht="16" customHeight="1">
+      <c r="A29" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2644,7 +2702,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2960,6 +3018,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="29" spans="1:3" ht="16" customHeight="1">
+      <c r="A29" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2968,7 +3037,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3284,6 +3353,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="29" spans="1:3" ht="16" customHeight="1">
+      <c r="A29" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3292,7 +3372,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3608,6 +3688,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="29" spans="1:3" ht="16" customHeight="1">
+      <c r="A29" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3616,7 +3707,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3932,6 +4023,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="29" spans="1:3" ht="16" customHeight="1">
+      <c r="A29" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3940,7 +4042,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4256,6 +4358,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="29" spans="1:3" ht="16" customHeight="1">
+      <c r="A29" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4264,7 +4377,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4580,6 +4693,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="29" spans="1:3" ht="16" customHeight="1">
+      <c r="A29" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4588,7 +4712,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4904,6 +5028,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="29" spans="1:3" ht="16" customHeight="1">
+      <c r="A29" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-07-07 13:11:41
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="988" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1024" uniqueCount="33">
   <si>
     <t>Date</t>
   </si>
@@ -121,6 +121,9 @@
   </si>
   <si>
     <t>2026-07-06</t>
+  </si>
+  <si>
+    <t>2026-07-07</t>
   </si>
 </sst>
 </file>
@@ -237,7 +240,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -257,7 +260,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -280,7 +283,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -300,7 +303,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -323,7 +326,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -343,7 +346,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -366,7 +369,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -386,7 +389,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -452,7 +455,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -472,7 +475,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -495,7 +498,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -515,7 +518,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -538,7 +541,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -558,7 +561,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -581,7 +584,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -601,7 +604,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -624,7 +627,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -644,7 +647,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -667,7 +670,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -687,7 +690,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1027,7 +1030,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1354,6 +1357,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="30" spans="1:3" ht="16" customHeight="1">
+      <c r="A30" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1362,7 +1376,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1689,6 +1703,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="30" spans="1:3" ht="16" customHeight="1">
+      <c r="A30" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1697,7 +1722,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2024,6 +2049,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="30" spans="1:3" ht="16" customHeight="1">
+      <c r="A30" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2032,7 +2068,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2359,6 +2395,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="30" spans="1:3" ht="16" customHeight="1">
+      <c r="A30" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2367,7 +2414,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2694,6 +2741,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="30" spans="1:3" ht="16" customHeight="1">
+      <c r="A30" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2702,7 +2760,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3029,6 +3087,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="30" spans="1:3" ht="16" customHeight="1">
+      <c r="A30" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3037,7 +3106,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3364,6 +3433,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="30" spans="1:3" ht="16" customHeight="1">
+      <c r="A30" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3372,7 +3452,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3699,6 +3779,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="30" spans="1:3" ht="16" customHeight="1">
+      <c r="A30" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3707,7 +3798,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4034,6 +4125,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="30" spans="1:3" ht="16" customHeight="1">
+      <c r="A30" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4042,7 +4144,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4369,6 +4471,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="30" spans="1:3" ht="16" customHeight="1">
+      <c r="A30" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4377,7 +4490,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4704,6 +4817,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="30" spans="1:3" ht="16" customHeight="1">
+      <c r="A30" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4712,7 +4836,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5039,6 +5163,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="30" spans="1:3" ht="16" customHeight="1">
+      <c r="A30" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-07-08 12:13:37
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1024" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1060" uniqueCount="34">
   <si>
     <t>Date</t>
   </si>
@@ -124,6 +124,9 @@
   </si>
   <si>
     <t>2026-07-07</t>
+  </si>
+  <si>
+    <t>2026-07-08</t>
   </si>
 </sst>
 </file>
@@ -1030,7 +1033,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1368,6 +1371,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="31" spans="1:3" ht="16" customHeight="1">
+      <c r="A31" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1376,7 +1390,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1714,6 +1728,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="31" spans="1:3" ht="16" customHeight="1">
+      <c r="A31" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1722,7 +1747,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2060,6 +2085,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="31" spans="1:3" ht="16" customHeight="1">
+      <c r="A31" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2068,7 +2104,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2406,6 +2442,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="31" spans="1:3" ht="16" customHeight="1">
+      <c r="A31" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2414,7 +2461,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2752,6 +2799,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="31" spans="1:3" ht="16" customHeight="1">
+      <c r="A31" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2760,7 +2818,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3098,6 +3156,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="31" spans="1:3" ht="16" customHeight="1">
+      <c r="A31" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3106,7 +3175,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3444,6 +3513,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="31" spans="1:3" ht="16" customHeight="1">
+      <c r="A31" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3452,7 +3532,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3790,6 +3870,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="31" spans="1:3" ht="16" customHeight="1">
+      <c r="A31" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3798,7 +3889,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4136,6 +4227,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="31" spans="1:3" ht="16" customHeight="1">
+      <c r="A31" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4144,7 +4246,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4482,6 +4584,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="31" spans="1:3" ht="16" customHeight="1">
+      <c r="A31" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4490,7 +4603,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4828,6 +4941,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="31" spans="1:3" ht="16" customHeight="1">
+      <c r="A31" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4836,7 +4960,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5174,6 +5298,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="31" spans="1:3" ht="16" customHeight="1">
+      <c r="A31" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-07-09 13:42:47
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1060" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1096" uniqueCount="35">
   <si>
     <t>Date</t>
   </si>
@@ -127,6 +127,9 @@
   </si>
   <si>
     <t>2026-07-08</t>
+  </si>
+  <si>
+    <t>2026-07-09</t>
   </si>
 </sst>
 </file>
@@ -1033,7 +1036,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1382,6 +1385,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="32" spans="1:3" ht="16" customHeight="1">
+      <c r="A32" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1390,7 +1404,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1739,6 +1753,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="32" spans="1:3" ht="16" customHeight="1">
+      <c r="A32" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1747,7 +1772,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2096,6 +2121,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="32" spans="1:3" ht="16" customHeight="1">
+      <c r="A32" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2104,7 +2140,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2453,6 +2489,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="32" spans="1:3" ht="16" customHeight="1">
+      <c r="A32" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2461,7 +2508,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2810,6 +2857,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="32" spans="1:3" ht="16" customHeight="1">
+      <c r="A32" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2818,7 +2876,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3167,6 +3225,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="32" spans="1:3" ht="16" customHeight="1">
+      <c r="A32" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3175,7 +3244,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3524,6 +3593,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="32" spans="1:3" ht="16" customHeight="1">
+      <c r="A32" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3532,7 +3612,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3881,6 +3961,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="32" spans="1:3" ht="16" customHeight="1">
+      <c r="A32" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3889,7 +3980,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4238,6 +4329,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="32" spans="1:3" ht="16" customHeight="1">
+      <c r="A32" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4246,7 +4348,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4595,6 +4697,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="32" spans="1:3" ht="16" customHeight="1">
+      <c r="A32" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4603,7 +4716,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4952,6 +5065,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="32" spans="1:3" ht="16" customHeight="1">
+      <c r="A32" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4960,7 +5084,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5309,6 +5433,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="32" spans="1:3" ht="16" customHeight="1">
+      <c r="A32" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-07-10 13:04:02
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1096" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1132" uniqueCount="36">
   <si>
     <t>Date</t>
   </si>
@@ -130,6 +130,9 @@
   </si>
   <si>
     <t>2026-07-09</t>
+  </si>
+  <si>
+    <t>2026-07-10</t>
   </si>
 </sst>
 </file>
@@ -1036,7 +1039,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1396,6 +1399,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="33" spans="1:3" ht="16" customHeight="1">
+      <c r="A33" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1404,7 +1418,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1764,6 +1778,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="33" spans="1:3" ht="16" customHeight="1">
+      <c r="A33" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1772,7 +1797,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2132,6 +2157,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="33" spans="1:3" ht="16" customHeight="1">
+      <c r="A33" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2140,7 +2176,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2500,6 +2536,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="33" spans="1:3" ht="16" customHeight="1">
+      <c r="A33" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2508,7 +2555,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2868,6 +2915,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="33" spans="1:3" ht="16" customHeight="1">
+      <c r="A33" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2876,7 +2934,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3236,6 +3294,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="33" spans="1:3" ht="16" customHeight="1">
+      <c r="A33" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3244,7 +3313,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3604,6 +3673,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="33" spans="1:3" ht="16" customHeight="1">
+      <c r="A33" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3612,7 +3692,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3972,6 +4052,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="33" spans="1:3" ht="16" customHeight="1">
+      <c r="A33" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3980,7 +4071,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4340,6 +4431,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="33" spans="1:3" ht="16" customHeight="1">
+      <c r="A33" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4348,7 +4450,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4708,6 +4810,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="33" spans="1:3" ht="16" customHeight="1">
+      <c r="A33" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4716,7 +4829,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5076,6 +5189,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="33" spans="1:3" ht="16" customHeight="1">
+      <c r="A33" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5084,7 +5208,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5444,6 +5568,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="33" spans="1:3" ht="16" customHeight="1">
+      <c r="A33" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-07-11 11:43:39
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1132" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1168" uniqueCount="37">
   <si>
     <t>Date</t>
   </si>
@@ -133,6 +133,9 @@
   </si>
   <si>
     <t>2026-07-10</t>
+  </si>
+  <si>
+    <t>2026-07-11</t>
   </si>
 </sst>
 </file>
@@ -249,7 +252,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -269,7 +272,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -292,7 +295,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -312,7 +315,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -335,7 +338,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -355,7 +358,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -378,7 +381,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -398,7 +401,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -464,7 +467,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -484,7 +487,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -507,7 +510,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -527,7 +530,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -550,7 +553,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -570,7 +573,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -593,7 +596,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -613,7 +616,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -636,7 +639,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -656,7 +659,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -679,7 +682,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -699,7 +702,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1039,7 +1042,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1410,6 +1413,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="34" spans="1:3" ht="16" customHeight="1">
+      <c r="A34" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1418,7 +1432,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1789,6 +1803,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="34" spans="1:3" ht="16" customHeight="1">
+      <c r="A34" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1797,7 +1822,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2168,6 +2193,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="34" spans="1:3" ht="16" customHeight="1">
+      <c r="A34" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2176,7 +2212,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2547,6 +2583,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="34" spans="1:3" ht="16" customHeight="1">
+      <c r="A34" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2555,7 +2602,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2926,6 +2973,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="34" spans="1:3" ht="16" customHeight="1">
+      <c r="A34" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2934,7 +2992,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3305,6 +3363,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="34" spans="1:3" ht="16" customHeight="1">
+      <c r="A34" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3313,7 +3382,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3684,6 +3753,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="34" spans="1:3" ht="16" customHeight="1">
+      <c r="A34" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3692,7 +3772,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4063,6 +4143,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="34" spans="1:3" ht="16" customHeight="1">
+      <c r="A34" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4071,7 +4162,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4442,6 +4533,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="34" spans="1:3" ht="16" customHeight="1">
+      <c r="A34" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4450,7 +4552,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4821,6 +4923,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="34" spans="1:3" ht="16" customHeight="1">
+      <c r="A34" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4829,7 +4942,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5200,6 +5313,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="34" spans="1:3" ht="16" customHeight="1">
+      <c r="A34" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5208,7 +5332,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5579,6 +5703,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="34" spans="1:3" ht="16" customHeight="1">
+      <c r="A34" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-07-12 11:50:38
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1168" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1204" uniqueCount="38">
   <si>
     <t>Date</t>
   </si>
@@ -136,6 +136,9 @@
   </si>
   <si>
     <t>2026-07-11</t>
+  </si>
+  <si>
+    <t>2026-07-12</t>
   </si>
 </sst>
 </file>
@@ -252,7 +255,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -272,7 +275,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -295,7 +298,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -315,7 +318,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -338,7 +341,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -358,7 +361,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -381,7 +384,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -401,7 +404,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -467,7 +470,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -487,7 +490,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -510,7 +513,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -530,7 +533,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -553,7 +556,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -573,7 +576,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -596,7 +599,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -616,7 +619,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -639,7 +642,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -659,7 +662,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -682,7 +685,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -702,7 +705,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1042,7 +1045,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1424,6 +1427,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="35" spans="1:3" ht="16" customHeight="1">
+      <c r="A35" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1432,7 +1446,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1814,6 +1828,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="35" spans="1:3" ht="16" customHeight="1">
+      <c r="A35" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1822,7 +1847,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2204,6 +2229,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="35" spans="1:3" ht="16" customHeight="1">
+      <c r="A35" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2212,7 +2248,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2594,6 +2630,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="35" spans="1:3" ht="16" customHeight="1">
+      <c r="A35" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2602,7 +2649,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2984,6 +3031,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="35" spans="1:3" ht="16" customHeight="1">
+      <c r="A35" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2992,7 +3050,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3374,6 +3432,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="35" spans="1:3" ht="16" customHeight="1">
+      <c r="A35" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3382,7 +3451,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3764,6 +3833,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="35" spans="1:3" ht="16" customHeight="1">
+      <c r="A35" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3772,7 +3852,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4154,6 +4234,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="35" spans="1:3" ht="16" customHeight="1">
+      <c r="A35" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4162,7 +4253,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4544,6 +4635,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="35" spans="1:3" ht="16" customHeight="1">
+      <c r="A35" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4552,7 +4654,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4934,6 +5036,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="35" spans="1:3" ht="16" customHeight="1">
+      <c r="A35" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4942,7 +5055,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5324,6 +5437,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="35" spans="1:3" ht="16" customHeight="1">
+      <c r="A35" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5332,7 +5456,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5714,6 +5838,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="35" spans="1:3" ht="16" customHeight="1">
+      <c r="A35" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-07-13 13:18:56
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1204" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1229" uniqueCount="39">
   <si>
     <t>Date</t>
   </si>
@@ -139,6 +139,9 @@
   </si>
   <si>
     <t>2026-07-12</t>
+  </si>
+  <si>
+    <t>2026-07-13</t>
   </si>
 </sst>
 </file>
@@ -1045,7 +1048,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1438,6 +1441,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="36" spans="1:3" ht="16" customHeight="1">
+      <c r="A36" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1446,7 +1460,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1839,6 +1853,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="36" spans="1:3" ht="16" customHeight="1">
+      <c r="A36" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1847,7 +1872,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2240,6 +2265,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="36" spans="1:3" ht="16" customHeight="1">
+      <c r="A36" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B36" s="3">
+        <v>0.88</v>
+      </c>
+      <c r="C36" s="3">
+        <v>1.43</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2248,7 +2284,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2641,6 +2677,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="36" spans="1:3" ht="16" customHeight="1">
+      <c r="A36" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2649,7 +2696,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3042,6 +3089,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="36" spans="1:3" ht="16" customHeight="1">
+      <c r="A36" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3050,7 +3108,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3443,6 +3501,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="36" spans="1:3" ht="16" customHeight="1">
+      <c r="A36" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C36" s="3">
+        <v>7.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3451,7 +3520,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3844,6 +3913,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="36" spans="1:3" ht="16" customHeight="1">
+      <c r="A36" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B36" s="3">
+        <v>3.44</v>
+      </c>
+      <c r="C36" s="3">
+        <v>4.81</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3852,7 +3932,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4245,6 +4325,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="36" spans="1:3" ht="16" customHeight="1">
+      <c r="A36" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B36" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4253,7 +4344,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4646,6 +4737,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="36" spans="1:3" ht="16" customHeight="1">
+      <c r="A36" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B36" s="3">
+        <v>1.99</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4654,7 +4756,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5047,6 +5149,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="36" spans="1:3" ht="16" customHeight="1">
+      <c r="A36" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B36" s="3">
+        <v>3.14</v>
+      </c>
+      <c r="C36" s="3">
+        <v>1.47</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5055,7 +5168,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5448,6 +5561,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="36" spans="1:3" ht="16" customHeight="1">
+      <c r="A36" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B36" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C36" s="3">
+        <v>2.91</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5456,7 +5580,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5849,6 +5973,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="36" spans="1:3" ht="16" customHeight="1">
+      <c r="A36" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-07-14 12:11:43
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1229" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1253" uniqueCount="40">
   <si>
     <t>Date</t>
   </si>
@@ -142,6 +142,9 @@
   </si>
   <si>
     <t>2026-07-13</t>
+  </si>
+  <si>
+    <t>2026-07-14</t>
   </si>
 </sst>
 </file>
@@ -1048,7 +1051,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1452,6 +1455,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="37" spans="1:3" ht="16" customHeight="1">
+      <c r="A37" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B37" s="3">
+        <v>7.5</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1460,7 +1474,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1864,6 +1878,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="37" spans="1:3" ht="16" customHeight="1">
+      <c r="A37" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B37" s="3">
+        <v>1.99</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1872,7 +1897,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2276,6 +2301,17 @@
         <v>1.43</v>
       </c>
     </row>
+    <row r="37" spans="1:3" ht="16" customHeight="1">
+      <c r="A37" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B37" s="3">
+        <v>0.87</v>
+      </c>
+      <c r="C37" s="3">
+        <v>0.8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2284,7 +2320,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2688,6 +2724,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="37" spans="1:3" ht="16" customHeight="1">
+      <c r="A37" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2696,7 +2743,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3100,6 +3147,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="37" spans="1:3" ht="16" customHeight="1">
+      <c r="A37" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3108,7 +3166,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3512,6 +3570,17 @@
         <v>7.5</v>
       </c>
     </row>
+    <row r="37" spans="1:3" ht="16" customHeight="1">
+      <c r="A37" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C37" s="3">
+        <v>8.75</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3520,7 +3589,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3924,6 +3993,17 @@
         <v>4.81</v>
       </c>
     </row>
+    <row r="37" spans="1:3" ht="16" customHeight="1">
+      <c r="A37" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B37" s="3">
+        <v>3.44</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3932,7 +4012,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4336,6 +4416,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="37" spans="1:3" ht="16" customHeight="1">
+      <c r="A37" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B37" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4344,7 +4435,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4748,6 +4839,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="37" spans="1:3" ht="16" customHeight="1">
+      <c r="A37" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B37" s="3">
+        <v>1.99</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4756,7 +4858,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5160,6 +5262,17 @@
         <v>1.47</v>
       </c>
     </row>
+    <row r="37" spans="1:3" ht="16" customHeight="1">
+      <c r="A37" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B37" s="3">
+        <v>3.14</v>
+      </c>
+      <c r="C37" s="3">
+        <v>2.2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5168,7 +5281,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5572,6 +5685,17 @@
         <v>2.91</v>
       </c>
     </row>
+    <row r="37" spans="1:3" ht="16" customHeight="1">
+      <c r="A37" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B37" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C37" s="3">
+        <v>2.95</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5580,7 +5704,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5984,6 +6108,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="37" spans="1:3" ht="16" customHeight="1">
+      <c r="A37" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-07-15 12:09:57
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1253" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1289" uniqueCount="41">
   <si>
     <t>Date</t>
   </si>
@@ -146,6 +146,9 @@
   <si>
     <t>2026-07-14</t>
   </si>
+  <si>
+    <t>2026-07-15</t>
+  </si>
 </sst>
 </file>
 
@@ -261,7 +264,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -281,7 +284,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -304,7 +307,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -324,7 +327,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -347,7 +350,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -367,7 +370,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -390,7 +393,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -410,7 +413,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -476,7 +479,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -496,7 +499,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -519,7 +522,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -539,7 +542,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -562,7 +565,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -582,7 +585,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -605,7 +608,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -625,7 +628,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -648,7 +651,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -668,7 +671,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -691,7 +694,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -711,7 +714,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1051,7 +1054,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C38"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1466,6 +1469,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="38" spans="1:3" ht="16" customHeight="1">
+      <c r="A38" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1474,7 +1488,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C38"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1889,6 +1903,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="38" spans="1:3" ht="16" customHeight="1">
+      <c r="A38" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1897,7 +1922,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C38"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2312,6 +2337,17 @@
         <v>0.8</v>
       </c>
     </row>
+    <row r="38" spans="1:3" ht="16" customHeight="1">
+      <c r="A38" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2320,7 +2356,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C38"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2735,6 +2771,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="38" spans="1:3" ht="16" customHeight="1">
+      <c r="A38" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2743,7 +2790,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C38"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3158,6 +3205,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="38" spans="1:3" ht="16" customHeight="1">
+      <c r="A38" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3166,7 +3224,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C38"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3581,6 +3639,17 @@
         <v>8.75</v>
       </c>
     </row>
+    <row r="38" spans="1:3" ht="16" customHeight="1">
+      <c r="A38" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3589,7 +3658,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C38"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4004,6 +4073,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="38" spans="1:3" ht="16" customHeight="1">
+      <c r="A38" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4012,7 +4092,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C38"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4427,6 +4507,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="38" spans="1:3" ht="16" customHeight="1">
+      <c r="A38" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4435,7 +4526,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C38"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4850,6 +4941,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="38" spans="1:3" ht="16" customHeight="1">
+      <c r="A38" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4858,7 +4960,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C38"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5273,6 +5375,17 @@
         <v>2.2</v>
       </c>
     </row>
+    <row r="38" spans="1:3" ht="16" customHeight="1">
+      <c r="A38" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5281,7 +5394,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C38"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5696,6 +5809,17 @@
         <v>2.95</v>
       </c>
     </row>
+    <row r="38" spans="1:3" ht="16" customHeight="1">
+      <c r="A38" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5704,7 +5828,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C38"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6119,6 +6243,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="38" spans="1:3" ht="16" customHeight="1">
+      <c r="A38" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-07-16 12:14:03
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1289" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1325" uniqueCount="42">
   <si>
     <t>Date</t>
   </si>
@@ -149,6 +149,9 @@
   <si>
     <t>2026-07-15</t>
   </si>
+  <si>
+    <t>2026-07-16</t>
+  </si>
 </sst>
 </file>
 
@@ -264,7 +267,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -284,7 +287,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -307,7 +310,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -327,7 +330,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -350,7 +353,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -370,7 +373,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -393,7 +396,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -413,7 +416,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -479,7 +482,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -499,7 +502,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -522,7 +525,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -542,7 +545,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -565,7 +568,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -585,7 +588,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -608,7 +611,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -628,7 +631,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -651,7 +654,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -671,7 +674,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -694,7 +697,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -714,7 +717,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1054,7 +1057,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1480,6 +1483,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="39" spans="1:3" ht="16" customHeight="1">
+      <c r="A39" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1488,7 +1502,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1914,6 +1928,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="39" spans="1:3" ht="16" customHeight="1">
+      <c r="A39" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1922,7 +1947,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2348,6 +2373,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="39" spans="1:3" ht="16" customHeight="1">
+      <c r="A39" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2356,7 +2392,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2782,6 +2818,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="39" spans="1:3" ht="16" customHeight="1">
+      <c r="A39" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2790,7 +2837,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3216,6 +3263,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="39" spans="1:3" ht="16" customHeight="1">
+      <c r="A39" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3224,7 +3282,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3650,6 +3708,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="39" spans="1:3" ht="16" customHeight="1">
+      <c r="A39" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3658,7 +3727,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4084,6 +4153,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="39" spans="1:3" ht="16" customHeight="1">
+      <c r="A39" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4092,7 +4172,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4518,6 +4598,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="39" spans="1:3" ht="16" customHeight="1">
+      <c r="A39" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4526,7 +4617,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4952,6 +5043,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="39" spans="1:3" ht="16" customHeight="1">
+      <c r="A39" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4960,7 +5062,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5386,6 +5488,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="39" spans="1:3" ht="16" customHeight="1">
+      <c r="A39" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5394,7 +5507,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5820,6 +5933,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="39" spans="1:3" ht="16" customHeight="1">
+      <c r="A39" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5828,7 +5952,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6254,6 +6378,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="39" spans="1:3" ht="16" customHeight="1">
+      <c r="A39" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-07-17 12:03:01
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1325" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1361" uniqueCount="43">
   <si>
     <t>Date</t>
   </si>
@@ -151,6 +151,9 @@
   </si>
   <si>
     <t>2026-07-16</t>
+  </si>
+  <si>
+    <t>2026-07-17</t>
   </si>
 </sst>
 </file>
@@ -1057,7 +1060,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1494,6 +1497,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="40" spans="1:3" ht="16" customHeight="1">
+      <c r="A40" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1502,7 +1516,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1939,6 +1953,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="40" spans="1:3" ht="16" customHeight="1">
+      <c r="A40" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1947,7 +1972,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2384,6 +2409,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="40" spans="1:3" ht="16" customHeight="1">
+      <c r="A40" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2392,7 +2428,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2829,6 +2865,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="40" spans="1:3" ht="16" customHeight="1">
+      <c r="A40" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2837,7 +2884,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3274,6 +3321,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="40" spans="1:3" ht="16" customHeight="1">
+      <c r="A40" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3282,7 +3340,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3719,6 +3777,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="40" spans="1:3" ht="16" customHeight="1">
+      <c r="A40" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3727,7 +3796,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4164,6 +4233,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="40" spans="1:3" ht="16" customHeight="1">
+      <c r="A40" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4172,7 +4252,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4609,6 +4689,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="40" spans="1:3" ht="16" customHeight="1">
+      <c r="A40" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4617,7 +4708,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5054,6 +5145,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="40" spans="1:3" ht="16" customHeight="1">
+      <c r="A40" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5062,7 +5164,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5499,6 +5601,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="40" spans="1:3" ht="16" customHeight="1">
+      <c r="A40" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5507,7 +5620,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5944,6 +6057,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="40" spans="1:3" ht="16" customHeight="1">
+      <c r="A40" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5952,7 +6076,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6389,6 +6513,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="40" spans="1:3" ht="16" customHeight="1">
+      <c r="A40" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-07-18 11:44:01
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1361" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1397" uniqueCount="44">
   <si>
     <t>Date</t>
   </si>
@@ -154,6 +154,9 @@
   </si>
   <si>
     <t>2026-07-17</t>
+  </si>
+  <si>
+    <t>2026-07-18</t>
   </si>
 </sst>
 </file>
@@ -442,7 +445,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>206501</xdr:colOff>
+      <xdr:colOff>213535</xdr:colOff>
       <xdr:row>22</xdr:row>
       <xdr:rowOff>51532</xdr:rowOff>
     </xdr:to>
@@ -462,7 +465,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8131301" cy="4480657"/>
+          <a:ext cx="8138335" cy="4480657"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -743,7 +746,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>206501</xdr:colOff>
+      <xdr:colOff>213535</xdr:colOff>
       <xdr:row>22</xdr:row>
       <xdr:rowOff>51532</xdr:rowOff>
     </xdr:to>
@@ -763,7 +766,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8131301" cy="4480657"/>
+          <a:ext cx="8138335" cy="4480657"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1060,7 +1063,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1508,6 +1511,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="41" spans="1:3" ht="16" customHeight="1">
+      <c r="A41" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1516,7 +1530,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1964,6 +1978,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="41" spans="1:3" ht="16" customHeight="1">
+      <c r="A41" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1972,7 +1997,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2420,6 +2445,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="41" spans="1:3" ht="16" customHeight="1">
+      <c r="A41" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2428,7 +2464,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2876,6 +2912,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="41" spans="1:3" ht="16" customHeight="1">
+      <c r="A41" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2884,7 +2931,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3332,6 +3379,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="41" spans="1:3" ht="16" customHeight="1">
+      <c r="A41" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3340,7 +3398,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3788,6 +3846,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="41" spans="1:3" ht="16" customHeight="1">
+      <c r="A41" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3796,7 +3865,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4244,6 +4313,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="41" spans="1:3" ht="16" customHeight="1">
+      <c r="A41" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4252,7 +4332,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4700,6 +4780,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="41" spans="1:3" ht="16" customHeight="1">
+      <c r="A41" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4708,7 +4799,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5156,6 +5247,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="41" spans="1:3" ht="16" customHeight="1">
+      <c r="A41" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5164,7 +5266,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5612,6 +5714,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="41" spans="1:3" ht="16" customHeight="1">
+      <c r="A41" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5620,7 +5733,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6068,6 +6181,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="41" spans="1:3" ht="16" customHeight="1">
+      <c r="A41" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6076,7 +6200,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6524,6 +6648,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="41" spans="1:3" ht="16" customHeight="1">
+      <c r="A41" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-07-19 11:48:49
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1397" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1433" uniqueCount="45">
   <si>
     <t>Date</t>
   </si>
@@ -158,6 +158,9 @@
   <si>
     <t>2026-07-18</t>
   </si>
+  <si>
+    <t>2026-07-19</t>
+  </si>
 </sst>
 </file>
 
@@ -273,7 +276,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -293,7 +296,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -316,7 +319,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -336,7 +339,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -359,7 +362,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -379,7 +382,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -402,7 +405,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -422,7 +425,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -488,7 +491,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -508,7 +511,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -531,7 +534,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -551,7 +554,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -574,7 +577,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -594,7 +597,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -617,7 +620,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -637,7 +640,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -660,7 +663,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -680,7 +683,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -703,7 +706,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -723,7 +726,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1063,7 +1066,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1522,6 +1525,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="42" spans="1:3" ht="16" customHeight="1">
+      <c r="A42" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1530,7 +1544,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1989,6 +2003,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="42" spans="1:3" ht="16" customHeight="1">
+      <c r="A42" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1997,7 +2022,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2456,6 +2481,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="42" spans="1:3" ht="16" customHeight="1">
+      <c r="A42" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2464,7 +2500,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2923,6 +2959,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="42" spans="1:3" ht="16" customHeight="1">
+      <c r="A42" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2931,7 +2978,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3390,6 +3437,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="42" spans="1:3" ht="16" customHeight="1">
+      <c r="A42" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3398,7 +3456,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3857,6 +3915,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="42" spans="1:3" ht="16" customHeight="1">
+      <c r="A42" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3865,7 +3934,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4324,6 +4393,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="42" spans="1:3" ht="16" customHeight="1">
+      <c r="A42" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4332,7 +4412,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4791,6 +4871,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="42" spans="1:3" ht="16" customHeight="1">
+      <c r="A42" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4799,7 +4890,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5258,6 +5349,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="42" spans="1:3" ht="16" customHeight="1">
+      <c r="A42" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5266,7 +5368,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5725,6 +5827,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="42" spans="1:3" ht="16" customHeight="1">
+      <c r="A42" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5733,7 +5846,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6192,6 +6305,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="42" spans="1:3" ht="16" customHeight="1">
+      <c r="A42" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6200,7 +6324,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6659,6 +6783,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="42" spans="1:3" ht="16" customHeight="1">
+      <c r="A42" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-07-20 13:00:38
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1433" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1469" uniqueCount="46">
   <si>
     <t>Date</t>
   </si>
@@ -161,6 +161,9 @@
   <si>
     <t>2026-07-19</t>
   </si>
+  <si>
+    <t>2026-07-20</t>
+  </si>
 </sst>
 </file>
 
@@ -276,7 +279,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -296,7 +299,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -319,7 +322,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -339,7 +342,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -362,7 +365,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -382,7 +385,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -405,7 +408,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -425,7 +428,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -491,7 +494,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -511,7 +514,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -534,7 +537,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -554,7 +557,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -577,7 +580,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -597,7 +600,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -620,7 +623,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -640,7 +643,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -663,7 +666,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -683,7 +686,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -706,7 +709,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -726,7 +729,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1066,7 +1069,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C43"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1536,6 +1539,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="43" spans="1:3" ht="16" customHeight="1">
+      <c r="A43" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1544,7 +1558,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C43"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2014,6 +2028,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="43" spans="1:3" ht="16" customHeight="1">
+      <c r="A43" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2022,7 +2047,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C43"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2492,6 +2517,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="43" spans="1:3" ht="16" customHeight="1">
+      <c r="A43" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2500,7 +2536,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C43"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2970,6 +3006,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="43" spans="1:3" ht="16" customHeight="1">
+      <c r="A43" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2978,7 +3025,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C43"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3448,6 +3495,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="43" spans="1:3" ht="16" customHeight="1">
+      <c r="A43" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3456,7 +3514,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C43"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3926,6 +3984,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="43" spans="1:3" ht="16" customHeight="1">
+      <c r="A43" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3934,7 +4003,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C43"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4404,6 +4473,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="43" spans="1:3" ht="16" customHeight="1">
+      <c r="A43" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4412,7 +4492,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C43"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4882,6 +4962,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="43" spans="1:3" ht="16" customHeight="1">
+      <c r="A43" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4890,7 +4981,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C43"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5360,6 +5451,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="43" spans="1:3" ht="16" customHeight="1">
+      <c r="A43" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5368,7 +5470,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C43"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5838,6 +5940,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="43" spans="1:3" ht="16" customHeight="1">
+      <c r="A43" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5846,7 +5959,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C43"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6316,6 +6429,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="43" spans="1:3" ht="16" customHeight="1">
+      <c r="A43" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6324,7 +6448,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C43"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6794,6 +6918,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="43" spans="1:3" ht="16" customHeight="1">
+      <c r="A43" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-07-21 12:18:47
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1469" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1505" uniqueCount="47">
   <si>
     <t>Date</t>
   </si>
@@ -163,6 +163,9 @@
   </si>
   <si>
     <t>2026-07-20</t>
+  </si>
+  <si>
+    <t>2026-07-21</t>
   </si>
 </sst>
 </file>
@@ -1069,7 +1072,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C43"/>
+  <dimension ref="A1:C44"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1550,6 +1553,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="44" spans="1:3" ht="16" customHeight="1">
+      <c r="A44" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1558,7 +1572,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C43"/>
+  <dimension ref="A1:C44"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2039,6 +2053,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="44" spans="1:3" ht="16" customHeight="1">
+      <c r="A44" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2047,7 +2072,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C43"/>
+  <dimension ref="A1:C44"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2528,6 +2553,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="44" spans="1:3" ht="16" customHeight="1">
+      <c r="A44" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2536,7 +2572,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C43"/>
+  <dimension ref="A1:C44"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3017,6 +3053,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="44" spans="1:3" ht="16" customHeight="1">
+      <c r="A44" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3025,7 +3072,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C43"/>
+  <dimension ref="A1:C44"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3506,6 +3553,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="44" spans="1:3" ht="16" customHeight="1">
+      <c r="A44" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3514,7 +3572,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C43"/>
+  <dimension ref="A1:C44"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3995,6 +4053,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="44" spans="1:3" ht="16" customHeight="1">
+      <c r="A44" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4003,7 +4072,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C43"/>
+  <dimension ref="A1:C44"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4484,6 +4553,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="44" spans="1:3" ht="16" customHeight="1">
+      <c r="A44" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4492,7 +4572,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C43"/>
+  <dimension ref="A1:C44"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4973,6 +5053,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="44" spans="1:3" ht="16" customHeight="1">
+      <c r="A44" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4981,7 +5072,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C43"/>
+  <dimension ref="A1:C44"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5462,6 +5553,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="44" spans="1:3" ht="16" customHeight="1">
+      <c r="A44" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5470,7 +5572,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C43"/>
+  <dimension ref="A1:C44"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5951,6 +6053,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="44" spans="1:3" ht="16" customHeight="1">
+      <c r="A44" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5959,7 +6072,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C43"/>
+  <dimension ref="A1:C44"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6440,6 +6553,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="44" spans="1:3" ht="16" customHeight="1">
+      <c r="A44" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6448,7 +6572,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C43"/>
+  <dimension ref="A1:C44"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6929,6 +7053,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="44" spans="1:3" ht="16" customHeight="1">
+      <c r="A44" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-07-22 12:21:12
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1505" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1541" uniqueCount="48">
   <si>
     <t>Date</t>
   </si>
@@ -166,6 +166,9 @@
   </si>
   <si>
     <t>2026-07-21</t>
+  </si>
+  <si>
+    <t>2026-07-22</t>
   </si>
 </sst>
 </file>
@@ -1072,7 +1075,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C44"/>
+  <dimension ref="A1:C45"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1564,6 +1567,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="45" spans="1:3" ht="16" customHeight="1">
+      <c r="A45" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1572,7 +1586,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C44"/>
+  <dimension ref="A1:C45"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2064,6 +2078,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="45" spans="1:3" ht="16" customHeight="1">
+      <c r="A45" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2072,7 +2097,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C44"/>
+  <dimension ref="A1:C45"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2564,6 +2589,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="45" spans="1:3" ht="16" customHeight="1">
+      <c r="A45" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2572,7 +2608,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C44"/>
+  <dimension ref="A1:C45"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3064,6 +3100,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="45" spans="1:3" ht="16" customHeight="1">
+      <c r="A45" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3072,7 +3119,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C44"/>
+  <dimension ref="A1:C45"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3564,6 +3611,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="45" spans="1:3" ht="16" customHeight="1">
+      <c r="A45" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3572,7 +3630,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C44"/>
+  <dimension ref="A1:C45"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4064,6 +4122,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="45" spans="1:3" ht="16" customHeight="1">
+      <c r="A45" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4072,7 +4141,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C44"/>
+  <dimension ref="A1:C45"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4564,6 +4633,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="45" spans="1:3" ht="16" customHeight="1">
+      <c r="A45" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4572,7 +4652,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C44"/>
+  <dimension ref="A1:C45"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5064,6 +5144,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="45" spans="1:3" ht="16" customHeight="1">
+      <c r="A45" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5072,7 +5163,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C44"/>
+  <dimension ref="A1:C45"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5564,6 +5655,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="45" spans="1:3" ht="16" customHeight="1">
+      <c r="A45" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5572,7 +5674,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C44"/>
+  <dimension ref="A1:C45"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6064,6 +6166,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="45" spans="1:3" ht="16" customHeight="1">
+      <c r="A45" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6072,7 +6185,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C44"/>
+  <dimension ref="A1:C45"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6564,6 +6677,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="45" spans="1:3" ht="16" customHeight="1">
+      <c r="A45" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6572,7 +6696,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C44"/>
+  <dimension ref="A1:C45"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7064,6 +7188,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="45" spans="1:3" ht="16" customHeight="1">
+      <c r="A45" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-07-23 12:18:35
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1541" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1577" uniqueCount="49">
   <si>
     <t>Date</t>
   </si>
@@ -169,6 +169,9 @@
   </si>
   <si>
     <t>2026-07-22</t>
+  </si>
+  <si>
+    <t>2026-07-23</t>
   </si>
 </sst>
 </file>
@@ -1075,7 +1078,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C45"/>
+  <dimension ref="A1:C46"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1578,6 +1581,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="46" spans="1:3" ht="16" customHeight="1">
+      <c r="A46" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1586,7 +1600,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C45"/>
+  <dimension ref="A1:C46"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2089,6 +2103,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="46" spans="1:3" ht="16" customHeight="1">
+      <c r="A46" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2097,7 +2122,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C45"/>
+  <dimension ref="A1:C46"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2600,6 +2625,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="46" spans="1:3" ht="16" customHeight="1">
+      <c r="A46" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2608,7 +2644,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C45"/>
+  <dimension ref="A1:C46"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3111,6 +3147,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="46" spans="1:3" ht="16" customHeight="1">
+      <c r="A46" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3119,7 +3166,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C45"/>
+  <dimension ref="A1:C46"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3622,6 +3669,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="46" spans="1:3" ht="16" customHeight="1">
+      <c r="A46" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3630,7 +3688,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C45"/>
+  <dimension ref="A1:C46"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4133,6 +4191,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="46" spans="1:3" ht="16" customHeight="1">
+      <c r="A46" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4141,7 +4210,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C45"/>
+  <dimension ref="A1:C46"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4644,6 +4713,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="46" spans="1:3" ht="16" customHeight="1">
+      <c r="A46" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4652,7 +4732,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C45"/>
+  <dimension ref="A1:C46"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5155,6 +5235,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="46" spans="1:3" ht="16" customHeight="1">
+      <c r="A46" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5163,7 +5254,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C45"/>
+  <dimension ref="A1:C46"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5666,6 +5757,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="46" spans="1:3" ht="16" customHeight="1">
+      <c r="A46" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5674,7 +5776,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C45"/>
+  <dimension ref="A1:C46"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6177,6 +6279,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="46" spans="1:3" ht="16" customHeight="1">
+      <c r="A46" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6185,7 +6298,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C45"/>
+  <dimension ref="A1:C46"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6688,6 +6801,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="46" spans="1:3" ht="16" customHeight="1">
+      <c r="A46" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6696,7 +6820,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C45"/>
+  <dimension ref="A1:C46"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7199,6 +7323,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="46" spans="1:3" ht="16" customHeight="1">
+      <c r="A46" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-07-24 12:12:08
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1577" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1613" uniqueCount="50">
   <si>
     <t>Date</t>
   </si>
@@ -173,6 +173,9 @@
   <si>
     <t>2026-07-23</t>
   </si>
+  <si>
+    <t>2026-07-24</t>
+  </si>
 </sst>
 </file>
 
@@ -288,7 +291,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -308,7 +311,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -331,7 +334,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -351,7 +354,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -374,7 +377,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -394,7 +397,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -417,7 +420,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -437,7 +440,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -503,7 +506,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -523,7 +526,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -546,7 +549,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -566,7 +569,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -589,7 +592,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -609,7 +612,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -632,7 +635,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -652,7 +655,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -675,7 +678,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -695,7 +698,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -718,7 +721,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>72855</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -738,7 +741,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="7997655" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1078,7 +1081,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C46"/>
+  <dimension ref="A1:C47"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1592,6 +1595,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="47" spans="1:3" ht="16" customHeight="1">
+      <c r="A47" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1600,7 +1614,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C46"/>
+  <dimension ref="A1:C47"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2114,6 +2128,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="47" spans="1:3" ht="16" customHeight="1">
+      <c r="A47" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2122,7 +2147,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C46"/>
+  <dimension ref="A1:C47"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2636,6 +2661,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="47" spans="1:3" ht="16" customHeight="1">
+      <c r="A47" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2644,7 +2680,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C46"/>
+  <dimension ref="A1:C47"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3158,6 +3194,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="47" spans="1:3" ht="16" customHeight="1">
+      <c r="A47" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3166,7 +3213,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C46"/>
+  <dimension ref="A1:C47"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3680,6 +3727,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="47" spans="1:3" ht="16" customHeight="1">
+      <c r="A47" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3688,7 +3746,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C46"/>
+  <dimension ref="A1:C47"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4202,6 +4260,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="47" spans="1:3" ht="16" customHeight="1">
+      <c r="A47" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4210,7 +4279,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C46"/>
+  <dimension ref="A1:C47"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4724,6 +4793,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="47" spans="1:3" ht="16" customHeight="1">
+      <c r="A47" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4732,7 +4812,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C46"/>
+  <dimension ref="A1:C47"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5246,6 +5326,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="47" spans="1:3" ht="16" customHeight="1">
+      <c r="A47" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5254,7 +5345,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C46"/>
+  <dimension ref="A1:C47"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5768,6 +5859,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="47" spans="1:3" ht="16" customHeight="1">
+      <c r="A47" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5776,7 +5878,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C46"/>
+  <dimension ref="A1:C47"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6290,6 +6392,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="47" spans="1:3" ht="16" customHeight="1">
+      <c r="A47" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6298,7 +6411,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C46"/>
+  <dimension ref="A1:C47"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6812,6 +6925,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="47" spans="1:3" ht="16" customHeight="1">
+      <c r="A47" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6820,7 +6944,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C46"/>
+  <dimension ref="A1:C47"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7334,6 +7458,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="47" spans="1:3" ht="16" customHeight="1">
+      <c r="A47" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-07-25 11:56:45
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1613" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1649" uniqueCount="51">
   <si>
     <t>Date</t>
   </si>
@@ -176,6 +176,9 @@
   <si>
     <t>2026-07-24</t>
   </si>
+  <si>
+    <t>2026-07-25</t>
+  </si>
 </sst>
 </file>
 
@@ -291,7 +294,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -311,7 +314,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -334,7 +337,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -354,7 +357,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -377,7 +380,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -397,7 +400,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -420,7 +423,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -440,7 +443,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -506,7 +509,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -526,7 +529,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -549,7 +552,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -569,7 +572,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -592,7 +595,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -612,7 +615,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -635,7 +638,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -655,7 +658,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -678,7 +681,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -698,7 +701,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -721,7 +724,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>72855</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -741,7 +744,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="7997655" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1081,7 +1084,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1606,6 +1609,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="48" spans="1:3" ht="16" customHeight="1">
+      <c r="A48" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1614,7 +1628,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2139,6 +2153,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="48" spans="1:3" ht="16" customHeight="1">
+      <c r="A48" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2147,7 +2172,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2672,6 +2697,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="48" spans="1:3" ht="16" customHeight="1">
+      <c r="A48" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2680,7 +2716,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3205,6 +3241,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="48" spans="1:3" ht="16" customHeight="1">
+      <c r="A48" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3213,7 +3260,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3738,6 +3785,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="48" spans="1:3" ht="16" customHeight="1">
+      <c r="A48" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3746,7 +3804,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4271,6 +4329,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="48" spans="1:3" ht="16" customHeight="1">
+      <c r="A48" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4279,7 +4348,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4804,6 +4873,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="48" spans="1:3" ht="16" customHeight="1">
+      <c r="A48" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4812,7 +4892,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5337,6 +5417,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="48" spans="1:3" ht="16" customHeight="1">
+      <c r="A48" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5345,7 +5436,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5870,6 +5961,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="48" spans="1:3" ht="16" customHeight="1">
+      <c r="A48" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5878,7 +5980,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6403,6 +6505,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="48" spans="1:3" ht="16" customHeight="1">
+      <c r="A48" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6411,7 +6524,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6936,6 +7049,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="48" spans="1:3" ht="16" customHeight="1">
+      <c r="A48" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6944,7 +7068,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7469,6 +7593,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="48" spans="1:3" ht="16" customHeight="1">
+      <c r="A48" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-07-26 11:54:26
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1649" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1685" uniqueCount="52">
   <si>
     <t>Date</t>
   </si>
@@ -178,6 +178,9 @@
   </si>
   <si>
     <t>2026-07-25</t>
+  </si>
+  <si>
+    <t>2026-07-26</t>
   </si>
 </sst>
 </file>
@@ -1084,7 +1087,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C48"/>
+  <dimension ref="A1:C49"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1620,6 +1623,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="49" spans="1:3" ht="16" customHeight="1">
+      <c r="A49" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1628,7 +1642,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C48"/>
+  <dimension ref="A1:C49"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2164,6 +2178,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="49" spans="1:3" ht="16" customHeight="1">
+      <c r="A49" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2172,7 +2197,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C48"/>
+  <dimension ref="A1:C49"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2708,6 +2733,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="49" spans="1:3" ht="16" customHeight="1">
+      <c r="A49" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2716,7 +2752,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C48"/>
+  <dimension ref="A1:C49"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3252,6 +3288,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="49" spans="1:3" ht="16" customHeight="1">
+      <c r="A49" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3260,7 +3307,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C48"/>
+  <dimension ref="A1:C49"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3796,6 +3843,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="49" spans="1:3" ht="16" customHeight="1">
+      <c r="A49" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3804,7 +3862,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C48"/>
+  <dimension ref="A1:C49"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4340,6 +4398,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="49" spans="1:3" ht="16" customHeight="1">
+      <c r="A49" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4348,7 +4417,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C48"/>
+  <dimension ref="A1:C49"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4884,6 +4953,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="49" spans="1:3" ht="16" customHeight="1">
+      <c r="A49" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4892,7 +4972,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C48"/>
+  <dimension ref="A1:C49"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5428,6 +5508,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="49" spans="1:3" ht="16" customHeight="1">
+      <c r="A49" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5436,7 +5527,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C48"/>
+  <dimension ref="A1:C49"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5972,6 +6063,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="49" spans="1:3" ht="16" customHeight="1">
+      <c r="A49" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5980,7 +6082,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C48"/>
+  <dimension ref="A1:C49"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6516,6 +6618,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="49" spans="1:3" ht="16" customHeight="1">
+      <c r="A49" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6524,7 +6637,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C48"/>
+  <dimension ref="A1:C49"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7060,6 +7173,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="49" spans="1:3" ht="16" customHeight="1">
+      <c r="A49" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7068,7 +7192,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C48"/>
+  <dimension ref="A1:C49"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7604,6 +7728,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="49" spans="1:3" ht="16" customHeight="1">
+      <c r="A49" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-07-27 (recovered from clobbered push)
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1685" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1721" uniqueCount="53">
   <si>
     <t>Date</t>
   </si>
@@ -182,6 +182,9 @@
   <si>
     <t>2026-07-26</t>
   </si>
+  <si>
+    <t>2026-07-27</t>
+  </si>
 </sst>
 </file>
 
@@ -297,9 +300,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>100991</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>139013</xdr:rowOff>
+      <xdr:rowOff>117911</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -317,7 +320,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8025791" cy="4347011"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -340,9 +343,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>100991</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>139013</xdr:rowOff>
+      <xdr:rowOff>117911</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -360,7 +363,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8025791" cy="4347011"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -383,9 +386,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>100991</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>139013</xdr:rowOff>
+      <xdr:rowOff>117911</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -403,7 +406,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8025791" cy="4347011"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -426,9 +429,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>93957</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>139013</xdr:rowOff>
+      <xdr:rowOff>117911</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -446,7 +449,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8018757" cy="4347011"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -469,7 +472,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>213535</xdr:colOff>
+      <xdr:colOff>206501</xdr:colOff>
       <xdr:row>22</xdr:row>
       <xdr:rowOff>51532</xdr:rowOff>
     </xdr:to>
@@ -489,7 +492,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8138335" cy="4480657"/>
+          <a:ext cx="8131301" cy="4480657"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -512,9 +515,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>100991</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>139013</xdr:rowOff>
+      <xdr:rowOff>117911</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -532,7 +535,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8025791" cy="4347011"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -555,9 +558,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>100991</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>139013</xdr:rowOff>
+      <xdr:rowOff>117911</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -575,7 +578,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8025791" cy="4347011"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -598,9 +601,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>100991</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>139013</xdr:rowOff>
+      <xdr:rowOff>117911</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -618,7 +621,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8025791" cy="4347011"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -641,9 +644,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>100991</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>139013</xdr:rowOff>
+      <xdr:rowOff>117911</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -661,7 +664,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8025791" cy="4347011"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -684,9 +687,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>100991</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>139013</xdr:rowOff>
+      <xdr:rowOff>117911</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -704,7 +707,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8025791" cy="4347011"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -727,9 +730,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>100991</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>139013</xdr:rowOff>
+      <xdr:rowOff>117911</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -747,7 +750,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8025791" cy="4347011"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -770,7 +773,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>213535</xdr:colOff>
+      <xdr:colOff>206501</xdr:colOff>
       <xdr:row>22</xdr:row>
       <xdr:rowOff>51532</xdr:rowOff>
     </xdr:to>
@@ -790,7 +793,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8138335" cy="4480657"/>
+          <a:ext cx="8131301" cy="4480657"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1087,7 +1090,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C49"/>
+  <dimension ref="A1:C50"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1634,6 +1637,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="50" spans="1:3" ht="16" customHeight="1">
+      <c r="A50" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1642,7 +1656,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C49"/>
+  <dimension ref="A1:C50"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2189,6 +2203,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="50" spans="1:3" ht="16" customHeight="1">
+      <c r="A50" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2197,7 +2222,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C49"/>
+  <dimension ref="A1:C50"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2744,6 +2769,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="50" spans="1:3" ht="16" customHeight="1">
+      <c r="A50" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2752,7 +2788,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C49"/>
+  <dimension ref="A1:C50"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3299,6 +3335,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="50" spans="1:3" ht="16" customHeight="1">
+      <c r="A50" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3307,7 +3354,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C49"/>
+  <dimension ref="A1:C50"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3854,6 +3901,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="50" spans="1:3" ht="16" customHeight="1">
+      <c r="A50" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3862,7 +3920,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C49"/>
+  <dimension ref="A1:C50"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4409,6 +4467,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="50" spans="1:3" ht="16" customHeight="1">
+      <c r="A50" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4417,7 +4486,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C49"/>
+  <dimension ref="A1:C50"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4964,6 +5033,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="50" spans="1:3" ht="16" customHeight="1">
+      <c r="A50" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4972,7 +5052,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C49"/>
+  <dimension ref="A1:C50"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5519,6 +5599,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="50" spans="1:3" ht="16" customHeight="1">
+      <c r="A50" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5527,7 +5618,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C49"/>
+  <dimension ref="A1:C50"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6074,6 +6165,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="50" spans="1:3" ht="16" customHeight="1">
+      <c r="A50" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6082,7 +6184,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C49"/>
+  <dimension ref="A1:C50"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6629,6 +6731,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="50" spans="1:3" ht="16" customHeight="1">
+      <c r="A50" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6637,7 +6750,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C49"/>
+  <dimension ref="A1:C50"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7184,6 +7297,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="50" spans="1:3" ht="16" customHeight="1">
+      <c r="A50" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7192,7 +7316,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C49"/>
+  <dimension ref="A1:C50"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7739,6 +7863,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="50" spans="1:3" ht="16" customHeight="1">
+      <c r="A50" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-07-27 04:15:35
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -300,9 +300,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>100991</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>117911</xdr:rowOff>
+      <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -320,7 +320,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8025791" cy="4347011"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -343,9 +343,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>100991</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>117911</xdr:rowOff>
+      <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -363,7 +363,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8025791" cy="4347011"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -386,9 +386,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>100991</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>117911</xdr:rowOff>
+      <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -406,7 +406,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8025791" cy="4347011"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -429,9 +429,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>93957</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>117911</xdr:rowOff>
+      <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -449,7 +449,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8018757" cy="4347011"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -472,7 +472,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>206501</xdr:colOff>
+      <xdr:colOff>213535</xdr:colOff>
       <xdr:row>22</xdr:row>
       <xdr:rowOff>51532</xdr:rowOff>
     </xdr:to>
@@ -492,7 +492,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8131301" cy="4480657"/>
+          <a:ext cx="8138335" cy="4480657"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -515,9 +515,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>100991</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>117911</xdr:rowOff>
+      <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -535,7 +535,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8025791" cy="4347011"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -558,9 +558,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>100991</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>117911</xdr:rowOff>
+      <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -578,7 +578,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8025791" cy="4347011"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -601,9 +601,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>100991</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>117911</xdr:rowOff>
+      <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -621,7 +621,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8025791" cy="4347011"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -644,9 +644,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>100991</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>117911</xdr:rowOff>
+      <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -664,7 +664,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8025791" cy="4347011"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -687,9 +687,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>100991</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>117911</xdr:rowOff>
+      <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -707,7 +707,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8025791" cy="4347011"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -730,9 +730,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>100991</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>117911</xdr:rowOff>
+      <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -750,7 +750,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8025791" cy="4347011"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -773,7 +773,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>206501</xdr:colOff>
+      <xdr:colOff>213535</xdr:colOff>
       <xdr:row>22</xdr:row>
       <xdr:rowOff>51532</xdr:rowOff>
     </xdr:to>
@@ -793,7 +793,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8131301" cy="4480657"/>
+          <a:ext cx="8138335" cy="4480657"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-07-28 12:28:56
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1721" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1757" uniqueCount="54">
   <si>
     <t>Date</t>
   </si>
@@ -184,6 +184,9 @@
   </si>
   <si>
     <t>2026-07-27</t>
+  </si>
+  <si>
+    <t>2026-07-28</t>
   </si>
 </sst>
 </file>
@@ -1090,7 +1093,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C50"/>
+  <dimension ref="A1:C51"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1648,6 +1651,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="51" spans="1:3" ht="16" customHeight="1">
+      <c r="A51" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1656,7 +1670,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C50"/>
+  <dimension ref="A1:C51"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2214,6 +2228,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="51" spans="1:3" ht="16" customHeight="1">
+      <c r="A51" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2222,7 +2247,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C50"/>
+  <dimension ref="A1:C51"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2780,6 +2805,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="51" spans="1:3" ht="16" customHeight="1">
+      <c r="A51" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2788,7 +2824,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C50"/>
+  <dimension ref="A1:C51"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3346,6 +3382,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="51" spans="1:3" ht="16" customHeight="1">
+      <c r="A51" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3354,7 +3401,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C50"/>
+  <dimension ref="A1:C51"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3912,6 +3959,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="51" spans="1:3" ht="16" customHeight="1">
+      <c r="A51" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3920,7 +3978,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C50"/>
+  <dimension ref="A1:C51"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4478,6 +4536,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="51" spans="1:3" ht="16" customHeight="1">
+      <c r="A51" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4486,7 +4555,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C50"/>
+  <dimension ref="A1:C51"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5044,6 +5113,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="51" spans="1:3" ht="16" customHeight="1">
+      <c r="A51" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5052,7 +5132,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C50"/>
+  <dimension ref="A1:C51"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5610,6 +5690,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="51" spans="1:3" ht="16" customHeight="1">
+      <c r="A51" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5618,7 +5709,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C50"/>
+  <dimension ref="A1:C51"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6176,6 +6267,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="51" spans="1:3" ht="16" customHeight="1">
+      <c r="A51" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6184,7 +6286,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C50"/>
+  <dimension ref="A1:C51"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6742,6 +6844,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="51" spans="1:3" ht="16" customHeight="1">
+      <c r="A51" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6750,7 +6863,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C50"/>
+  <dimension ref="A1:C51"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7308,6 +7421,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="51" spans="1:3" ht="16" customHeight="1">
+      <c r="A51" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7316,7 +7440,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C50"/>
+  <dimension ref="A1:C51"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7874,6 +7998,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="51" spans="1:3" ht="16" customHeight="1">
+      <c r="A51" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-07-29 12:53:38
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1757" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1793" uniqueCount="55">
   <si>
     <t>Date</t>
   </si>
@@ -187,6 +187,9 @@
   </si>
   <si>
     <t>2026-07-28</t>
+  </si>
+  <si>
+    <t>2026-07-29</t>
   </si>
 </sst>
 </file>
@@ -1093,7 +1096,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C51"/>
+  <dimension ref="A1:C52"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1662,6 +1665,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="52" spans="1:3" ht="16" customHeight="1">
+      <c r="A52" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1670,7 +1684,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C51"/>
+  <dimension ref="A1:C52"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2239,6 +2253,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="52" spans="1:3" ht="16" customHeight="1">
+      <c r="A52" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2247,7 +2272,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C51"/>
+  <dimension ref="A1:C52"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2816,6 +2841,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="52" spans="1:3" ht="16" customHeight="1">
+      <c r="A52" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2824,7 +2860,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C51"/>
+  <dimension ref="A1:C52"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3393,6 +3429,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="52" spans="1:3" ht="16" customHeight="1">
+      <c r="A52" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3401,7 +3448,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C51"/>
+  <dimension ref="A1:C52"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3970,6 +4017,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="52" spans="1:3" ht="16" customHeight="1">
+      <c r="A52" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3978,7 +4036,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C51"/>
+  <dimension ref="A1:C52"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4547,6 +4605,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="52" spans="1:3" ht="16" customHeight="1">
+      <c r="A52" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4555,7 +4624,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C51"/>
+  <dimension ref="A1:C52"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5124,6 +5193,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="52" spans="1:3" ht="16" customHeight="1">
+      <c r="A52" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5132,7 +5212,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C51"/>
+  <dimension ref="A1:C52"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5701,6 +5781,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="52" spans="1:3" ht="16" customHeight="1">
+      <c r="A52" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5709,7 +5800,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C51"/>
+  <dimension ref="A1:C52"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6278,6 +6369,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="52" spans="1:3" ht="16" customHeight="1">
+      <c r="A52" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6286,7 +6388,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C51"/>
+  <dimension ref="A1:C52"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6855,6 +6957,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="52" spans="1:3" ht="16" customHeight="1">
+      <c r="A52" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6863,7 +6976,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C51"/>
+  <dimension ref="A1:C52"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7432,6 +7545,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="52" spans="1:3" ht="16" customHeight="1">
+      <c r="A52" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7440,7 +7564,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C51"/>
+  <dimension ref="A1:C52"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8009,6 +8133,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="52" spans="1:3" ht="16" customHeight="1">
+      <c r="A52" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-07-30 12:21:19
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1793" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1829" uniqueCount="56">
   <si>
     <t>Date</t>
   </si>
@@ -190,6 +190,9 @@
   </si>
   <si>
     <t>2026-07-29</t>
+  </si>
+  <si>
+    <t>2026-07-30</t>
   </si>
 </sst>
 </file>
@@ -1096,7 +1099,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C52"/>
+  <dimension ref="A1:C53"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1676,6 +1679,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="53" spans="1:3" ht="16" customHeight="1">
+      <c r="A53" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1684,7 +1698,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C52"/>
+  <dimension ref="A1:C53"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2264,6 +2278,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="53" spans="1:3" ht="16" customHeight="1">
+      <c r="A53" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2272,7 +2297,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C52"/>
+  <dimension ref="A1:C53"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2852,6 +2877,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="53" spans="1:3" ht="16" customHeight="1">
+      <c r="A53" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2860,7 +2896,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C52"/>
+  <dimension ref="A1:C53"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3440,6 +3476,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="53" spans="1:3" ht="16" customHeight="1">
+      <c r="A53" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3448,7 +3495,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C52"/>
+  <dimension ref="A1:C53"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4028,6 +4075,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="53" spans="1:3" ht="16" customHeight="1">
+      <c r="A53" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4036,7 +4094,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C52"/>
+  <dimension ref="A1:C53"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4616,6 +4674,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="53" spans="1:3" ht="16" customHeight="1">
+      <c r="A53" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4624,7 +4693,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C52"/>
+  <dimension ref="A1:C53"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5204,6 +5273,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="53" spans="1:3" ht="16" customHeight="1">
+      <c r="A53" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5212,7 +5292,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C52"/>
+  <dimension ref="A1:C53"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5792,6 +5872,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="53" spans="1:3" ht="16" customHeight="1">
+      <c r="A53" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5800,7 +5891,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C52"/>
+  <dimension ref="A1:C53"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6380,6 +6471,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="53" spans="1:3" ht="16" customHeight="1">
+      <c r="A53" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6388,7 +6490,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C52"/>
+  <dimension ref="A1:C53"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6968,6 +7070,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="53" spans="1:3" ht="16" customHeight="1">
+      <c r="A53" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6976,7 +7089,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C52"/>
+  <dimension ref="A1:C53"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7556,6 +7669,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="53" spans="1:3" ht="16" customHeight="1">
+      <c r="A53" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7564,7 +7688,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C52"/>
+  <dimension ref="A1:C53"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8144,6 +8268,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="53" spans="1:3" ht="16" customHeight="1">
+      <c r="A53" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-07-31 12:52:51
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1829" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1865" uniqueCount="57">
   <si>
     <t>Date</t>
   </si>
@@ -193,6 +193,9 @@
   </si>
   <si>
     <t>2026-07-30</t>
+  </si>
+  <si>
+    <t>2026-07-31</t>
   </si>
 </sst>
 </file>
@@ -1099,7 +1102,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1690,6 +1693,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="54" spans="1:3" ht="16" customHeight="1">
+      <c r="A54" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1698,7 +1712,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2289,6 +2303,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="54" spans="1:3" ht="16" customHeight="1">
+      <c r="A54" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2297,7 +2322,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2888,6 +2913,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="54" spans="1:3" ht="16" customHeight="1">
+      <c r="A54" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2896,7 +2932,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3487,6 +3523,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="54" spans="1:3" ht="16" customHeight="1">
+      <c r="A54" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3495,7 +3542,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4086,6 +4133,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="54" spans="1:3" ht="16" customHeight="1">
+      <c r="A54" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4094,7 +4152,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4685,6 +4743,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="54" spans="1:3" ht="16" customHeight="1">
+      <c r="A54" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4693,7 +4762,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5284,6 +5353,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="54" spans="1:3" ht="16" customHeight="1">
+      <c r="A54" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5292,7 +5372,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5883,6 +5963,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="54" spans="1:3" ht="16" customHeight="1">
+      <c r="A54" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5891,7 +5982,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6482,6 +6573,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="54" spans="1:3" ht="16" customHeight="1">
+      <c r="A54" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6490,7 +6592,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7081,6 +7183,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="54" spans="1:3" ht="16" customHeight="1">
+      <c r="A54" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7089,7 +7202,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7680,6 +7793,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="54" spans="1:3" ht="16" customHeight="1">
+      <c r="A54" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7688,7 +7812,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8279,6 +8403,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="54" spans="1:3" ht="16" customHeight="1">
+      <c r="A54" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-08-01 11:54:05
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1865" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1901" uniqueCount="58">
   <si>
     <t>Date</t>
   </si>
@@ -196,6 +196,9 @@
   </si>
   <si>
     <t>2026-07-31</t>
+  </si>
+  <si>
+    <t>2026-08-01</t>
   </si>
 </sst>
 </file>
@@ -1102,7 +1105,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C54"/>
+  <dimension ref="A1:C55"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1704,6 +1707,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="55" spans="1:3" ht="16" customHeight="1">
+      <c r="A55" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1712,7 +1726,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C54"/>
+  <dimension ref="A1:C55"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2314,6 +2328,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="55" spans="1:3" ht="16" customHeight="1">
+      <c r="A55" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2322,7 +2347,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C54"/>
+  <dimension ref="A1:C55"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2924,6 +2949,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="55" spans="1:3" ht="16" customHeight="1">
+      <c r="A55" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2932,7 +2968,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C54"/>
+  <dimension ref="A1:C55"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3534,6 +3570,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="55" spans="1:3" ht="16" customHeight="1">
+      <c r="A55" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3542,7 +3589,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C54"/>
+  <dimension ref="A1:C55"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4144,6 +4191,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="55" spans="1:3" ht="16" customHeight="1">
+      <c r="A55" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4152,7 +4210,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C54"/>
+  <dimension ref="A1:C55"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4754,6 +4812,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="55" spans="1:3" ht="16" customHeight="1">
+      <c r="A55" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4762,7 +4831,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C54"/>
+  <dimension ref="A1:C55"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5364,6 +5433,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="55" spans="1:3" ht="16" customHeight="1">
+      <c r="A55" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5372,7 +5452,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C54"/>
+  <dimension ref="A1:C55"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5974,6 +6054,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="55" spans="1:3" ht="16" customHeight="1">
+      <c r="A55" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5982,7 +6073,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C54"/>
+  <dimension ref="A1:C55"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6584,6 +6675,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="55" spans="1:3" ht="16" customHeight="1">
+      <c r="A55" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6592,7 +6694,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C54"/>
+  <dimension ref="A1:C55"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7194,6 +7296,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="55" spans="1:3" ht="16" customHeight="1">
+      <c r="A55" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7202,7 +7315,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C54"/>
+  <dimension ref="A1:C55"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7804,6 +7917,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="55" spans="1:3" ht="16" customHeight="1">
+      <c r="A55" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7812,7 +7936,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C54"/>
+  <dimension ref="A1:C55"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8414,6 +8538,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="55" spans="1:3" ht="16" customHeight="1">
+      <c r="A55" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Replace Playwright pagination with direct gpuindexes.com API calls
gpuperhour.com's own pagination has a client-side hydration bug: clicking
"Next" fires the correct backend request but the table never re-renders,
so scraping was silently stuck on page 1 (20 consumer-GPU rows) almost
every day since mid-June. Since the site's frontend is backed by a public,
unauthenticated JSON API (api.gpuindexes.com/api/offers), scrape.py now
pages through that directly instead of driving a browser — no more
click races, no Playwright/Chromium dependency in CI.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1829" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1854" uniqueCount="57">
   <si>
     <t>Date</t>
   </si>
@@ -194,6 +194,9 @@
   <si>
     <t>2026-07-30</t>
   </si>
+  <si>
+    <t>2026-07-31</t>
+  </si>
 </sst>
 </file>
 
@@ -309,9 +312,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>100991</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>139013</xdr:rowOff>
+      <xdr:rowOff>117911</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -329,7 +332,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8025791" cy="4347011"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -352,9 +355,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>100991</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>139013</xdr:rowOff>
+      <xdr:rowOff>117911</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -372,7 +375,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8025791" cy="4347011"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -395,9 +398,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>100991</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>139013</xdr:rowOff>
+      <xdr:rowOff>117911</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -415,7 +418,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8025791" cy="4347011"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -438,9 +441,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>100991</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>139013</xdr:rowOff>
+      <xdr:rowOff>117911</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -458,7 +461,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8025791" cy="4347011"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -481,7 +484,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>213535</xdr:colOff>
+      <xdr:colOff>206501</xdr:colOff>
       <xdr:row>22</xdr:row>
       <xdr:rowOff>51532</xdr:rowOff>
     </xdr:to>
@@ -501,7 +504,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8138335" cy="4480657"/>
+          <a:ext cx="8131301" cy="4480657"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -524,9 +527,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>100991</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>139013</xdr:rowOff>
+      <xdr:rowOff>117911</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -544,7 +547,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8025791" cy="4347011"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -567,9 +570,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>100991</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>139013</xdr:rowOff>
+      <xdr:rowOff>117911</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -587,7 +590,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8025791" cy="4347011"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -610,9 +613,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>100991</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>139013</xdr:rowOff>
+      <xdr:rowOff>117911</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -630,7 +633,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8025791" cy="4347011"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -653,9 +656,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>100991</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>139013</xdr:rowOff>
+      <xdr:rowOff>117911</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -673,7 +676,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8025791" cy="4347011"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -696,9 +699,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>100991</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>139013</xdr:rowOff>
+      <xdr:rowOff>117911</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -716,7 +719,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8025791" cy="4347011"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -739,9 +742,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>100991</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>139013</xdr:rowOff>
+      <xdr:rowOff>117911</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -759,7 +762,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8025791" cy="4347011"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -782,7 +785,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>213535</xdr:colOff>
+      <xdr:colOff>206501</xdr:colOff>
       <xdr:row>22</xdr:row>
       <xdr:rowOff>51532</xdr:rowOff>
     </xdr:to>
@@ -802,7 +805,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8138335" cy="4480657"/>
+          <a:ext cx="8131301" cy="4480657"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1099,7 +1102,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1690,6 +1693,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="54" spans="1:3" ht="16" customHeight="1">
+      <c r="A54" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1698,7 +1712,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2289,6 +2303,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="54" spans="1:3" ht="16" customHeight="1">
+      <c r="A54" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B54" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2297,7 +2322,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2888,6 +2913,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="54" spans="1:3" ht="16" customHeight="1">
+      <c r="A54" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B54" s="3">
+        <v>0.88</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2896,7 +2932,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3487,6 +3523,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="54" spans="1:3" ht="16" customHeight="1">
+      <c r="A54" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C54" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3495,7 +3542,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4086,6 +4133,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="54" spans="1:3" ht="16" customHeight="1">
+      <c r="A54" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4094,7 +4152,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4685,6 +4743,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="54" spans="1:3" ht="16" customHeight="1">
+      <c r="A54" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B54" s="3">
+        <v>6.11</v>
+      </c>
+      <c r="C54" s="3">
+        <v>6.6875</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4693,7 +4762,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5284,6 +5353,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="54" spans="1:3" ht="16" customHeight="1">
+      <c r="A54" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5292,7 +5372,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5883,6 +5963,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="54" spans="1:3" ht="16" customHeight="1">
+      <c r="A54" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B54" s="3">
+        <v>4</v>
+      </c>
+      <c r="C54" s="3">
+        <v>3.6842</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5891,7 +5982,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6482,6 +6573,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="54" spans="1:3" ht="16" customHeight="1">
+      <c r="A54" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B54" s="3">
+        <v>2.29</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6490,7 +6592,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7081,6 +7183,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="54" spans="1:3" ht="16" customHeight="1">
+      <c r="A54" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B54" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C54" s="3">
+        <v>3.3929</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7089,7 +7202,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7680,6 +7793,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="54" spans="1:3" ht="16" customHeight="1">
+      <c r="A54" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B54" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7688,7 +7812,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8279,6 +8403,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="54" spans="1:3" ht="16" customHeight="1">
+      <c r="A54" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-08-01 18:40:23
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1890" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1875" uniqueCount="58">
   <si>
     <t>Date</t>
   </si>
@@ -315,9 +315,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>100991</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>117911</xdr:rowOff>
+      <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -335,7 +335,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8025791" cy="4347011"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -358,9 +358,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>100991</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>117911</xdr:rowOff>
+      <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -378,7 +378,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8025791" cy="4347011"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -401,9 +401,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>100991</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>117911</xdr:rowOff>
+      <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -421,7 +421,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8025791" cy="4347011"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -444,9 +444,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>100991</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>117911</xdr:rowOff>
+      <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -464,7 +464,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8025791" cy="4347011"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -487,7 +487,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>206501</xdr:colOff>
+      <xdr:colOff>213535</xdr:colOff>
       <xdr:row>22</xdr:row>
       <xdr:rowOff>51532</xdr:rowOff>
     </xdr:to>
@@ -507,7 +507,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8131301" cy="4480657"/>
+          <a:ext cx="8138335" cy="4480657"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -530,9 +530,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>100991</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>117911</xdr:rowOff>
+      <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -550,7 +550,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8025791" cy="4347011"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -573,9 +573,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>100991</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>117911</xdr:rowOff>
+      <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -593,7 +593,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8025791" cy="4347011"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -616,9 +616,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>100991</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>117911</xdr:rowOff>
+      <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -636,7 +636,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8025791" cy="4347011"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -659,9 +659,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>100991</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>117911</xdr:rowOff>
+      <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -679,7 +679,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8025791" cy="4347011"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -702,9 +702,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>100991</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>117911</xdr:rowOff>
+      <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -722,7 +722,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8025791" cy="4347011"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -745,9 +745,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>100991</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>117911</xdr:rowOff>
+      <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -765,7 +765,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8025791" cy="4347011"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -788,7 +788,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>206501</xdr:colOff>
+      <xdr:colOff>213535</xdr:colOff>
       <xdr:row>22</xdr:row>
       <xdr:rowOff>51532</xdr:rowOff>
     </xdr:to>
@@ -808,7 +808,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8131301" cy="4480657"/>
+          <a:ext cx="8138335" cy="4480657"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1711,8 +1711,8 @@
       <c r="A55" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B55" s="4" t="s">
-        <v>4</v>
+      <c r="B55" s="3">
+        <v>7.5</v>
       </c>
       <c r="C55" s="4" t="s">
         <v>4</v>
@@ -2332,8 +2332,8 @@
       <c r="A55" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B55" s="4" t="s">
-        <v>4</v>
+      <c r="B55" s="3">
+        <v>2.99</v>
       </c>
       <c r="C55" s="4" t="s">
         <v>4</v>
@@ -2953,11 +2953,11 @@
       <c r="A55" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B55" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C55" s="4" t="s">
-        <v>4</v>
+      <c r="B55" s="3">
+        <v>0.88</v>
+      </c>
+      <c r="C55" s="3">
+        <v>0.8</v>
       </c>
     </row>
   </sheetData>
@@ -3577,8 +3577,8 @@
       <c r="B55" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C55" s="4" t="s">
-        <v>4</v>
+      <c r="C55" s="3">
+        <v>0.9115</v>
       </c>
     </row>
   </sheetData>
@@ -4816,11 +4816,11 @@
       <c r="A55" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B55" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C55" s="4" t="s">
-        <v>4</v>
+      <c r="B55" s="3">
+        <v>6.11</v>
+      </c>
+      <c r="C55" s="3">
+        <v>6.25</v>
       </c>
     </row>
   </sheetData>
@@ -5437,11 +5437,11 @@
       <c r="A55" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B55" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C55" s="4" t="s">
-        <v>4</v>
+      <c r="B55" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C55" s="3">
+        <v>4.6866</v>
       </c>
     </row>
   </sheetData>
@@ -6058,7 +6058,7 @@
       <c r="A55" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B55" s="4" t="s">
+      <c r="B55" s="3">
         <v>4</v>
       </c>
       <c r="C55" s="4" t="s">
@@ -6679,8 +6679,8 @@
       <c r="A55" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B55" s="4" t="s">
-        <v>4</v>
+      <c r="B55" s="3">
+        <v>2.29</v>
       </c>
       <c r="C55" s="4" t="s">
         <v>4</v>
@@ -7300,11 +7300,11 @@
       <c r="A55" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B55" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C55" s="4" t="s">
-        <v>4</v>
+      <c r="B55" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C55" s="3">
+        <v>3.3929</v>
       </c>
     </row>
   </sheetData>
@@ -7921,11 +7921,11 @@
       <c r="A55" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B55" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C55" s="4" t="s">
-        <v>4</v>
+      <c r="B55" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C55" s="3">
+        <v>2.1813</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-08-02 11:51:00
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1875" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1897" uniqueCount="59">
   <si>
     <t>Date</t>
   </si>
@@ -200,6 +200,9 @@
   <si>
     <t>2026-08-01</t>
   </si>
+  <si>
+    <t>2026-08-02</t>
+  </si>
 </sst>
 </file>
 
@@ -315,7 +318,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -335,7 +338,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -358,7 +361,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -378,7 +381,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -401,7 +404,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -421,7 +424,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -444,7 +447,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -464,7 +467,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -530,7 +533,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -550,7 +553,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -573,7 +576,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -593,7 +596,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -616,7 +619,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -636,7 +639,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -659,7 +662,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -679,7 +682,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -702,7 +705,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -722,7 +725,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -745,7 +748,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -765,7 +768,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1105,7 +1108,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C55"/>
+  <dimension ref="A1:C56"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1718,6 +1721,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="56" spans="1:3" ht="16" customHeight="1">
+      <c r="A56" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B56" s="3">
+        <v>7.5</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1726,7 +1740,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C55"/>
+  <dimension ref="A1:C56"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2339,6 +2353,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="56" spans="1:3" ht="16" customHeight="1">
+      <c r="A56" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B56" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2347,7 +2372,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C55"/>
+  <dimension ref="A1:C56"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2960,6 +2985,17 @@
         <v>0.8</v>
       </c>
     </row>
+    <row r="56" spans="1:3" ht="16" customHeight="1">
+      <c r="A56" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B56" s="3">
+        <v>0.88</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2968,7 +3004,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C55"/>
+  <dimension ref="A1:C56"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3581,6 +3617,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="56" spans="1:3" ht="16" customHeight="1">
+      <c r="A56" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C56" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3589,7 +3636,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C55"/>
+  <dimension ref="A1:C56"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4202,6 +4249,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="56" spans="1:3" ht="16" customHeight="1">
+      <c r="A56" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4210,7 +4268,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C55"/>
+  <dimension ref="A1:C56"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4823,6 +4881,17 @@
         <v>6.25</v>
       </c>
     </row>
+    <row r="56" spans="1:3" ht="16" customHeight="1">
+      <c r="A56" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B56" s="3">
+        <v>6.11</v>
+      </c>
+      <c r="C56" s="3">
+        <v>5.9125</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4831,7 +4900,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C55"/>
+  <dimension ref="A1:C56"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5444,6 +5513,17 @@
         <v>4.6866</v>
       </c>
     </row>
+    <row r="56" spans="1:3" ht="16" customHeight="1">
+      <c r="A56" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B56" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C56" s="3">
+        <v>4.1373</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5452,7 +5532,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C55"/>
+  <dimension ref="A1:C56"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6065,6 +6145,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="56" spans="1:3" ht="16" customHeight="1">
+      <c r="A56" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B56" s="3">
+        <v>3.99</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6073,7 +6164,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C55"/>
+  <dimension ref="A1:C56"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6686,6 +6777,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="56" spans="1:3" ht="16" customHeight="1">
+      <c r="A56" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B56" s="3">
+        <v>1.99</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6694,7 +6796,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C55"/>
+  <dimension ref="A1:C56"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7307,6 +7409,17 @@
         <v>3.3929</v>
       </c>
     </row>
+    <row r="56" spans="1:3" ht="16" customHeight="1">
+      <c r="A56" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B56" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C56" s="3">
+        <v>2.2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7315,7 +7428,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C55"/>
+  <dimension ref="A1:C56"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7928,6 +8041,17 @@
         <v>2.1813</v>
       </c>
     </row>
+    <row r="56" spans="1:3" ht="16" customHeight="1">
+      <c r="A56" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B56" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C56" s="3">
+        <v>2.2533</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7936,7 +8060,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C55"/>
+  <dimension ref="A1:C56"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8549,6 +8673,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="56" spans="1:3" ht="16" customHeight="1">
+      <c r="A56" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-08-03 13:32:46
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1897" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1921" uniqueCount="60">
   <si>
     <t>Date</t>
   </si>
@@ -203,6 +203,9 @@
   <si>
     <t>2026-08-02</t>
   </si>
+  <si>
+    <t>2026-08-03</t>
+  </si>
 </sst>
 </file>
 
@@ -318,7 +321,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -338,7 +341,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -361,7 +364,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -381,7 +384,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -404,7 +407,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -424,7 +427,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -447,7 +450,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -467,7 +470,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -533,7 +536,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -553,7 +556,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -576,7 +579,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -596,7 +599,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -619,7 +622,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -639,7 +642,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -662,7 +665,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -682,7 +685,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -705,7 +708,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -725,7 +728,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -748,7 +751,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -768,7 +771,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1108,7 +1111,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:C57"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1732,6 +1735,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="57" spans="1:3" ht="16" customHeight="1">
+      <c r="A57" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1740,7 +1754,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:C57"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2364,6 +2378,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="57" spans="1:3" ht="16" customHeight="1">
+      <c r="A57" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B57" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2372,7 +2397,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:C57"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2996,6 +3021,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="57" spans="1:3" ht="16" customHeight="1">
+      <c r="A57" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B57" s="3">
+        <v>0.88</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3004,7 +3040,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:C57"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3628,6 +3664,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="57" spans="1:3" ht="16" customHeight="1">
+      <c r="A57" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C57" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3636,7 +3683,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:C57"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4260,6 +4307,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="57" spans="1:3" ht="16" customHeight="1">
+      <c r="A57" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4268,7 +4326,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:C57"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4892,6 +4950,17 @@
         <v>5.9125</v>
       </c>
     </row>
+    <row r="57" spans="1:3" ht="16" customHeight="1">
+      <c r="A57" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C57" s="3">
+        <v>5.875</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4900,7 +4969,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:C57"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5524,6 +5593,17 @@
         <v>4.1373</v>
       </c>
     </row>
+    <row r="57" spans="1:3" ht="16" customHeight="1">
+      <c r="A57" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B57" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C57" s="3">
+        <v>4.8867</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5532,7 +5612,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:C57"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6156,6 +6236,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="57" spans="1:3" ht="16" customHeight="1">
+      <c r="A57" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B57" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6164,7 +6255,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:C57"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6788,6 +6879,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="57" spans="1:3" ht="16" customHeight="1">
+      <c r="A57" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B57" s="3">
+        <v>2.29</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6796,7 +6898,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:C57"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7420,6 +7522,17 @@
         <v>2.2</v>
       </c>
     </row>
+    <row r="57" spans="1:3" ht="16" customHeight="1">
+      <c r="A57" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B57" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C57" s="3">
+        <v>2.4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7428,7 +7541,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:C57"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8052,6 +8165,17 @@
         <v>2.2533</v>
       </c>
     </row>
+    <row r="57" spans="1:3" ht="16" customHeight="1">
+      <c r="A57" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B57" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C57" s="3">
+        <v>2.5453</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8060,7 +8184,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:C57"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8684,6 +8808,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="57" spans="1:3" ht="16" customHeight="1">
+      <c r="A57" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-08-04 12:51:43
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1921" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1946" uniqueCount="61">
   <si>
     <t>Date</t>
   </si>
@@ -205,6 +205,9 @@
   </si>
   <si>
     <t>2026-08-03</t>
+  </si>
+  <si>
+    <t>2026-08-04</t>
   </si>
 </sst>
 </file>
@@ -1111,7 +1114,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C57"/>
+  <dimension ref="A1:C58"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1746,6 +1749,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="58" spans="1:3" ht="16" customHeight="1">
+      <c r="A58" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B58" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C58" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1754,7 +1768,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C57"/>
+  <dimension ref="A1:C58"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2389,6 +2403,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="58" spans="1:3" ht="16" customHeight="1">
+      <c r="A58" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B58" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C58" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2397,7 +2422,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C57"/>
+  <dimension ref="A1:C58"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3032,6 +3057,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="58" spans="1:3" ht="16" customHeight="1">
+      <c r="A58" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B58" s="3">
+        <v>0.88</v>
+      </c>
+      <c r="C58" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3040,7 +3076,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C57"/>
+  <dimension ref="A1:C58"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3675,6 +3711,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="58" spans="1:3" ht="16" customHeight="1">
+      <c r="A58" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B58" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C58" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3683,7 +3730,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C57"/>
+  <dimension ref="A1:C58"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4318,6 +4365,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="58" spans="1:3" ht="16" customHeight="1">
+      <c r="A58" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B58" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C58" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4326,7 +4384,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C57"/>
+  <dimension ref="A1:C58"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4961,6 +5019,17 @@
         <v>5.875</v>
       </c>
     </row>
+    <row r="58" spans="1:3" ht="16" customHeight="1">
+      <c r="A58" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B58" s="3">
+        <v>6.11</v>
+      </c>
+      <c r="C58" s="3">
+        <v>5.875</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4969,7 +5038,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C57"/>
+  <dimension ref="A1:C58"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5604,6 +5673,17 @@
         <v>4.8867</v>
       </c>
     </row>
+    <row r="58" spans="1:3" ht="16" customHeight="1">
+      <c r="A58" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B58" s="3">
+        <v>4.47</v>
+      </c>
+      <c r="C58" s="3">
+        <v>3.4787</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5612,7 +5692,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C57"/>
+  <dimension ref="A1:C58"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6247,6 +6327,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="58" spans="1:3" ht="16" customHeight="1">
+      <c r="A58" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B58" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C58" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6255,7 +6346,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C57"/>
+  <dimension ref="A1:C58"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6890,6 +6981,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="58" spans="1:3" ht="16" customHeight="1">
+      <c r="A58" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B58" s="3">
+        <v>1.99</v>
+      </c>
+      <c r="C58" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6898,7 +7000,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C57"/>
+  <dimension ref="A1:C58"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7533,6 +7635,17 @@
         <v>2.4</v>
       </c>
     </row>
+    <row r="58" spans="1:3" ht="16" customHeight="1">
+      <c r="A58" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B58" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C58" s="3">
+        <v>2.2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7541,7 +7654,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C57"/>
+  <dimension ref="A1:C58"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8176,6 +8289,17 @@
         <v>2.5453</v>
       </c>
     </row>
+    <row r="58" spans="1:3" ht="16" customHeight="1">
+      <c r="A58" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B58" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C58" s="3">
+        <v>2.8267</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8184,7 +8308,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C57"/>
+  <dimension ref="A1:C58"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8819,6 +8943,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="58" spans="1:3" ht="16" customHeight="1">
+      <c r="A58" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B58" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C58" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-08-05 12:30:40
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1946" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1973" uniqueCount="62">
   <si>
     <t>Date</t>
   </si>
@@ -208,6 +208,9 @@
   </si>
   <si>
     <t>2026-08-04</t>
+  </si>
+  <si>
+    <t>2026-08-05</t>
   </si>
 </sst>
 </file>
@@ -1114,7 +1117,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C58"/>
+  <dimension ref="A1:C59"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1760,6 +1763,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="59" spans="1:3" ht="16" customHeight="1">
+      <c r="A59" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1768,7 +1782,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C58"/>
+  <dimension ref="A1:C59"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2414,6 +2428,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="59" spans="1:3" ht="16" customHeight="1">
+      <c r="A59" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2422,7 +2447,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C58"/>
+  <dimension ref="A1:C59"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3068,6 +3093,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="59" spans="1:3" ht="16" customHeight="1">
+      <c r="A59" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B59" s="3">
+        <v>0.88</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3076,7 +3112,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C58"/>
+  <dimension ref="A1:C59"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3722,6 +3758,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="59" spans="1:3" ht="16" customHeight="1">
+      <c r="A59" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C59" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3730,7 +3777,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C58"/>
+  <dimension ref="A1:C59"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4376,6 +4423,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="59" spans="1:3" ht="16" customHeight="1">
+      <c r="A59" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4384,7 +4442,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C58"/>
+  <dimension ref="A1:C59"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5030,6 +5088,17 @@
         <v>5.875</v>
       </c>
     </row>
+    <row r="59" spans="1:3" ht="16" customHeight="1">
+      <c r="A59" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C59" s="3">
+        <v>5.5625</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5038,7 +5107,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C58"/>
+  <dimension ref="A1:C59"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5684,6 +5753,17 @@
         <v>3.4787</v>
       </c>
     </row>
+    <row r="59" spans="1:3" ht="16" customHeight="1">
+      <c r="A59" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B59" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5692,7 +5772,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C58"/>
+  <dimension ref="A1:C59"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6338,6 +6418,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="59" spans="1:3" ht="16" customHeight="1">
+      <c r="A59" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B59" s="3">
+        <v>4</v>
+      </c>
+      <c r="C59" s="3">
+        <v>4.7355</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6346,7 +6437,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C58"/>
+  <dimension ref="A1:C59"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6992,6 +7083,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="59" spans="1:3" ht="16" customHeight="1">
+      <c r="A59" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7000,7 +7102,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C58"/>
+  <dimension ref="A1:C59"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7646,6 +7748,17 @@
         <v>2.2</v>
       </c>
     </row>
+    <row r="59" spans="1:3" ht="16" customHeight="1">
+      <c r="A59" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B59" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C59" s="3">
+        <v>2.4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7654,7 +7767,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C58"/>
+  <dimension ref="A1:C59"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8300,6 +8413,17 @@
         <v>2.8267</v>
       </c>
     </row>
+    <row r="59" spans="1:3" ht="16" customHeight="1">
+      <c r="A59" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B59" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8308,7 +8432,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C58"/>
+  <dimension ref="A1:C59"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8954,6 +9078,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="59" spans="1:3" ht="16" customHeight="1">
+      <c r="A59" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-08-06 12:48:26
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1973" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1998" uniqueCount="63">
   <si>
     <t>Date</t>
   </si>
@@ -211,6 +211,9 @@
   </si>
   <si>
     <t>2026-08-05</t>
+  </si>
+  <si>
+    <t>2026-08-06</t>
   </si>
 </sst>
 </file>
@@ -1117,7 +1120,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C59"/>
+  <dimension ref="A1:C60"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1774,6 +1777,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="60" spans="1:3" ht="16" customHeight="1">
+      <c r="A60" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B60" s="3">
+        <v>7.5</v>
+      </c>
+      <c r="C60" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1782,7 +1796,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C59"/>
+  <dimension ref="A1:C60"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2439,6 +2453,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="60" spans="1:3" ht="16" customHeight="1">
+      <c r="A60" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B60" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C60" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2447,7 +2472,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C59"/>
+  <dimension ref="A1:C60"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3104,6 +3129,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="60" spans="1:3" ht="16" customHeight="1">
+      <c r="A60" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B60" s="3">
+        <v>0.88</v>
+      </c>
+      <c r="C60" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3112,7 +3148,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C59"/>
+  <dimension ref="A1:C60"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3769,6 +3805,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="60" spans="1:3" ht="16" customHeight="1">
+      <c r="A60" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B60" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C60" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3777,7 +3824,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C59"/>
+  <dimension ref="A1:C60"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4434,6 +4481,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="60" spans="1:3" ht="16" customHeight="1">
+      <c r="A60" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B60" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C60" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4442,7 +4500,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C59"/>
+  <dimension ref="A1:C60"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5099,6 +5157,17 @@
         <v>5.5625</v>
       </c>
     </row>
+    <row r="60" spans="1:3" ht="16" customHeight="1">
+      <c r="A60" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B60" s="3">
+        <v>6.11</v>
+      </c>
+      <c r="C60" s="3">
+        <v>5.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5107,7 +5176,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C59"/>
+  <dimension ref="A1:C60"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5764,6 +5833,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="60" spans="1:3" ht="16" customHeight="1">
+      <c r="A60" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B60" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C60" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5772,7 +5852,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C59"/>
+  <dimension ref="A1:C60"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6429,6 +6509,17 @@
         <v>4.7355</v>
       </c>
     </row>
+    <row r="60" spans="1:3" ht="16" customHeight="1">
+      <c r="A60" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B60" s="3">
+        <v>4</v>
+      </c>
+      <c r="C60" s="3">
+        <v>4.8684</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6437,7 +6528,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C59"/>
+  <dimension ref="A1:C60"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7094,6 +7185,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="60" spans="1:3" ht="16" customHeight="1">
+      <c r="A60" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B60" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C60" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7102,7 +7204,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C59"/>
+  <dimension ref="A1:C60"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7759,6 +7861,17 @@
         <v>2.4</v>
       </c>
     </row>
+    <row r="60" spans="1:3" ht="16" customHeight="1">
+      <c r="A60" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B60" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C60" s="3">
+        <v>2.6267</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7767,7 +7880,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C59"/>
+  <dimension ref="A1:C60"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8424,6 +8537,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="60" spans="1:3" ht="16" customHeight="1">
+      <c r="A60" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B60" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C60" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8432,7 +8556,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C59"/>
+  <dimension ref="A1:C60"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9089,6 +9213,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="60" spans="1:3" ht="16" customHeight="1">
+      <c r="A60" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B60" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C60" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-08-07 11:36:02
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1998" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2024" uniqueCount="64">
   <si>
     <t>Date</t>
   </si>
@@ -214,6 +214,9 @@
   </si>
   <si>
     <t>2026-08-06</t>
+  </si>
+  <si>
+    <t>2026-08-07</t>
   </si>
 </sst>
 </file>
@@ -1120,7 +1123,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C60"/>
+  <dimension ref="A1:C61"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1788,6 +1791,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="61" spans="1:3" ht="16" customHeight="1">
+      <c r="A61" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C61" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1796,7 +1810,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C60"/>
+  <dimension ref="A1:C61"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2464,6 +2478,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="61" spans="1:3" ht="16" customHeight="1">
+      <c r="A61" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C61" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2472,7 +2497,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C60"/>
+  <dimension ref="A1:C61"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3140,6 +3165,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="61" spans="1:3" ht="16" customHeight="1">
+      <c r="A61" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B61" s="3">
+        <v>0.88</v>
+      </c>
+      <c r="C61" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3148,7 +3184,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C60"/>
+  <dimension ref="A1:C61"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3816,6 +3852,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="61" spans="1:3" ht="16" customHeight="1">
+      <c r="A61" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C61" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3824,7 +3871,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C60"/>
+  <dimension ref="A1:C61"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4492,6 +4539,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="61" spans="1:3" ht="16" customHeight="1">
+      <c r="A61" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C61" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4500,7 +4558,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C60"/>
+  <dimension ref="A1:C61"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5168,6 +5226,17 @@
         <v>5.5</v>
       </c>
     </row>
+    <row r="61" spans="1:3" ht="16" customHeight="1">
+      <c r="A61" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B61" s="3">
+        <v>6.11</v>
+      </c>
+      <c r="C61" s="3">
+        <v>5.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5176,7 +5245,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C60"/>
+  <dimension ref="A1:C61"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5844,6 +5913,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="61" spans="1:3" ht="16" customHeight="1">
+      <c r="A61" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B61" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C61" s="3">
+        <v>4.2187</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5852,7 +5932,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C60"/>
+  <dimension ref="A1:C61"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6520,6 +6600,17 @@
         <v>4.8684</v>
       </c>
     </row>
+    <row r="61" spans="1:3" ht="16" customHeight="1">
+      <c r="A61" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B61" s="3">
+        <v>4</v>
+      </c>
+      <c r="C61" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6528,7 +6619,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C60"/>
+  <dimension ref="A1:C61"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7196,6 +7287,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="61" spans="1:3" ht="16" customHeight="1">
+      <c r="A61" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B61" s="3">
+        <v>1.99</v>
+      </c>
+      <c r="C61" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7204,7 +7306,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C60"/>
+  <dimension ref="A1:C61"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7872,6 +7974,17 @@
         <v>2.6267</v>
       </c>
     </row>
+    <row r="61" spans="1:3" ht="16" customHeight="1">
+      <c r="A61" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B61" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C61" s="3">
+        <v>2.4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7880,7 +7993,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C60"/>
+  <dimension ref="A1:C61"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8548,6 +8661,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="61" spans="1:3" ht="16" customHeight="1">
+      <c r="A61" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C61" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8556,7 +8680,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C60"/>
+  <dimension ref="A1:C61"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9224,6 +9348,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="61" spans="1:3" ht="16" customHeight="1">
+      <c r="A61" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C61" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-08-08 11:17:54
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2024" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2049" uniqueCount="65">
   <si>
     <t>Date</t>
   </si>
@@ -217,6 +217,9 @@
   </si>
   <si>
     <t>2026-08-07</t>
+  </si>
+  <si>
+    <t>2026-08-08</t>
   </si>
 </sst>
 </file>
@@ -1123,7 +1126,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C61"/>
+  <dimension ref="A1:C62"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1802,6 +1805,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="62" spans="1:3" ht="16" customHeight="1">
+      <c r="A62" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B62" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C62" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1810,7 +1824,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C61"/>
+  <dimension ref="A1:C62"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2489,6 +2503,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="62" spans="1:3" ht="16" customHeight="1">
+      <c r="A62" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B62" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C62" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2497,7 +2522,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C61"/>
+  <dimension ref="A1:C62"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3176,6 +3201,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="62" spans="1:3" ht="16" customHeight="1">
+      <c r="A62" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B62" s="3">
+        <v>0.88</v>
+      </c>
+      <c r="C62" s="3">
+        <v>0.8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3184,7 +3220,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C61"/>
+  <dimension ref="A1:C62"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3863,6 +3899,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="62" spans="1:3" ht="16" customHeight="1">
+      <c r="A62" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B62" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C62" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3871,7 +3918,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C61"/>
+  <dimension ref="A1:C62"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4550,6 +4597,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="62" spans="1:3" ht="16" customHeight="1">
+      <c r="A62" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B62" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C62" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4558,7 +4616,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C61"/>
+  <dimension ref="A1:C62"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5237,6 +5295,17 @@
         <v>5.5</v>
       </c>
     </row>
+    <row r="62" spans="1:3" ht="16" customHeight="1">
+      <c r="A62" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B62" s="3">
+        <v>6.11</v>
+      </c>
+      <c r="C62" s="3">
+        <v>5.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5245,7 +5314,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C61"/>
+  <dimension ref="A1:C62"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5924,6 +5993,17 @@
         <v>4.2187</v>
       </c>
     </row>
+    <row r="62" spans="1:3" ht="16" customHeight="1">
+      <c r="A62" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B62" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C62" s="3">
+        <v>3.8134</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5932,7 +6012,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C61"/>
+  <dimension ref="A1:C62"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6611,6 +6691,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="62" spans="1:3" ht="16" customHeight="1">
+      <c r="A62" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B62" s="3">
+        <v>4</v>
+      </c>
+      <c r="C62" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6619,7 +6710,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C61"/>
+  <dimension ref="A1:C62"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7298,6 +7389,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="62" spans="1:3" ht="16" customHeight="1">
+      <c r="A62" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B62" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C62" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7306,7 +7408,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C61"/>
+  <dimension ref="A1:C62"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7985,6 +8087,17 @@
         <v>2.4</v>
       </c>
     </row>
+    <row r="62" spans="1:3" ht="16" customHeight="1">
+      <c r="A62" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B62" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C62" s="3">
+        <v>2.2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7993,7 +8106,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C61"/>
+  <dimension ref="A1:C62"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8672,6 +8785,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="62" spans="1:3" ht="16" customHeight="1">
+      <c r="A62" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B62" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C62" s="3">
+        <v>2.7867</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8680,7 +8804,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C61"/>
+  <dimension ref="A1:C62"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9359,6 +9483,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="62" spans="1:3" ht="16" customHeight="1">
+      <c r="A62" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B62" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C62" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-08-09 11:18:34
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2049" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2074" uniqueCount="66">
   <si>
     <t>Date</t>
   </si>
@@ -220,6 +220,9 @@
   </si>
   <si>
     <t>2026-08-08</t>
+  </si>
+  <si>
+    <t>2026-08-09</t>
   </si>
 </sst>
 </file>
@@ -1126,7 +1129,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C62"/>
+  <dimension ref="A1:C63"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1816,6 +1819,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="63" spans="1:3" ht="16" customHeight="1">
+      <c r="A63" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C63" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1824,7 +1838,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C62"/>
+  <dimension ref="A1:C63"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2514,6 +2528,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="63" spans="1:3" ht="16" customHeight="1">
+      <c r="A63" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C63" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2522,7 +2547,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C62"/>
+  <dimension ref="A1:C63"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3212,6 +3237,17 @@
         <v>0.8</v>
       </c>
     </row>
+    <row r="63" spans="1:3" ht="16" customHeight="1">
+      <c r="A63" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B63" s="3">
+        <v>0.88</v>
+      </c>
+      <c r="C63" s="3">
+        <v>0.8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3220,7 +3256,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C62"/>
+  <dimension ref="A1:C63"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3910,6 +3946,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="63" spans="1:3" ht="16" customHeight="1">
+      <c r="A63" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C63" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3918,7 +3965,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C62"/>
+  <dimension ref="A1:C63"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4608,6 +4655,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="63" spans="1:3" ht="16" customHeight="1">
+      <c r="A63" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C63" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4616,7 +4674,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C62"/>
+  <dimension ref="A1:C63"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5306,6 +5364,17 @@
         <v>5.5</v>
       </c>
     </row>
+    <row r="63" spans="1:3" ht="16" customHeight="1">
+      <c r="A63" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C63" s="3">
+        <v>5.5625</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5314,7 +5383,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C62"/>
+  <dimension ref="A1:C63"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6004,6 +6073,17 @@
         <v>3.8134</v>
       </c>
     </row>
+    <row r="63" spans="1:3" ht="16" customHeight="1">
+      <c r="A63" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B63" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C63" s="3">
+        <v>3.976</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6012,7 +6092,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C62"/>
+  <dimension ref="A1:C63"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6702,6 +6782,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="63" spans="1:3" ht="16" customHeight="1">
+      <c r="A63" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B63" s="3">
+        <v>4</v>
+      </c>
+      <c r="C63" s="3">
+        <v>4.3408</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6710,7 +6801,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C62"/>
+  <dimension ref="A1:C63"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7400,6 +7491,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="63" spans="1:3" ht="16" customHeight="1">
+      <c r="A63" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C63" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7408,7 +7510,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C62"/>
+  <dimension ref="A1:C63"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8098,6 +8200,17 @@
         <v>2.2</v>
       </c>
     </row>
+    <row r="63" spans="1:3" ht="16" customHeight="1">
+      <c r="A63" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B63" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C63" s="3">
+        <v>2.2667</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8106,7 +8219,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C62"/>
+  <dimension ref="A1:C63"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8796,6 +8909,17 @@
         <v>2.7867</v>
       </c>
     </row>
+    <row r="63" spans="1:3" ht="16" customHeight="1">
+      <c r="A63" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C63" s="3">
+        <v>2.6667</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8804,7 +8928,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C62"/>
+  <dimension ref="A1:C63"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9494,6 +9618,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="63" spans="1:3" ht="16" customHeight="1">
+      <c r="A63" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C63" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-08-10 11:39:22
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2074" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2102" uniqueCount="67">
   <si>
     <t>Date</t>
   </si>
@@ -223,6 +223,9 @@
   </si>
   <si>
     <t>2026-08-09</t>
+  </si>
+  <si>
+    <t>2026-08-10</t>
   </si>
 </sst>
 </file>
@@ -1129,7 +1132,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C63"/>
+  <dimension ref="A1:C64"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1830,6 +1833,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="64" spans="1:3" ht="16" customHeight="1">
+      <c r="A64" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B64" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C64" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1838,7 +1852,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C63"/>
+  <dimension ref="A1:C64"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2539,6 +2553,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="64" spans="1:3" ht="16" customHeight="1">
+      <c r="A64" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B64" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C64" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2547,7 +2572,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C63"/>
+  <dimension ref="A1:C64"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3248,6 +3273,17 @@
         <v>0.8</v>
       </c>
     </row>
+    <row r="64" spans="1:3" ht="16" customHeight="1">
+      <c r="A64" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B64" s="3">
+        <v>0.88</v>
+      </c>
+      <c r="C64" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3256,7 +3292,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C63"/>
+  <dimension ref="A1:C64"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3957,6 +3993,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="64" spans="1:3" ht="16" customHeight="1">
+      <c r="A64" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B64" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C64" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3965,7 +4012,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C63"/>
+  <dimension ref="A1:C64"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4666,6 +4713,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="64" spans="1:3" ht="16" customHeight="1">
+      <c r="A64" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B64" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C64" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4674,7 +4732,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C63"/>
+  <dimension ref="A1:C64"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5375,6 +5433,17 @@
         <v>5.5625</v>
       </c>
     </row>
+    <row r="64" spans="1:3" ht="16" customHeight="1">
+      <c r="A64" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B64" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C64" s="3">
+        <v>5.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5383,7 +5452,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C63"/>
+  <dimension ref="A1:C64"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6084,6 +6153,17 @@
         <v>3.976</v>
       </c>
     </row>
+    <row r="64" spans="1:3" ht="16" customHeight="1">
+      <c r="A64" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B64" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C64" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6092,7 +6172,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C63"/>
+  <dimension ref="A1:C64"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6793,6 +6873,17 @@
         <v>4.3408</v>
       </c>
     </row>
+    <row r="64" spans="1:3" ht="16" customHeight="1">
+      <c r="A64" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B64" s="3">
+        <v>3.99</v>
+      </c>
+      <c r="C64" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6801,7 +6892,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C63"/>
+  <dimension ref="A1:C64"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7502,6 +7593,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="64" spans="1:3" ht="16" customHeight="1">
+      <c r="A64" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B64" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C64" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7510,7 +7612,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C63"/>
+  <dimension ref="A1:C64"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8211,6 +8313,17 @@
         <v>2.2667</v>
       </c>
     </row>
+    <row r="64" spans="1:3" ht="16" customHeight="1">
+      <c r="A64" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B64" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C64" s="3">
+        <v>2.1867</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8219,7 +8332,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C63"/>
+  <dimension ref="A1:C64"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8920,6 +9033,17 @@
         <v>2.6667</v>
       </c>
     </row>
+    <row r="64" spans="1:3" ht="16" customHeight="1">
+      <c r="A64" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B64" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C64" s="3">
+        <v>2.1333</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8928,7 +9052,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C63"/>
+  <dimension ref="A1:C64"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9629,6 +9753,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="64" spans="1:3" ht="16" customHeight="1">
+      <c r="A64" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B64" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C64" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-08-11 11:35:25
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2102" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2130" uniqueCount="68">
   <si>
     <t>Date</t>
   </si>
@@ -226,6 +226,9 @@
   </si>
   <si>
     <t>2026-08-10</t>
+  </si>
+  <si>
+    <t>2026-08-11</t>
   </si>
 </sst>
 </file>
@@ -1132,7 +1135,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C64"/>
+  <dimension ref="A1:C65"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1844,6 +1847,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="65" spans="1:3" ht="16" customHeight="1">
+      <c r="A65" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B65" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C65" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1852,7 +1866,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C64"/>
+  <dimension ref="A1:C65"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2564,6 +2578,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="65" spans="1:3" ht="16" customHeight="1">
+      <c r="A65" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B65" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C65" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2572,7 +2597,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C64"/>
+  <dimension ref="A1:C65"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3284,6 +3309,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="65" spans="1:3" ht="16" customHeight="1">
+      <c r="A65" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B65" s="3">
+        <v>0.88</v>
+      </c>
+      <c r="C65" s="3">
+        <v>0.8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3292,7 +3328,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C64"/>
+  <dimension ref="A1:C65"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4004,6 +4040,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="65" spans="1:3" ht="16" customHeight="1">
+      <c r="A65" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B65" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C65" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4012,7 +4059,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C64"/>
+  <dimension ref="A1:C65"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4724,6 +4771,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="65" spans="1:3" ht="16" customHeight="1">
+      <c r="A65" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B65" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C65" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4732,7 +4790,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C64"/>
+  <dimension ref="A1:C65"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5444,6 +5502,17 @@
         <v>5.5</v>
       </c>
     </row>
+    <row r="65" spans="1:3" ht="16" customHeight="1">
+      <c r="A65" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B65" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C65" s="3">
+        <v>5.5625</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5452,7 +5521,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C64"/>
+  <dimension ref="A1:C65"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6164,6 +6233,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="65" spans="1:3" ht="16" customHeight="1">
+      <c r="A65" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B65" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C65" s="3">
+        <v>4.444</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6172,7 +6252,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C64"/>
+  <dimension ref="A1:C65"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6884,6 +6964,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="65" spans="1:3" ht="16" customHeight="1">
+      <c r="A65" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B65" s="3">
+        <v>3.99</v>
+      </c>
+      <c r="C65" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6892,7 +6983,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C64"/>
+  <dimension ref="A1:C65"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7604,6 +7695,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="65" spans="1:3" ht="16" customHeight="1">
+      <c r="A65" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B65" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C65" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7612,7 +7714,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C64"/>
+  <dimension ref="A1:C65"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8324,6 +8426,17 @@
         <v>2.1867</v>
       </c>
     </row>
+    <row r="65" spans="1:3" ht="16" customHeight="1">
+      <c r="A65" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B65" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C65" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8332,7 +8445,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C64"/>
+  <dimension ref="A1:C65"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9044,6 +9157,17 @@
         <v>2.1333</v>
       </c>
     </row>
+    <row r="65" spans="1:3" ht="16" customHeight="1">
+      <c r="A65" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B65" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C65" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9052,7 +9176,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C64"/>
+  <dimension ref="A1:C65"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9764,6 +9888,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="65" spans="1:3" ht="16" customHeight="1">
+      <c r="A65" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B65" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C65" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-08-12 11:36:41
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2130" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2154" uniqueCount="69">
   <si>
     <t>Date</t>
   </si>
@@ -230,6 +230,9 @@
   <si>
     <t>2026-08-11</t>
   </si>
+  <si>
+    <t>2026-08-12</t>
+  </si>
 </sst>
 </file>
 
@@ -345,7 +348,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -365,7 +368,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -388,7 +391,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -408,7 +411,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -431,7 +434,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -451,7 +454,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -474,7 +477,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -494,7 +497,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -560,7 +563,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -580,7 +583,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -603,7 +606,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -623,7 +626,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -646,7 +649,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -666,7 +669,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -689,7 +692,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -709,7 +712,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -732,7 +735,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -752,7 +755,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -775,7 +778,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -795,7 +798,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1135,7 +1138,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C65"/>
+  <dimension ref="A1:C66"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1858,6 +1861,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="66" spans="1:3" ht="16" customHeight="1">
+      <c r="A66" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B66" s="3">
+        <v>7.5</v>
+      </c>
+      <c r="C66" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1866,7 +1880,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C65"/>
+  <dimension ref="A1:C66"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2589,6 +2603,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="66" spans="1:3" ht="16" customHeight="1">
+      <c r="A66" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B66" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C66" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2597,7 +2622,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C65"/>
+  <dimension ref="A1:C66"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3320,6 +3345,17 @@
         <v>0.8</v>
       </c>
     </row>
+    <row r="66" spans="1:3" ht="16" customHeight="1">
+      <c r="A66" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B66" s="3">
+        <v>0.88</v>
+      </c>
+      <c r="C66" s="3">
+        <v>0.8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3328,7 +3364,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C65"/>
+  <dimension ref="A1:C66"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4051,6 +4087,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="66" spans="1:3" ht="16" customHeight="1">
+      <c r="A66" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B66" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C66" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4059,7 +4106,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C65"/>
+  <dimension ref="A1:C66"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4782,6 +4829,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="66" spans="1:3" ht="16" customHeight="1">
+      <c r="A66" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B66" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C66" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4790,7 +4848,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C65"/>
+  <dimension ref="A1:C66"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5513,6 +5571,17 @@
         <v>5.5625</v>
       </c>
     </row>
+    <row r="66" spans="1:3" ht="16" customHeight="1">
+      <c r="A66" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B66" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C66" s="3">
+        <v>5.575</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5521,7 +5590,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C65"/>
+  <dimension ref="A1:C66"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6244,6 +6313,17 @@
         <v>4.444</v>
       </c>
     </row>
+    <row r="66" spans="1:3" ht="16" customHeight="1">
+      <c r="A66" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B66" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C66" s="3">
+        <v>4.6453</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6252,7 +6332,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C65"/>
+  <dimension ref="A1:C66"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6975,6 +7055,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="66" spans="1:3" ht="16" customHeight="1">
+      <c r="A66" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B66" s="3">
+        <v>3.99</v>
+      </c>
+      <c r="C66" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6983,7 +7074,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C65"/>
+  <dimension ref="A1:C66"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7706,6 +7797,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="66" spans="1:3" ht="16" customHeight="1">
+      <c r="A66" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B66" s="3">
+        <v>2.29</v>
+      </c>
+      <c r="C66" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7714,7 +7816,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C65"/>
+  <dimension ref="A1:C66"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8437,6 +8539,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="66" spans="1:3" ht="16" customHeight="1">
+      <c r="A66" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B66" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C66" s="3">
+        <v>2.2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8445,7 +8558,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C65"/>
+  <dimension ref="A1:C66"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9168,6 +9281,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="66" spans="1:3" ht="16" customHeight="1">
+      <c r="A66" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B66" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C66" s="3">
+        <v>2.3827</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9176,7 +9300,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C65"/>
+  <dimension ref="A1:C66"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9899,6 +10023,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="66" spans="1:3" ht="16" customHeight="1">
+      <c r="A66" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B66" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C66" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-08-13 11:36:47
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2154" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2180" uniqueCount="70">
   <si>
     <t>Date</t>
   </si>
@@ -233,6 +233,9 @@
   <si>
     <t>2026-08-12</t>
   </si>
+  <si>
+    <t>2026-08-13</t>
+  </si>
 </sst>
 </file>
 
@@ -348,7 +351,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -368,7 +371,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -391,7 +394,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -411,7 +414,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -434,7 +437,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -454,7 +457,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -477,7 +480,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -497,7 +500,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -563,7 +566,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -583,7 +586,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -606,7 +609,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -626,7 +629,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -649,7 +652,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -669,7 +672,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -692,7 +695,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -712,7 +715,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -735,7 +738,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -755,7 +758,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -778,7 +781,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -798,7 +801,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1138,7 +1141,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C66"/>
+  <dimension ref="A1:C67"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1872,6 +1875,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="67" spans="1:3" ht="16" customHeight="1">
+      <c r="A67" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B67" s="3">
+        <v>7.5</v>
+      </c>
+      <c r="C67" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1880,7 +1894,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C66"/>
+  <dimension ref="A1:C67"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2614,6 +2628,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="67" spans="1:3" ht="16" customHeight="1">
+      <c r="A67" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B67" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C67" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2622,7 +2647,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C66"/>
+  <dimension ref="A1:C67"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3356,6 +3381,17 @@
         <v>0.8</v>
       </c>
     </row>
+    <row r="67" spans="1:3" ht="16" customHeight="1">
+      <c r="A67" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B67" s="3">
+        <v>0.88</v>
+      </c>
+      <c r="C67" s="3">
+        <v>0.8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3364,7 +3400,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C66"/>
+  <dimension ref="A1:C67"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4098,6 +4134,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="67" spans="1:3" ht="16" customHeight="1">
+      <c r="A67" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B67" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C67" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4106,7 +4153,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C66"/>
+  <dimension ref="A1:C67"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4840,6 +4887,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="67" spans="1:3" ht="16" customHeight="1">
+      <c r="A67" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B67" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C67" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4848,7 +4906,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C66"/>
+  <dimension ref="A1:C67"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5582,6 +5640,17 @@
         <v>5.575</v>
       </c>
     </row>
+    <row r="67" spans="1:3" ht="16" customHeight="1">
+      <c r="A67" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B67" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C67" s="3">
+        <v>6.125</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5590,7 +5659,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C66"/>
+  <dimension ref="A1:C67"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6324,6 +6393,17 @@
         <v>4.6453</v>
       </c>
     </row>
+    <row r="67" spans="1:3" ht="16" customHeight="1">
+      <c r="A67" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B67" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C67" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6332,7 +6412,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C66"/>
+  <dimension ref="A1:C67"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7066,6 +7146,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="67" spans="1:3" ht="16" customHeight="1">
+      <c r="A67" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B67" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C67" s="3">
+        <v>4.1421</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7074,7 +7165,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C66"/>
+  <dimension ref="A1:C67"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7808,6 +7899,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="67" spans="1:3" ht="16" customHeight="1">
+      <c r="A67" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B67" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C67" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7816,7 +7918,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C66"/>
+  <dimension ref="A1:C67"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8550,6 +8652,17 @@
         <v>2.2</v>
       </c>
     </row>
+    <row r="67" spans="1:3" ht="16" customHeight="1">
+      <c r="A67" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B67" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C67" s="3">
+        <v>2.5853</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8558,7 +8671,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C66"/>
+  <dimension ref="A1:C67"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9292,6 +9405,17 @@
         <v>2.3827</v>
       </c>
     </row>
+    <row r="67" spans="1:3" ht="16" customHeight="1">
+      <c r="A67" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B67" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C67" s="3">
+        <v>2.5453</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9300,7 +9424,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C66"/>
+  <dimension ref="A1:C67"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10034,6 +10158,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="67" spans="1:3" ht="16" customHeight="1">
+      <c r="A67" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B67" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C67" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-08-14 11:34:31
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2180" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2205" uniqueCount="71">
   <si>
     <t>Date</t>
   </si>
@@ -235,6 +235,9 @@
   </si>
   <si>
     <t>2026-08-13</t>
+  </si>
+  <si>
+    <t>2026-08-14</t>
   </si>
 </sst>
 </file>
@@ -1141,7 +1144,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C67"/>
+  <dimension ref="A1:C68"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1886,6 +1889,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="68" spans="1:3" ht="16" customHeight="1">
+      <c r="A68" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B68" s="3">
+        <v>7.5</v>
+      </c>
+      <c r="C68" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1894,7 +1908,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C67"/>
+  <dimension ref="A1:C68"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2639,6 +2653,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="68" spans="1:3" ht="16" customHeight="1">
+      <c r="A68" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B68" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C68" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2647,7 +2672,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C67"/>
+  <dimension ref="A1:C68"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3392,6 +3417,17 @@
         <v>0.8</v>
       </c>
     </row>
+    <row r="68" spans="1:3" ht="16" customHeight="1">
+      <c r="A68" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B68" s="3">
+        <v>0.88</v>
+      </c>
+      <c r="C68" s="3">
+        <v>0.8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3400,7 +3436,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C67"/>
+  <dimension ref="A1:C68"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4145,6 +4181,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="68" spans="1:3" ht="16" customHeight="1">
+      <c r="A68" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B68" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C68" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4153,7 +4200,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C67"/>
+  <dimension ref="A1:C68"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4898,6 +4945,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="68" spans="1:3" ht="16" customHeight="1">
+      <c r="A68" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B68" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C68" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4906,7 +4964,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C67"/>
+  <dimension ref="A1:C68"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5651,6 +5709,17 @@
         <v>6.125</v>
       </c>
     </row>
+    <row r="68" spans="1:3" ht="16" customHeight="1">
+      <c r="A68" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B68" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C68" s="3">
+        <v>6.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5659,7 +5728,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C67"/>
+  <dimension ref="A1:C68"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6404,6 +6473,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="68" spans="1:3" ht="16" customHeight="1">
+      <c r="A68" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B68" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C68" s="3">
+        <v>3.0307</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6412,7 +6492,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C67"/>
+  <dimension ref="A1:C68"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7157,6 +7237,17 @@
         <v>4.1421</v>
       </c>
     </row>
+    <row r="68" spans="1:3" ht="16" customHeight="1">
+      <c r="A68" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B68" s="3">
+        <v>3.99</v>
+      </c>
+      <c r="C68" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7165,7 +7256,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C67"/>
+  <dimension ref="A1:C68"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7910,6 +8001,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="68" spans="1:3" ht="16" customHeight="1">
+      <c r="A68" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B68" s="3">
+        <v>2.29</v>
+      </c>
+      <c r="C68" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7918,7 +8020,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C67"/>
+  <dimension ref="A1:C68"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8663,6 +8765,17 @@
         <v>2.5853</v>
       </c>
     </row>
+    <row r="68" spans="1:3" ht="16" customHeight="1">
+      <c r="A68" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B68" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C68" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8671,7 +8784,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C67"/>
+  <dimension ref="A1:C68"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9416,6 +9529,17 @@
         <v>2.5453</v>
       </c>
     </row>
+    <row r="68" spans="1:3" ht="16" customHeight="1">
+      <c r="A68" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B68" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C68" s="3">
+        <v>2.5453</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9424,7 +9548,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C67"/>
+  <dimension ref="A1:C68"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10169,6 +10293,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="68" spans="1:3" ht="16" customHeight="1">
+      <c r="A68" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B68" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C68" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-08-15 11:08:11
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2205" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2232" uniqueCount="72">
   <si>
     <t>Date</t>
   </si>
@@ -238,6 +238,9 @@
   </si>
   <si>
     <t>2026-08-14</t>
+  </si>
+  <si>
+    <t>2026-08-15</t>
   </si>
 </sst>
 </file>
@@ -1144,7 +1147,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C68"/>
+  <dimension ref="A1:C69"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1900,6 +1903,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="69" spans="1:3" ht="16" customHeight="1">
+      <c r="A69" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B69" s="3">
+        <v>7.5</v>
+      </c>
+      <c r="C69" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1908,7 +1922,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C68"/>
+  <dimension ref="A1:C69"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2664,6 +2678,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="69" spans="1:3" ht="16" customHeight="1">
+      <c r="A69" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B69" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C69" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2672,7 +2697,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C68"/>
+  <dimension ref="A1:C69"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3428,6 +3453,17 @@
         <v>0.8</v>
       </c>
     </row>
+    <row r="69" spans="1:3" ht="16" customHeight="1">
+      <c r="A69" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B69" s="3">
+        <v>0.88</v>
+      </c>
+      <c r="C69" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3436,7 +3472,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C68"/>
+  <dimension ref="A1:C69"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4192,6 +4228,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="69" spans="1:3" ht="16" customHeight="1">
+      <c r="A69" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B69" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C69" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4200,7 +4247,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C68"/>
+  <dimension ref="A1:C69"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4956,6 +5003,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="69" spans="1:3" ht="16" customHeight="1">
+      <c r="A69" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B69" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C69" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4964,7 +5022,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C68"/>
+  <dimension ref="A1:C69"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5720,6 +5778,17 @@
         <v>6.5</v>
       </c>
     </row>
+    <row r="69" spans="1:3" ht="16" customHeight="1">
+      <c r="A69" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B69" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C69" s="3">
+        <v>6.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5728,7 +5797,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C68"/>
+  <dimension ref="A1:C69"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6484,6 +6553,17 @@
         <v>3.0307</v>
       </c>
     </row>
+    <row r="69" spans="1:3" ht="16" customHeight="1">
+      <c r="A69" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B69" s="3">
+        <v>4.47</v>
+      </c>
+      <c r="C69" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6492,7 +6572,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C68"/>
+  <dimension ref="A1:C69"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7248,6 +7328,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="69" spans="1:3" ht="16" customHeight="1">
+      <c r="A69" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B69" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C69" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7256,7 +7347,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C68"/>
+  <dimension ref="A1:C69"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8012,6 +8103,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="69" spans="1:3" ht="16" customHeight="1">
+      <c r="A69" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B69" s="3">
+        <v>2.29</v>
+      </c>
+      <c r="C69" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8020,7 +8122,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C68"/>
+  <dimension ref="A1:C69"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8776,6 +8878,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="69" spans="1:3" ht="16" customHeight="1">
+      <c r="A69" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B69" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C69" s="3">
+        <v>2.4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8784,7 +8897,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C68"/>
+  <dimension ref="A1:C69"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9540,6 +9653,17 @@
         <v>2.5453</v>
       </c>
     </row>
+    <row r="69" spans="1:3" ht="16" customHeight="1">
+      <c r="A69" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B69" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C69" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9548,7 +9672,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C68"/>
+  <dimension ref="A1:C69"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10304,6 +10428,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="69" spans="1:3" ht="16" customHeight="1">
+      <c r="A69" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B69" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C69" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-08-16 11:09:08
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2232" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2258" uniqueCount="73">
   <si>
     <t>Date</t>
   </si>
@@ -241,6 +241,9 @@
   </si>
   <si>
     <t>2026-08-15</t>
+  </si>
+  <si>
+    <t>2026-08-16</t>
   </si>
 </sst>
 </file>
@@ -1147,7 +1150,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C69"/>
+  <dimension ref="A1:C70"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1914,6 +1917,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="70" spans="1:3" ht="16" customHeight="1">
+      <c r="A70" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B70" s="3">
+        <v>7.5</v>
+      </c>
+      <c r="C70" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1922,7 +1936,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C69"/>
+  <dimension ref="A1:C70"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2689,6 +2703,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="70" spans="1:3" ht="16" customHeight="1">
+      <c r="A70" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B70" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C70" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2697,7 +2722,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C69"/>
+  <dimension ref="A1:C70"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3464,6 +3489,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="70" spans="1:3" ht="16" customHeight="1">
+      <c r="A70" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B70" s="3">
+        <v>0.88</v>
+      </c>
+      <c r="C70" s="3">
+        <v>0.8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3472,7 +3508,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C69"/>
+  <dimension ref="A1:C70"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4239,6 +4275,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="70" spans="1:3" ht="16" customHeight="1">
+      <c r="A70" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B70" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C70" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4247,7 +4294,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C69"/>
+  <dimension ref="A1:C70"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5014,6 +5061,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="70" spans="1:3" ht="16" customHeight="1">
+      <c r="A70" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B70" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C70" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5022,7 +5080,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C69"/>
+  <dimension ref="A1:C70"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5789,6 +5847,17 @@
         <v>6.5</v>
       </c>
     </row>
+    <row r="70" spans="1:3" ht="16" customHeight="1">
+      <c r="A70" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B70" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C70" s="3">
+        <v>6.25</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5797,7 +5866,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C69"/>
+  <dimension ref="A1:C70"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6564,6 +6633,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="70" spans="1:3" ht="16" customHeight="1">
+      <c r="A70" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B70" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C70" s="3">
+        <v>4.764</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6572,7 +6652,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C69"/>
+  <dimension ref="A1:C70"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7339,6 +7419,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="70" spans="1:3" ht="16" customHeight="1">
+      <c r="A70" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B70" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C70" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7347,7 +7438,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C69"/>
+  <dimension ref="A1:C70"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8114,6 +8205,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="70" spans="1:3" ht="16" customHeight="1">
+      <c r="A70" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B70" s="3">
+        <v>2.29</v>
+      </c>
+      <c r="C70" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8122,7 +8224,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C69"/>
+  <dimension ref="A1:C70"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8889,6 +8991,17 @@
         <v>2.4</v>
       </c>
     </row>
+    <row r="70" spans="1:3" ht="16" customHeight="1">
+      <c r="A70" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B70" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C70" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8897,7 +9010,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C69"/>
+  <dimension ref="A1:C70"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9664,6 +9777,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="70" spans="1:3" ht="16" customHeight="1">
+      <c r="A70" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B70" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C70" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9672,7 +9796,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C69"/>
+  <dimension ref="A1:C70"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10439,6 +10563,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="70" spans="1:3" ht="16" customHeight="1">
+      <c r="A70" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B70" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C70" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-08-17 11:14:12
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2258" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2282" uniqueCount="74">
   <si>
     <t>Date</t>
   </si>
@@ -244,6 +244,9 @@
   </si>
   <si>
     <t>2026-08-16</t>
+  </si>
+  <si>
+    <t>2026-08-17</t>
   </si>
 </sst>
 </file>
@@ -1150,7 +1153,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C70"/>
+  <dimension ref="A1:C71"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1928,6 +1931,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="71" spans="1:3" ht="16" customHeight="1">
+      <c r="A71" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B71" s="3">
+        <v>7.5</v>
+      </c>
+      <c r="C71" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1936,7 +1950,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C70"/>
+  <dimension ref="A1:C71"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2714,6 +2728,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="71" spans="1:3" ht="16" customHeight="1">
+      <c r="A71" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B71" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C71" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2722,7 +2747,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C70"/>
+  <dimension ref="A1:C71"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3500,6 +3525,17 @@
         <v>0.8</v>
       </c>
     </row>
+    <row r="71" spans="1:3" ht="16" customHeight="1">
+      <c r="A71" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B71" s="3">
+        <v>0.88</v>
+      </c>
+      <c r="C71" s="3">
+        <v>0.8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3508,7 +3544,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C70"/>
+  <dimension ref="A1:C71"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4286,6 +4322,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="71" spans="1:3" ht="16" customHeight="1">
+      <c r="A71" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B71" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C71" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4294,7 +4341,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C70"/>
+  <dimension ref="A1:C71"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5072,6 +5119,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="71" spans="1:3" ht="16" customHeight="1">
+      <c r="A71" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B71" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C71" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5080,7 +5138,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C70"/>
+  <dimension ref="A1:C71"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5858,6 +5916,17 @@
         <v>6.25</v>
       </c>
     </row>
+    <row r="71" spans="1:3" ht="16" customHeight="1">
+      <c r="A71" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B71" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C71" s="3">
+        <v>6.875</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5866,7 +5935,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C70"/>
+  <dimension ref="A1:C71"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6644,6 +6713,17 @@
         <v>4.764</v>
       </c>
     </row>
+    <row r="71" spans="1:3" ht="16" customHeight="1">
+      <c r="A71" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B71" s="3">
+        <v>4.47</v>
+      </c>
+      <c r="C71" s="3">
+        <v>3.588</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6652,7 +6732,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C70"/>
+  <dimension ref="A1:C71"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7430,6 +7510,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="71" spans="1:3" ht="16" customHeight="1">
+      <c r="A71" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B71" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C71" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7438,7 +7529,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C70"/>
+  <dimension ref="A1:C71"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8216,6 +8307,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="71" spans="1:3" ht="16" customHeight="1">
+      <c r="A71" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B71" s="3">
+        <v>2.29</v>
+      </c>
+      <c r="C71" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8224,7 +8326,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C70"/>
+  <dimension ref="A1:C71"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9002,6 +9104,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="71" spans="1:3" ht="16" customHeight="1">
+      <c r="A71" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B71" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C71" s="3">
+        <v>4.6667</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9010,7 +9123,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C70"/>
+  <dimension ref="A1:C71"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9788,6 +9901,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="71" spans="1:3" ht="16" customHeight="1">
+      <c r="A71" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B71" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C71" s="3">
+        <v>3.0667</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9796,7 +9920,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C70"/>
+  <dimension ref="A1:C71"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10574,6 +10698,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="71" spans="1:3" ht="16" customHeight="1">
+      <c r="A71" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B71" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C71" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-08-18 11:14:06
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2282" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2309" uniqueCount="75">
   <si>
     <t>Date</t>
   </si>
@@ -247,6 +247,9 @@
   </si>
   <si>
     <t>2026-08-17</t>
+  </si>
+  <si>
+    <t>2026-08-18</t>
   </si>
 </sst>
 </file>
@@ -1153,7 +1156,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C71"/>
+  <dimension ref="A1:C72"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1942,6 +1945,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="72" spans="1:3" ht="16" customHeight="1">
+      <c r="A72" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B72" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C72" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1950,7 +1964,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C71"/>
+  <dimension ref="A1:C72"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2739,6 +2753,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="72" spans="1:3" ht="16" customHeight="1">
+      <c r="A72" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B72" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C72" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2747,7 +2772,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C71"/>
+  <dimension ref="A1:C72"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3536,6 +3561,17 @@
         <v>0.8</v>
       </c>
     </row>
+    <row r="72" spans="1:3" ht="16" customHeight="1">
+      <c r="A72" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B72" s="3">
+        <v>0.88</v>
+      </c>
+      <c r="C72" s="3">
+        <v>0.8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3544,7 +3580,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C71"/>
+  <dimension ref="A1:C72"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4333,6 +4369,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="72" spans="1:3" ht="16" customHeight="1">
+      <c r="A72" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B72" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C72" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4341,7 +4388,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C71"/>
+  <dimension ref="A1:C72"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5130,6 +5177,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="72" spans="1:3" ht="16" customHeight="1">
+      <c r="A72" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B72" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C72" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5138,7 +5196,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C71"/>
+  <dimension ref="A1:C72"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5927,6 +5985,17 @@
         <v>6.875</v>
       </c>
     </row>
+    <row r="72" spans="1:3" ht="16" customHeight="1">
+      <c r="A72" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B72" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C72" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5935,7 +6004,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C71"/>
+  <dimension ref="A1:C72"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6724,6 +6793,17 @@
         <v>3.588</v>
       </c>
     </row>
+    <row r="72" spans="1:3" ht="16" customHeight="1">
+      <c r="A72" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B72" s="3">
+        <v>4.47</v>
+      </c>
+      <c r="C72" s="3">
+        <v>3.2213</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6732,7 +6812,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C71"/>
+  <dimension ref="A1:C72"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7521,6 +7601,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="72" spans="1:3" ht="16" customHeight="1">
+      <c r="A72" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B72" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C72" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7529,7 +7620,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C71"/>
+  <dimension ref="A1:C72"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8318,6 +8409,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="72" spans="1:3" ht="16" customHeight="1">
+      <c r="A72" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B72" s="3">
+        <v>2.29</v>
+      </c>
+      <c r="C72" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8326,7 +8428,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C71"/>
+  <dimension ref="A1:C72"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9115,6 +9217,17 @@
         <v>4.6667</v>
       </c>
     </row>
+    <row r="72" spans="1:3" ht="16" customHeight="1">
+      <c r="A72" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B72" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C72" s="3">
+        <v>2.2667</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9123,7 +9236,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C71"/>
+  <dimension ref="A1:C72"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9912,6 +10025,17 @@
         <v>3.0667</v>
       </c>
     </row>
+    <row r="72" spans="1:3" ht="16" customHeight="1">
+      <c r="A72" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B72" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C72" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9920,7 +10044,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C71"/>
+  <dimension ref="A1:C72"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10709,6 +10833,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="72" spans="1:3" ht="16" customHeight="1">
+      <c r="A72" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B72" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C72" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-08-19 11:13:27
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2309" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2335" uniqueCount="76">
   <si>
     <t>Date</t>
   </si>
@@ -250,6 +250,9 @@
   </si>
   <si>
     <t>2026-08-18</t>
+  </si>
+  <si>
+    <t>2026-08-19</t>
   </si>
 </sst>
 </file>
@@ -1156,7 +1159,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C72"/>
+  <dimension ref="A1:C73"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1956,6 +1959,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="73" spans="1:3" ht="16" customHeight="1">
+      <c r="A73" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B73" s="3">
+        <v>7.5</v>
+      </c>
+      <c r="C73" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1964,7 +1978,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C72"/>
+  <dimension ref="A1:C73"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2764,6 +2778,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="73" spans="1:3" ht="16" customHeight="1">
+      <c r="A73" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B73" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C73" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2772,7 +2797,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C72"/>
+  <dimension ref="A1:C73"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3572,6 +3597,17 @@
         <v>0.8</v>
       </c>
     </row>
+    <row r="73" spans="1:3" ht="16" customHeight="1">
+      <c r="A73" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B73" s="3">
+        <v>0.88</v>
+      </c>
+      <c r="C73" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3580,7 +3616,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C72"/>
+  <dimension ref="A1:C73"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4380,6 +4416,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="73" spans="1:3" ht="16" customHeight="1">
+      <c r="A73" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B73" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C73" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4388,7 +4435,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C72"/>
+  <dimension ref="A1:C73"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5188,6 +5235,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="73" spans="1:3" ht="16" customHeight="1">
+      <c r="A73" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B73" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C73" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5196,7 +5254,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C72"/>
+  <dimension ref="A1:C73"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5996,6 +6054,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="73" spans="1:3" ht="16" customHeight="1">
+      <c r="A73" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B73" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C73" s="3">
+        <v>8.125</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6004,7 +6073,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C72"/>
+  <dimension ref="A1:C73"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6804,6 +6873,17 @@
         <v>3.2213</v>
       </c>
     </row>
+    <row r="73" spans="1:3" ht="16" customHeight="1">
+      <c r="A73" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B73" s="3">
+        <v>4.47</v>
+      </c>
+      <c r="C73" s="3">
+        <v>3.0667</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6812,7 +6892,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C72"/>
+  <dimension ref="A1:C73"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7612,6 +7692,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="73" spans="1:3" ht="16" customHeight="1">
+      <c r="A73" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B73" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C73" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7620,7 +7711,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C72"/>
+  <dimension ref="A1:C73"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8420,6 +8511,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="73" spans="1:3" ht="16" customHeight="1">
+      <c r="A73" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B73" s="3">
+        <v>2.29</v>
+      </c>
+      <c r="C73" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8428,7 +8530,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C72"/>
+  <dimension ref="A1:C73"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9228,6 +9330,17 @@
         <v>2.2667</v>
       </c>
     </row>
+    <row r="73" spans="1:3" ht="16" customHeight="1">
+      <c r="A73" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B73" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C73" s="3">
+        <v>2.2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9236,7 +9349,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C72"/>
+  <dimension ref="A1:C73"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10036,6 +10149,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="73" spans="1:3" ht="16" customHeight="1">
+      <c r="A73" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B73" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C73" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10044,7 +10168,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C72"/>
+  <dimension ref="A1:C73"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10844,6 +10968,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="73" spans="1:3" ht="16" customHeight="1">
+      <c r="A73" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B73" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C73" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-08-20 11:15:03
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2335" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2360" uniqueCount="77">
   <si>
     <t>Date</t>
   </si>
@@ -254,6 +254,9 @@
   <si>
     <t>2026-08-19</t>
   </si>
+  <si>
+    <t>2026-08-20</t>
+  </si>
 </sst>
 </file>
 
@@ -369,7 +372,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -389,7 +392,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -412,7 +415,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -432,7 +435,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -455,7 +458,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -475,7 +478,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -498,7 +501,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -518,7 +521,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -584,7 +587,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -604,7 +607,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -627,7 +630,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -647,7 +650,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -670,7 +673,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -690,7 +693,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -713,7 +716,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -733,7 +736,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -756,7 +759,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -776,7 +779,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -799,7 +802,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -819,7 +822,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1159,7 +1162,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C73"/>
+  <dimension ref="A1:C74"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1970,6 +1973,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="74" spans="1:3" ht="16" customHeight="1">
+      <c r="A74" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B74" s="3">
+        <v>7.5</v>
+      </c>
+      <c r="C74" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1978,7 +1992,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C73"/>
+  <dimension ref="A1:C74"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2789,6 +2803,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="74" spans="1:3" ht="16" customHeight="1">
+      <c r="A74" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B74" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C74" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2797,7 +2822,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C73"/>
+  <dimension ref="A1:C74"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3608,6 +3633,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="74" spans="1:3" ht="16" customHeight="1">
+      <c r="A74" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B74" s="3">
+        <v>0.88</v>
+      </c>
+      <c r="C74" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3616,7 +3652,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C73"/>
+  <dimension ref="A1:C74"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4427,6 +4463,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="74" spans="1:3" ht="16" customHeight="1">
+      <c r="A74" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B74" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C74" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4435,7 +4482,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C73"/>
+  <dimension ref="A1:C74"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5246,6 +5293,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="74" spans="1:3" ht="16" customHeight="1">
+      <c r="A74" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B74" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C74" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5254,7 +5312,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C73"/>
+  <dimension ref="A1:C74"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6065,6 +6123,17 @@
         <v>8.125</v>
       </c>
     </row>
+    <row r="74" spans="1:3" ht="16" customHeight="1">
+      <c r="A74" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B74" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C74" s="3">
+        <v>8.125</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6073,7 +6142,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C73"/>
+  <dimension ref="A1:C74"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6884,6 +6953,17 @@
         <v>3.0667</v>
       </c>
     </row>
+    <row r="74" spans="1:3" ht="16" customHeight="1">
+      <c r="A74" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B74" s="3">
+        <v>4.47</v>
+      </c>
+      <c r="C74" s="3">
+        <v>4.0614</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6892,7 +6972,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C73"/>
+  <dimension ref="A1:C74"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7703,6 +7783,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="74" spans="1:3" ht="16" customHeight="1">
+      <c r="A74" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B74" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C74" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7711,7 +7802,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C73"/>
+  <dimension ref="A1:C74"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8522,6 +8613,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="74" spans="1:3" ht="16" customHeight="1">
+      <c r="A74" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B74" s="3">
+        <v>2.29</v>
+      </c>
+      <c r="C74" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8530,7 +8632,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C73"/>
+  <dimension ref="A1:C74"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9341,6 +9443,17 @@
         <v>2.2</v>
       </c>
     </row>
+    <row r="74" spans="1:3" ht="16" customHeight="1">
+      <c r="A74" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B74" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C74" s="3">
+        <v>2.2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9349,7 +9462,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C73"/>
+  <dimension ref="A1:C74"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10160,6 +10273,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="74" spans="1:3" ht="16" customHeight="1">
+      <c r="A74" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B74" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C74" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10168,7 +10292,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C73"/>
+  <dimension ref="A1:C74"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10979,6 +11103,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="74" spans="1:3" ht="16" customHeight="1">
+      <c r="A74" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B74" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C74" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-08-21 11:14:45
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2360" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2384" uniqueCount="78">
   <si>
     <t>Date</t>
   </si>
@@ -257,6 +257,9 @@
   <si>
     <t>2026-08-20</t>
   </si>
+  <si>
+    <t>2026-08-21</t>
+  </si>
 </sst>
 </file>
 
@@ -372,7 +375,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -392,7 +395,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -415,7 +418,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -435,7 +438,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -458,7 +461,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -478,7 +481,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -501,7 +504,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -521,7 +524,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -587,7 +590,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -607,7 +610,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -630,7 +633,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -650,7 +653,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -673,7 +676,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -693,7 +696,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -716,7 +719,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -736,7 +739,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -759,7 +762,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -779,7 +782,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -802,7 +805,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -822,7 +825,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1162,7 +1165,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C74"/>
+  <dimension ref="A1:C75"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1984,6 +1987,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="75" spans="1:3" ht="16" customHeight="1">
+      <c r="A75" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B75" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C75" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1992,7 +2006,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C74"/>
+  <dimension ref="A1:C75"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2814,6 +2828,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="75" spans="1:3" ht="16" customHeight="1">
+      <c r="A75" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B75" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C75" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2822,7 +2847,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C74"/>
+  <dimension ref="A1:C75"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3644,6 +3669,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="75" spans="1:3" ht="16" customHeight="1">
+      <c r="A75" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B75" s="3">
+        <v>0.88</v>
+      </c>
+      <c r="C75" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3652,7 +3688,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C74"/>
+  <dimension ref="A1:C75"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4474,6 +4510,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="75" spans="1:3" ht="16" customHeight="1">
+      <c r="A75" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B75" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C75" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4482,7 +4529,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C74"/>
+  <dimension ref="A1:C75"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5304,6 +5351,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="75" spans="1:3" ht="16" customHeight="1">
+      <c r="A75" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B75" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C75" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5312,7 +5370,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C74"/>
+  <dimension ref="A1:C75"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6134,6 +6192,17 @@
         <v>8.125</v>
       </c>
     </row>
+    <row r="75" spans="1:3" ht="16" customHeight="1">
+      <c r="A75" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B75" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C75" s="3">
+        <v>8.75</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6142,7 +6211,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C74"/>
+  <dimension ref="A1:C75"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6964,6 +7033,17 @@
         <v>4.0614</v>
       </c>
     </row>
+    <row r="75" spans="1:3" ht="16" customHeight="1">
+      <c r="A75" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B75" s="3">
+        <v>4.47</v>
+      </c>
+      <c r="C75" s="3">
+        <v>4.0946</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6972,7 +7052,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C74"/>
+  <dimension ref="A1:C75"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7794,6 +7874,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="75" spans="1:3" ht="16" customHeight="1">
+      <c r="A75" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B75" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C75" s="3">
+        <v>4.2079</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7802,7 +7893,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C74"/>
+  <dimension ref="A1:C75"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8624,6 +8715,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="75" spans="1:3" ht="16" customHeight="1">
+      <c r="A75" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B75" s="3">
+        <v>2.29</v>
+      </c>
+      <c r="C75" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8632,7 +8734,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C74"/>
+  <dimension ref="A1:C75"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9454,6 +9556,17 @@
         <v>2.2</v>
       </c>
     </row>
+    <row r="75" spans="1:3" ht="16" customHeight="1">
+      <c r="A75" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B75" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C75" s="3">
+        <v>2.4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9462,7 +9575,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C74"/>
+  <dimension ref="A1:C75"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10284,6 +10397,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="75" spans="1:3" ht="16" customHeight="1">
+      <c r="A75" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B75" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C75" s="3">
+        <v>2.3827</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10292,7 +10416,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C74"/>
+  <dimension ref="A1:C75"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11114,6 +11238,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="75" spans="1:3" ht="16" customHeight="1">
+      <c r="A75" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B75" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C75" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-08-22 11:10:08
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2384" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2409" uniqueCount="79">
   <si>
     <t>Date</t>
   </si>
@@ -259,6 +259,9 @@
   </si>
   <si>
     <t>2026-08-21</t>
+  </si>
+  <si>
+    <t>2026-08-22</t>
   </si>
 </sst>
 </file>
@@ -1165,7 +1168,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C75"/>
+  <dimension ref="A1:C76"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -1998,6 +2001,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="76" spans="1:3" ht="16" customHeight="1">
+      <c r="A76" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B76" s="3">
+        <v>7.4</v>
+      </c>
+      <c r="C76" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2006,7 +2020,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C75"/>
+  <dimension ref="A1:C76"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2839,6 +2853,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="76" spans="1:3" ht="16" customHeight="1">
+      <c r="A76" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B76" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C76" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2847,7 +2872,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C75"/>
+  <dimension ref="A1:C76"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3680,6 +3705,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="76" spans="1:3" ht="16" customHeight="1">
+      <c r="A76" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B76" s="3">
+        <v>0.88</v>
+      </c>
+      <c r="C76" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3688,7 +3724,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C75"/>
+  <dimension ref="A1:C76"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4521,6 +4557,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="76" spans="1:3" ht="16" customHeight="1">
+      <c r="A76" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B76" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C76" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4529,7 +4576,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C75"/>
+  <dimension ref="A1:C76"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5362,6 +5409,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="76" spans="1:3" ht="16" customHeight="1">
+      <c r="A76" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B76" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C76" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5370,7 +5428,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C75"/>
+  <dimension ref="A1:C76"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6203,6 +6261,17 @@
         <v>8.75</v>
       </c>
     </row>
+    <row r="76" spans="1:3" ht="16" customHeight="1">
+      <c r="A76" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B76" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C76" s="3">
+        <v>7.125</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6211,7 +6280,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C75"/>
+  <dimension ref="A1:C76"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7044,6 +7113,17 @@
         <v>4.0946</v>
       </c>
     </row>
+    <row r="76" spans="1:3" ht="16" customHeight="1">
+      <c r="A76" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B76" s="3">
+        <v>4.47</v>
+      </c>
+      <c r="C76" s="3">
+        <v>3.6707</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7052,7 +7132,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C75"/>
+  <dimension ref="A1:C76"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7885,6 +7965,17 @@
         <v>4.2079</v>
       </c>
     </row>
+    <row r="76" spans="1:3" ht="16" customHeight="1">
+      <c r="A76" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B76" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C76" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7893,7 +7984,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C75"/>
+  <dimension ref="A1:C76"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8726,6 +8817,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="76" spans="1:3" ht="16" customHeight="1">
+      <c r="A76" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B76" s="3">
+        <v>1.99</v>
+      </c>
+      <c r="C76" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8734,7 +8836,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C75"/>
+  <dimension ref="A1:C76"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9567,6 +9669,17 @@
         <v>2.4</v>
       </c>
     </row>
+    <row r="76" spans="1:3" ht="16" customHeight="1">
+      <c r="A76" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B76" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C76" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9575,7 +9688,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C75"/>
+  <dimension ref="A1:C76"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10408,6 +10521,17 @@
         <v>2.3827</v>
       </c>
     </row>
+    <row r="76" spans="1:3" ht="16" customHeight="1">
+      <c r="A76" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B76" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C76" s="3">
+        <v>2.8267</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10416,7 +10540,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C75"/>
+  <dimension ref="A1:C76"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11249,6 +11373,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="76" spans="1:3" ht="16" customHeight="1">
+      <c r="A76" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B76" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C76" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-08-23 11:10:18
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2409" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2433" uniqueCount="80">
   <si>
     <t>Date</t>
   </si>
@@ -262,6 +262,9 @@
   </si>
   <si>
     <t>2026-08-22</t>
+  </si>
+  <si>
+    <t>2026-08-23</t>
   </si>
 </sst>
 </file>
@@ -1168,7 +1171,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C76"/>
+  <dimension ref="A1:C77"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2012,6 +2015,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="77" spans="1:3" ht="16" customHeight="1">
+      <c r="A77" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B77" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C77" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2020,7 +2034,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C76"/>
+  <dimension ref="A1:C77"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2864,6 +2878,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="77" spans="1:3" ht="16" customHeight="1">
+      <c r="A77" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B77" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C77" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2872,7 +2897,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C76"/>
+  <dimension ref="A1:C77"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3716,6 +3741,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="77" spans="1:3" ht="16" customHeight="1">
+      <c r="A77" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B77" s="3">
+        <v>0.88</v>
+      </c>
+      <c r="C77" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3724,7 +3760,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C76"/>
+  <dimension ref="A1:C77"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4568,6 +4604,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="77" spans="1:3" ht="16" customHeight="1">
+      <c r="A77" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B77" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C77" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4576,7 +4623,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C76"/>
+  <dimension ref="A1:C77"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5420,6 +5467,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="77" spans="1:3" ht="16" customHeight="1">
+      <c r="A77" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B77" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C77" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5428,7 +5486,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C76"/>
+  <dimension ref="A1:C77"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6272,6 +6330,17 @@
         <v>7.125</v>
       </c>
     </row>
+    <row r="77" spans="1:3" ht="16" customHeight="1">
+      <c r="A77" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B77" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C77" s="3">
+        <v>6.625</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6280,7 +6349,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C76"/>
+  <dimension ref="A1:C77"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7124,6 +7193,17 @@
         <v>3.6707</v>
       </c>
     </row>
+    <row r="77" spans="1:3" ht="16" customHeight="1">
+      <c r="A77" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B77" s="3">
+        <v>4.47</v>
+      </c>
+      <c r="C77" s="3">
+        <v>3.2214</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7132,7 +7212,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C76"/>
+  <dimension ref="A1:C77"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7976,6 +8056,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="77" spans="1:3" ht="16" customHeight="1">
+      <c r="A77" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B77" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C77" s="3">
+        <v>3.9421</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7984,7 +8075,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C76"/>
+  <dimension ref="A1:C77"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8828,6 +8919,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="77" spans="1:3" ht="16" customHeight="1">
+      <c r="A77" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B77" s="3">
+        <v>1.99</v>
+      </c>
+      <c r="C77" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8836,7 +8938,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C76"/>
+  <dimension ref="A1:C77"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9680,6 +9782,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="77" spans="1:3" ht="16" customHeight="1">
+      <c r="A77" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B77" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C77" s="3">
+        <v>2.2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9688,7 +9801,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C76"/>
+  <dimension ref="A1:C77"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10532,6 +10645,17 @@
         <v>2.8267</v>
       </c>
     </row>
+    <row r="77" spans="1:3" ht="16" customHeight="1">
+      <c r="A77" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B77" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C77" s="3">
+        <v>2.9067</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10540,7 +10664,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C76"/>
+  <dimension ref="A1:C77"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11384,6 +11508,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="77" spans="1:3" ht="16" customHeight="1">
+      <c r="A77" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B77" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C77" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-08-24 11:16:18
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2433" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2458" uniqueCount="81">
   <si>
     <t>Date</t>
   </si>
@@ -265,6 +265,9 @@
   </si>
   <si>
     <t>2026-08-23</t>
+  </si>
+  <si>
+    <t>2026-08-24</t>
   </si>
 </sst>
 </file>
@@ -1171,7 +1174,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C77"/>
+  <dimension ref="A1:C78"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2026,6 +2029,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="78" spans="1:3" ht="16" customHeight="1">
+      <c r="A78" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B78" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C78" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2034,7 +2048,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C77"/>
+  <dimension ref="A1:C78"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2889,6 +2903,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="78" spans="1:3" ht="16" customHeight="1">
+      <c r="A78" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B78" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C78" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2897,7 +2922,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C77"/>
+  <dimension ref="A1:C78"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3752,6 +3777,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="78" spans="1:3" ht="16" customHeight="1">
+      <c r="A78" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B78" s="3">
+        <v>0.88</v>
+      </c>
+      <c r="C78" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3760,7 +3796,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C77"/>
+  <dimension ref="A1:C78"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4615,6 +4651,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="78" spans="1:3" ht="16" customHeight="1">
+      <c r="A78" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B78" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C78" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4623,7 +4670,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C77"/>
+  <dimension ref="A1:C78"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5478,6 +5525,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="78" spans="1:3" ht="16" customHeight="1">
+      <c r="A78" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B78" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C78" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5486,7 +5544,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C77"/>
+  <dimension ref="A1:C78"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6341,6 +6399,17 @@
         <v>6.625</v>
       </c>
     </row>
+    <row r="78" spans="1:3" ht="16" customHeight="1">
+      <c r="A78" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B78" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C78" s="3">
+        <v>6.625</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6349,7 +6418,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C77"/>
+  <dimension ref="A1:C78"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7204,6 +7273,17 @@
         <v>3.2214</v>
       </c>
     </row>
+    <row r="78" spans="1:3" ht="16" customHeight="1">
+      <c r="A78" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B78" s="3">
+        <v>4.47</v>
+      </c>
+      <c r="C78" s="3">
+        <v>3.488</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7212,7 +7292,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C77"/>
+  <dimension ref="A1:C78"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8067,6 +8147,17 @@
         <v>3.9421</v>
       </c>
     </row>
+    <row r="78" spans="1:3" ht="16" customHeight="1">
+      <c r="A78" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B78" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C78" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8075,7 +8166,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C77"/>
+  <dimension ref="A1:C78"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8930,6 +9021,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="78" spans="1:3" ht="16" customHeight="1">
+      <c r="A78" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B78" s="3">
+        <v>1.99</v>
+      </c>
+      <c r="C78" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8938,7 +9040,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C77"/>
+  <dimension ref="A1:C78"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9793,6 +9895,17 @@
         <v>2.2</v>
       </c>
     </row>
+    <row r="78" spans="1:3" ht="16" customHeight="1">
+      <c r="A78" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B78" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C78" s="3">
+        <v>2.504</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9801,7 +9914,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C77"/>
+  <dimension ref="A1:C78"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10656,6 +10769,17 @@
         <v>2.9067</v>
       </c>
     </row>
+    <row r="78" spans="1:3" ht="16" customHeight="1">
+      <c r="A78" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B78" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C78" s="3">
+        <v>2.3827</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10664,7 +10788,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C77"/>
+  <dimension ref="A1:C78"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11519,6 +11643,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="78" spans="1:3" ht="16" customHeight="1">
+      <c r="A78" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B78" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C78" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-08-25 11:15:10
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2458" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2481" uniqueCount="82">
   <si>
     <t>Date</t>
   </si>
@@ -268,6 +268,9 @@
   </si>
   <si>
     <t>2026-08-24</t>
+  </si>
+  <si>
+    <t>2026-08-25</t>
   </si>
 </sst>
 </file>
@@ -1174,7 +1177,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C78"/>
+  <dimension ref="A1:C79"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2040,6 +2043,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="79" spans="1:3" ht="16" customHeight="1">
+      <c r="A79" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B79" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C79" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2048,7 +2062,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C78"/>
+  <dimension ref="A1:C79"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2914,6 +2928,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="79" spans="1:3" ht="16" customHeight="1">
+      <c r="A79" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B79" s="3">
+        <v>3.39</v>
+      </c>
+      <c r="C79" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2922,7 +2947,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C78"/>
+  <dimension ref="A1:C79"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3788,6 +3813,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="79" spans="1:3" ht="16" customHeight="1">
+      <c r="A79" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B79" s="3">
+        <v>0.88</v>
+      </c>
+      <c r="C79" s="3">
+        <v>0.8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3796,7 +3832,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C78"/>
+  <dimension ref="A1:C79"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4662,6 +4698,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="79" spans="1:3" ht="16" customHeight="1">
+      <c r="A79" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B79" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C79" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4670,7 +4717,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C78"/>
+  <dimension ref="A1:C79"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5536,6 +5583,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="79" spans="1:3" ht="16" customHeight="1">
+      <c r="A79" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B79" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C79" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5544,7 +5602,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C78"/>
+  <dimension ref="A1:C79"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6410,6 +6468,17 @@
         <v>6.625</v>
       </c>
     </row>
+    <row r="79" spans="1:3" ht="16" customHeight="1">
+      <c r="A79" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B79" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C79" s="3">
+        <v>7.125</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6418,7 +6487,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C78"/>
+  <dimension ref="A1:C79"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7284,6 +7353,17 @@
         <v>3.488</v>
       </c>
     </row>
+    <row r="79" spans="1:3" ht="16" customHeight="1">
+      <c r="A79" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B79" s="3">
+        <v>4.47</v>
+      </c>
+      <c r="C79" s="3">
+        <v>3.924</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7292,7 +7372,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C78"/>
+  <dimension ref="A1:C79"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8158,6 +8238,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="79" spans="1:3" ht="16" customHeight="1">
+      <c r="A79" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B79" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C79" s="3">
+        <v>4.4066</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8166,7 +8257,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C78"/>
+  <dimension ref="A1:C79"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9032,6 +9123,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="79" spans="1:3" ht="16" customHeight="1">
+      <c r="A79" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B79" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C79" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9040,7 +9142,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C78"/>
+  <dimension ref="A1:C79"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9906,6 +10008,17 @@
         <v>2.504</v>
       </c>
     </row>
+    <row r="79" spans="1:3" ht="16" customHeight="1">
+      <c r="A79" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B79" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C79" s="3">
+        <v>2.6667</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9914,7 +10027,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C78"/>
+  <dimension ref="A1:C79"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10780,6 +10893,17 @@
         <v>2.3827</v>
       </c>
     </row>
+    <row r="79" spans="1:3" ht="16" customHeight="1">
+      <c r="A79" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B79" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C79" s="3">
+        <v>4.6667</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10788,7 +10912,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C78"/>
+  <dimension ref="A1:C79"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11654,6 +11778,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="79" spans="1:3" ht="16" customHeight="1">
+      <c r="A79" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B79" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C79" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-08-26 11:17:55
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2481" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2506" uniqueCount="83">
   <si>
     <t>Date</t>
   </si>
@@ -271,6 +271,9 @@
   </si>
   <si>
     <t>2026-08-25</t>
+  </si>
+  <si>
+    <t>2026-08-26</t>
   </si>
 </sst>
 </file>
@@ -1177,7 +1180,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C79"/>
+  <dimension ref="A1:C80"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2054,6 +2057,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="80" spans="1:3" ht="16" customHeight="1">
+      <c r="A80" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B80" s="3">
+        <v>7.5</v>
+      </c>
+      <c r="C80" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2062,7 +2076,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C79"/>
+  <dimension ref="A1:C80"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2939,6 +2953,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="80" spans="1:3" ht="16" customHeight="1">
+      <c r="A80" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B80" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C80" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2947,7 +2972,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C79"/>
+  <dimension ref="A1:C80"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3824,6 +3849,17 @@
         <v>0.8</v>
       </c>
     </row>
+    <row r="80" spans="1:3" ht="16" customHeight="1">
+      <c r="A80" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B80" s="3">
+        <v>0.88</v>
+      </c>
+      <c r="C80" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3832,7 +3868,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C79"/>
+  <dimension ref="A1:C80"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4709,6 +4745,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="80" spans="1:3" ht="16" customHeight="1">
+      <c r="A80" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B80" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C80" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4717,7 +4764,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C79"/>
+  <dimension ref="A1:C80"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5594,6 +5641,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="80" spans="1:3" ht="16" customHeight="1">
+      <c r="A80" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B80" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C80" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5602,7 +5660,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C79"/>
+  <dimension ref="A1:C80"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6479,6 +6537,17 @@
         <v>7.125</v>
       </c>
     </row>
+    <row r="80" spans="1:3" ht="16" customHeight="1">
+      <c r="A80" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B80" s="3">
+        <v>6.99</v>
+      </c>
+      <c r="C80" s="3">
+        <v>5.625</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6487,7 +6556,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C79"/>
+  <dimension ref="A1:C80"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7364,6 +7433,17 @@
         <v>3.924</v>
       </c>
     </row>
+    <row r="80" spans="1:3" ht="16" customHeight="1">
+      <c r="A80" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B80" s="3">
+        <v>4.47</v>
+      </c>
+      <c r="C80" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7372,7 +7452,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C79"/>
+  <dimension ref="A1:C80"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8249,6 +8329,17 @@
         <v>4.4066</v>
       </c>
     </row>
+    <row r="80" spans="1:3" ht="16" customHeight="1">
+      <c r="A80" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B80" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C80" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8257,7 +8348,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C79"/>
+  <dimension ref="A1:C80"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9134,6 +9225,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="80" spans="1:3" ht="16" customHeight="1">
+      <c r="A80" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B80" s="3">
+        <v>2.29</v>
+      </c>
+      <c r="C80" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9142,7 +9244,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C79"/>
+  <dimension ref="A1:C80"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10019,6 +10121,17 @@
         <v>2.6667</v>
       </c>
     </row>
+    <row r="80" spans="1:3" ht="16" customHeight="1">
+      <c r="A80" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B80" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C80" s="3">
+        <v>3.2133</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10027,7 +10140,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C79"/>
+  <dimension ref="A1:C80"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10904,6 +11017,17 @@
         <v>4.6667</v>
       </c>
     </row>
+    <row r="80" spans="1:3" ht="16" customHeight="1">
+      <c r="A80" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B80" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C80" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10912,7 +11036,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C79"/>
+  <dimension ref="A1:C80"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11789,6 +11913,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="80" spans="1:3" ht="16" customHeight="1">
+      <c r="A80" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B80" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C80" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-08-27 20:50:06
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2506" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2530" uniqueCount="84">
   <si>
     <t>Date</t>
   </si>
@@ -274,6 +274,9 @@
   </si>
   <si>
     <t>2026-08-26</t>
+  </si>
+  <si>
+    <t>2026-08-27</t>
   </si>
 </sst>
 </file>
@@ -1180,7 +1183,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C80"/>
+  <dimension ref="A1:C81"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2068,6 +2071,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="81" spans="1:3" ht="16" customHeight="1">
+      <c r="A81" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B81" s="3">
+        <v>7.5</v>
+      </c>
+      <c r="C81" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2076,7 +2090,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C80"/>
+  <dimension ref="A1:C81"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2964,6 +2978,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="81" spans="1:3" ht="16" customHeight="1">
+      <c r="A81" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B81" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C81" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2972,7 +2997,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C80"/>
+  <dimension ref="A1:C81"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3860,6 +3885,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="81" spans="1:3" ht="16" customHeight="1">
+      <c r="A81" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B81" s="3">
+        <v>0.88</v>
+      </c>
+      <c r="C81" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3868,7 +3904,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C80"/>
+  <dimension ref="A1:C81"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4756,6 +4792,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="81" spans="1:3" ht="16" customHeight="1">
+      <c r="A81" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B81" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C81" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4764,7 +4811,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C80"/>
+  <dimension ref="A1:C81"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5652,6 +5699,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="81" spans="1:3" ht="16" customHeight="1">
+      <c r="A81" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B81" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C81" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5660,7 +5718,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C80"/>
+  <dimension ref="A1:C81"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6548,6 +6606,17 @@
         <v>5.625</v>
       </c>
     </row>
+    <row r="81" spans="1:3" ht="16" customHeight="1">
+      <c r="A81" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B81" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C81" s="3">
+        <v>5.625</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6556,7 +6625,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C80"/>
+  <dimension ref="A1:C81"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7444,6 +7513,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="81" spans="1:3" ht="16" customHeight="1">
+      <c r="A81" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B81" s="3">
+        <v>4.47</v>
+      </c>
+      <c r="C81" s="3">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7452,7 +7532,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C80"/>
+  <dimension ref="A1:C81"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8340,6 +8420,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="81" spans="1:3" ht="16" customHeight="1">
+      <c r="A81" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B81" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C81" s="3">
+        <v>4.3408</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8348,7 +8439,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C80"/>
+  <dimension ref="A1:C81"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9236,6 +9327,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="81" spans="1:3" ht="16" customHeight="1">
+      <c r="A81" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B81" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C81" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9244,7 +9346,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C80"/>
+  <dimension ref="A1:C81"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10132,6 +10234,17 @@
         <v>3.2133</v>
       </c>
     </row>
+    <row r="81" spans="1:3" ht="16" customHeight="1">
+      <c r="A81" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B81" s="3">
+        <v>2.9</v>
+      </c>
+      <c r="C81" s="3">
+        <v>2.2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10140,7 +10253,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C80"/>
+  <dimension ref="A1:C81"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11028,6 +11141,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="81" spans="1:3" ht="16" customHeight="1">
+      <c r="A81" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B81" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C81" s="3">
+        <v>2.68</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11036,7 +11160,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C80"/>
+  <dimension ref="A1:C81"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11924,6 +12048,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="81" spans="1:3" ht="16" customHeight="1">
+      <c r="A81" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B81" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C81" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-08-28 21:17:00
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2530" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2554" uniqueCount="85">
   <si>
     <t>Date</t>
   </si>
@@ -278,6 +278,9 @@
   <si>
     <t>2026-08-27</t>
   </si>
+  <si>
+    <t>2026-08-28</t>
+  </si>
 </sst>
 </file>
 
@@ -393,7 +396,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -413,7 +416,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -436,7 +439,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -456,7 +459,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -479,7 +482,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -499,7 +502,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -522,7 +525,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -542,7 +545,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -608,7 +611,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -628,7 +631,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -651,7 +654,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -671,7 +674,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -694,7 +697,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -714,7 +717,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -737,7 +740,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -757,7 +760,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -780,7 +783,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -800,7 +803,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -823,7 +826,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -843,7 +846,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1183,7 +1186,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C81"/>
+  <dimension ref="A1:C82"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2082,6 +2085,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="82" spans="1:3" ht="16" customHeight="1">
+      <c r="A82" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B82" s="3">
+        <v>7.4</v>
+      </c>
+      <c r="C82" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2090,7 +2104,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C81"/>
+  <dimension ref="A1:C82"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2989,6 +3003,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="82" spans="1:3" ht="16" customHeight="1">
+      <c r="A82" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B82" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C82" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2997,7 +3022,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C81"/>
+  <dimension ref="A1:C82"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3896,6 +3921,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="82" spans="1:3" ht="16" customHeight="1">
+      <c r="A82" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B82" s="3">
+        <v>0.88</v>
+      </c>
+      <c r="C82" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3904,7 +3940,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C81"/>
+  <dimension ref="A1:C82"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4803,6 +4839,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="82" spans="1:3" ht="16" customHeight="1">
+      <c r="A82" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B82" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C82" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4811,7 +4858,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C81"/>
+  <dimension ref="A1:C82"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5710,6 +5757,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="82" spans="1:3" ht="16" customHeight="1">
+      <c r="A82" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B82" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C82" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5718,7 +5776,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C81"/>
+  <dimension ref="A1:C82"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6617,6 +6675,17 @@
         <v>5.625</v>
       </c>
     </row>
+    <row r="82" spans="1:3" ht="16" customHeight="1">
+      <c r="A82" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B82" s="3">
+        <v>6</v>
+      </c>
+      <c r="C82" s="3">
+        <v>5.875</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6625,7 +6694,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C81"/>
+  <dimension ref="A1:C82"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7524,6 +7593,17 @@
         <v>5</v>
       </c>
     </row>
+    <row r="82" spans="1:3" ht="16" customHeight="1">
+      <c r="A82" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B82" s="3">
+        <v>4.47</v>
+      </c>
+      <c r="C82" s="3">
+        <v>4.1373</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7532,7 +7612,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C81"/>
+  <dimension ref="A1:C82"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8431,6 +8511,17 @@
         <v>4.3408</v>
       </c>
     </row>
+    <row r="82" spans="1:3" ht="16" customHeight="1">
+      <c r="A82" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B82" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C82" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8439,7 +8530,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C81"/>
+  <dimension ref="A1:C82"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9338,6 +9429,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="82" spans="1:3" ht="16" customHeight="1">
+      <c r="A82" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B82" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C82" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9346,7 +9448,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C81"/>
+  <dimension ref="A1:C82"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10245,6 +10347,17 @@
         <v>2.2</v>
       </c>
     </row>
+    <row r="82" spans="1:3" ht="16" customHeight="1">
+      <c r="A82" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B82" s="3">
+        <v>2.89</v>
+      </c>
+      <c r="C82" s="3">
+        <v>2.2667</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10253,7 +10366,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C81"/>
+  <dimension ref="A1:C82"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11152,6 +11265,17 @@
         <v>2.68</v>
       </c>
     </row>
+    <row r="82" spans="1:3" ht="16" customHeight="1">
+      <c r="A82" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B82" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C82" s="3">
+        <v>3.0133</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11160,7 +11284,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C81"/>
+  <dimension ref="A1:C82"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12059,6 +12183,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="82" spans="1:3" ht="16" customHeight="1">
+      <c r="A82" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B82" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C82" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-08-29 15:21:48
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2554" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2576" uniqueCount="86">
   <si>
     <t>Date</t>
   </si>
@@ -281,6 +281,9 @@
   <si>
     <t>2026-08-28</t>
   </si>
+  <si>
+    <t>2026-08-29</t>
+  </si>
 </sst>
 </file>
 
@@ -396,7 +399,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -416,7 +419,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -439,7 +442,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -459,7 +462,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -482,7 +485,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -502,7 +505,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -525,7 +528,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -545,7 +548,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -611,7 +614,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -631,7 +634,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -654,7 +657,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -674,7 +677,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -697,7 +700,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -717,7 +720,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -740,7 +743,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -760,7 +763,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -783,7 +786,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -803,7 +806,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -826,7 +829,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -846,7 +849,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1186,7 +1189,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C82"/>
+  <dimension ref="A1:C83"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2096,6 +2099,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="83" spans="1:3" ht="16" customHeight="1">
+      <c r="A83" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B83" s="3">
+        <v>7.4</v>
+      </c>
+      <c r="C83" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2104,7 +2118,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C82"/>
+  <dimension ref="A1:C83"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3014,6 +3028,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="83" spans="1:3" ht="16" customHeight="1">
+      <c r="A83" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B83" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C83" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3022,7 +3047,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C82"/>
+  <dimension ref="A1:C83"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3932,6 +3957,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="83" spans="1:3" ht="16" customHeight="1">
+      <c r="A83" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B83" s="3">
+        <v>0.88</v>
+      </c>
+      <c r="C83" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3940,7 +3976,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C82"/>
+  <dimension ref="A1:C83"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4850,6 +4886,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="83" spans="1:3" ht="16" customHeight="1">
+      <c r="A83" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B83" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C83" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4858,7 +4905,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C82"/>
+  <dimension ref="A1:C83"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5768,6 +5815,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="83" spans="1:3" ht="16" customHeight="1">
+      <c r="A83" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B83" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C83" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5776,7 +5834,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C82"/>
+  <dimension ref="A1:C83"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6686,6 +6744,17 @@
         <v>5.875</v>
       </c>
     </row>
+    <row r="83" spans="1:3" ht="16" customHeight="1">
+      <c r="A83" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B83" s="3">
+        <v>6</v>
+      </c>
+      <c r="C83" s="3">
+        <v>5.875</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6694,7 +6763,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C82"/>
+  <dimension ref="A1:C83"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7604,6 +7673,17 @@
         <v>4.1373</v>
       </c>
     </row>
+    <row r="83" spans="1:3" ht="16" customHeight="1">
+      <c r="A83" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B83" s="3">
+        <v>4.47</v>
+      </c>
+      <c r="C83" s="3">
+        <v>4.4507</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7612,7 +7692,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C82"/>
+  <dimension ref="A1:C83"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8522,6 +8602,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="83" spans="1:3" ht="16" customHeight="1">
+      <c r="A83" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B83" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C83" s="3">
+        <v>4.5382</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8530,7 +8621,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C82"/>
+  <dimension ref="A1:C83"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9440,6 +9531,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="83" spans="1:3" ht="16" customHeight="1">
+      <c r="A83" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B83" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C83" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9448,7 +9550,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C82"/>
+  <dimension ref="A1:C83"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10358,6 +10460,17 @@
         <v>2.2667</v>
       </c>
     </row>
+    <row r="83" spans="1:3" ht="16" customHeight="1">
+      <c r="A83" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B83" s="3">
+        <v>2.89</v>
+      </c>
+      <c r="C83" s="3">
+        <v>2.972</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10366,7 +10479,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C82"/>
+  <dimension ref="A1:C83"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11276,6 +11389,17 @@
         <v>3.0133</v>
       </c>
     </row>
+    <row r="83" spans="1:3" ht="16" customHeight="1">
+      <c r="A83" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B83" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C83" s="3">
+        <v>2.7334</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11284,7 +11408,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C82"/>
+  <dimension ref="A1:C83"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12194,6 +12318,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="83" spans="1:3" ht="16" customHeight="1">
+      <c r="A83" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B83" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C83" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-08-30 15:05:20
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2576" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2599" uniqueCount="87">
   <si>
     <t>Date</t>
   </si>
@@ -283,6 +283,9 @@
   </si>
   <si>
     <t>2026-08-29</t>
+  </si>
+  <si>
+    <t>2026-08-30</t>
   </si>
 </sst>
 </file>
@@ -1189,7 +1192,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C83"/>
+  <dimension ref="A1:C84"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2110,6 +2113,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="84" spans="1:3" ht="16" customHeight="1">
+      <c r="A84" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B84" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C84" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2118,7 +2132,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C83"/>
+  <dimension ref="A1:C84"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3039,6 +3053,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="84" spans="1:3" ht="16" customHeight="1">
+      <c r="A84" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B84" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C84" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3047,7 +3072,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C83"/>
+  <dimension ref="A1:C84"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3968,6 +3993,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="84" spans="1:3" ht="16" customHeight="1">
+      <c r="A84" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B84" s="3">
+        <v>0.88</v>
+      </c>
+      <c r="C84" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3976,7 +4012,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C83"/>
+  <dimension ref="A1:C84"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4897,6 +4933,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="84" spans="1:3" ht="16" customHeight="1">
+      <c r="A84" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B84" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C84" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4905,7 +4952,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C83"/>
+  <dimension ref="A1:C84"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5826,6 +5873,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="84" spans="1:3" ht="16" customHeight="1">
+      <c r="A84" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B84" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C84" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5834,7 +5892,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C83"/>
+  <dimension ref="A1:C84"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6755,6 +6813,17 @@
         <v>5.875</v>
       </c>
     </row>
+    <row r="84" spans="1:3" ht="16" customHeight="1">
+      <c r="A84" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B84" s="3">
+        <v>6</v>
+      </c>
+      <c r="C84" s="3">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6763,7 +6832,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C83"/>
+  <dimension ref="A1:C84"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7684,6 +7753,17 @@
         <v>4.4507</v>
       </c>
     </row>
+    <row r="84" spans="1:3" ht="16" customHeight="1">
+      <c r="A84" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B84" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C84" s="3">
+        <v>4.4534</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7692,7 +7772,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C83"/>
+  <dimension ref="A1:C84"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8613,6 +8693,17 @@
         <v>4.5382</v>
       </c>
     </row>
+    <row r="84" spans="1:3" ht="16" customHeight="1">
+      <c r="A84" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B84" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C84" s="3">
+        <v>7.8947</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8621,7 +8712,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C83"/>
+  <dimension ref="A1:C84"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9542,6 +9633,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="84" spans="1:3" ht="16" customHeight="1">
+      <c r="A84" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B84" s="3">
+        <v>2.29</v>
+      </c>
+      <c r="C84" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9550,7 +9652,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C83"/>
+  <dimension ref="A1:C84"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10471,6 +10573,17 @@
         <v>2.972</v>
       </c>
     </row>
+    <row r="84" spans="1:3" ht="16" customHeight="1">
+      <c r="A84" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B84" s="3">
+        <v>2.89</v>
+      </c>
+      <c r="C84" s="3">
+        <v>2.2667</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10479,7 +10592,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C83"/>
+  <dimension ref="A1:C84"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11400,6 +11513,17 @@
         <v>2.7334</v>
       </c>
     </row>
+    <row r="84" spans="1:3" ht="16" customHeight="1">
+      <c r="A84" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B84" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C84" s="3">
+        <v>2.7333</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11408,7 +11532,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C83"/>
+  <dimension ref="A1:C84"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12329,6 +12453,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="84" spans="1:3" ht="16" customHeight="1">
+      <c r="A84" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B84" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C84" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-08-31 17:44:08
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2599" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2623" uniqueCount="88">
   <si>
     <t>Date</t>
   </si>
@@ -286,6 +286,9 @@
   </si>
   <si>
     <t>2026-08-30</t>
+  </si>
+  <si>
+    <t>2026-08-31</t>
   </si>
 </sst>
 </file>
@@ -1192,7 +1195,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C84"/>
+  <dimension ref="A1:C85"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2124,6 +2127,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="85" spans="1:3" ht="16" customHeight="1">
+      <c r="A85" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B85" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C85" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2132,7 +2146,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C84"/>
+  <dimension ref="A1:C85"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3064,6 +3078,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="85" spans="1:3" ht="16" customHeight="1">
+      <c r="A85" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B85" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C85" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3072,7 +3097,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C84"/>
+  <dimension ref="A1:C85"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4004,6 +4029,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="85" spans="1:3" ht="16" customHeight="1">
+      <c r="A85" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B85" s="3">
+        <v>0.88</v>
+      </c>
+      <c r="C85" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4012,7 +4048,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C84"/>
+  <dimension ref="A1:C85"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4944,6 +4980,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="85" spans="1:3" ht="16" customHeight="1">
+      <c r="A85" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B85" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C85" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4952,7 +4999,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C84"/>
+  <dimension ref="A1:C85"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5884,6 +5931,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="85" spans="1:3" ht="16" customHeight="1">
+      <c r="A85" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B85" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C85" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5892,7 +5950,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C84"/>
+  <dimension ref="A1:C85"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6824,6 +6882,17 @@
         <v>6</v>
       </c>
     </row>
+    <row r="85" spans="1:3" ht="16" customHeight="1">
+      <c r="A85" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B85" s="3">
+        <v>6</v>
+      </c>
+      <c r="C85" s="3">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6832,7 +6901,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C84"/>
+  <dimension ref="A1:C85"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7764,6 +7833,17 @@
         <v>4.4534</v>
       </c>
     </row>
+    <row r="85" spans="1:3" ht="16" customHeight="1">
+      <c r="A85" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B85" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C85" s="3">
+        <v>3.768</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7772,7 +7852,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C84"/>
+  <dimension ref="A1:C85"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8704,6 +8784,17 @@
         <v>7.8947</v>
       </c>
     </row>
+    <row r="85" spans="1:3" ht="16" customHeight="1">
+      <c r="A85" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B85" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C85" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8712,7 +8803,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C84"/>
+  <dimension ref="A1:C85"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9644,6 +9735,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="85" spans="1:3" ht="16" customHeight="1">
+      <c r="A85" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B85" s="3">
+        <v>1.99</v>
+      </c>
+      <c r="C85" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9652,7 +9754,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C84"/>
+  <dimension ref="A1:C85"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10584,6 +10686,17 @@
         <v>2.2667</v>
       </c>
     </row>
+    <row r="85" spans="1:3" ht="16" customHeight="1">
+      <c r="A85" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B85" s="3">
+        <v>2.89</v>
+      </c>
+      <c r="C85" s="3">
+        <v>2.96</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10592,7 +10705,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C84"/>
+  <dimension ref="A1:C85"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11524,6 +11637,17 @@
         <v>2.7333</v>
       </c>
     </row>
+    <row r="85" spans="1:3" ht="16" customHeight="1">
+      <c r="A85" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B85" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C85" s="3">
+        <v>6.6667</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11532,7 +11656,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C84"/>
+  <dimension ref="A1:C85"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12464,6 +12588,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="85" spans="1:3" ht="16" customHeight="1">
+      <c r="A85" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B85" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C85" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-09-01 15:15:54
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2623" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2645" uniqueCount="89">
   <si>
     <t>Date</t>
   </si>
@@ -289,6 +289,9 @@
   </si>
   <si>
     <t>2026-08-31</t>
+  </si>
+  <si>
+    <t>2026-09-01</t>
   </si>
 </sst>
 </file>
@@ -1195,7 +1198,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C85"/>
+  <dimension ref="A1:C86"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2138,6 +2141,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="86" spans="1:3" ht="16" customHeight="1">
+      <c r="A86" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B86" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C86" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2146,7 +2160,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C85"/>
+  <dimension ref="A1:C86"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3089,6 +3103,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="86" spans="1:3" ht="16" customHeight="1">
+      <c r="A86" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B86" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C86" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3097,7 +3122,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C85"/>
+  <dimension ref="A1:C86"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4040,6 +4065,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="86" spans="1:3" ht="16" customHeight="1">
+      <c r="A86" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B86" s="3">
+        <v>0.88</v>
+      </c>
+      <c r="C86" s="3">
+        <v>0.8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4048,7 +4084,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C85"/>
+  <dimension ref="A1:C86"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4991,6 +5027,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="86" spans="1:3" ht="16" customHeight="1">
+      <c r="A86" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B86" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C86" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4999,7 +5046,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C85"/>
+  <dimension ref="A1:C86"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5942,6 +5989,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="86" spans="1:3" ht="16" customHeight="1">
+      <c r="A86" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B86" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C86" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5950,7 +6008,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C85"/>
+  <dimension ref="A1:C86"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6893,6 +6951,17 @@
         <v>6</v>
       </c>
     </row>
+    <row r="86" spans="1:3" ht="16" customHeight="1">
+      <c r="A86" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B86" s="3">
+        <v>3.75</v>
+      </c>
+      <c r="C86" s="3">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6901,7 +6970,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C85"/>
+  <dimension ref="A1:C86"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7844,6 +7913,17 @@
         <v>3.768</v>
       </c>
     </row>
+    <row r="86" spans="1:3" ht="16" customHeight="1">
+      <c r="A86" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B86" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C86" s="3">
+        <v>4.6213</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7852,7 +7932,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C85"/>
+  <dimension ref="A1:C86"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8795,6 +8875,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="86" spans="1:3" ht="16" customHeight="1">
+      <c r="A86" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B86" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C86" s="3">
+        <v>4.075</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8803,7 +8894,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C85"/>
+  <dimension ref="A1:C86"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9746,6 +9837,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="86" spans="1:3" ht="16" customHeight="1">
+      <c r="A86" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B86" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C86" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9754,7 +9856,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C85"/>
+  <dimension ref="A1:C86"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10697,6 +10799,17 @@
         <v>2.96</v>
       </c>
     </row>
+    <row r="86" spans="1:3" ht="16" customHeight="1">
+      <c r="A86" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B86" s="3">
+        <v>2.79</v>
+      </c>
+      <c r="C86" s="3">
+        <v>3.092</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10705,7 +10818,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C85"/>
+  <dimension ref="A1:C86"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11648,6 +11761,17 @@
         <v>6.6667</v>
       </c>
     </row>
+    <row r="86" spans="1:3" ht="16" customHeight="1">
+      <c r="A86" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B86" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C86" s="3">
+        <v>3.1733</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11656,7 +11780,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C85"/>
+  <dimension ref="A1:C86"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12599,6 +12723,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="86" spans="1:3" ht="16" customHeight="1">
+      <c r="A86" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B86" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C86" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-09-02 14:46:09
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2645" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2665" uniqueCount="90">
   <si>
     <t>Date</t>
   </si>
@@ -292,6 +292,9 @@
   </si>
   <si>
     <t>2026-09-01</t>
+  </si>
+  <si>
+    <t>2026-09-02</t>
   </si>
 </sst>
 </file>
@@ -1198,7 +1201,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C86"/>
+  <dimension ref="A1:C87"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2152,6 +2155,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="87" spans="1:3" ht="16" customHeight="1">
+      <c r="A87" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B87" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C87" s="3">
+        <v>7.89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2160,7 +2174,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C86"/>
+  <dimension ref="A1:C87"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3114,6 +3128,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="87" spans="1:3" ht="16" customHeight="1">
+      <c r="A87" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B87" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C87" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3122,7 +3147,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C86"/>
+  <dimension ref="A1:C87"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4076,6 +4101,17 @@
         <v>0.8</v>
       </c>
     </row>
+    <row r="87" spans="1:3" ht="16" customHeight="1">
+      <c r="A87" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B87" s="3">
+        <v>0.88</v>
+      </c>
+      <c r="C87" s="3">
+        <v>0.99</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4084,7 +4120,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C86"/>
+  <dimension ref="A1:C87"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5038,6 +5074,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="87" spans="1:3" ht="16" customHeight="1">
+      <c r="A87" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B87" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C87" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5046,7 +5093,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C86"/>
+  <dimension ref="A1:C87"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6000,6 +6047,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="87" spans="1:3" ht="16" customHeight="1">
+      <c r="A87" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B87" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C87" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6008,7 +6066,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C86"/>
+  <dimension ref="A1:C87"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6962,6 +7020,17 @@
         <v>6</v>
       </c>
     </row>
+    <row r="87" spans="1:3" ht="16" customHeight="1">
+      <c r="A87" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B87" s="3">
+        <v>3.75</v>
+      </c>
+      <c r="C87" s="3">
+        <v>6.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6970,7 +7039,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C86"/>
+  <dimension ref="A1:C87"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7924,6 +7993,17 @@
         <v>4.6213</v>
       </c>
     </row>
+    <row r="87" spans="1:3" ht="16" customHeight="1">
+      <c r="A87" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B87" s="3">
+        <v>4.47</v>
+      </c>
+      <c r="C87" s="3">
+        <v>5.4667</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7932,7 +8012,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C86"/>
+  <dimension ref="A1:C87"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8886,6 +8966,17 @@
         <v>4.075</v>
       </c>
     </row>
+    <row r="87" spans="1:3" ht="16" customHeight="1">
+      <c r="A87" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B87" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C87" s="3">
+        <v>4.59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8894,7 +8985,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C86"/>
+  <dimension ref="A1:C87"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9848,6 +9939,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="87" spans="1:3" ht="16" customHeight="1">
+      <c r="A87" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B87" s="3">
+        <v>2.29</v>
+      </c>
+      <c r="C87" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9856,7 +9958,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C86"/>
+  <dimension ref="A1:C87"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10810,6 +10912,17 @@
         <v>3.092</v>
       </c>
     </row>
+    <row r="87" spans="1:3" ht="16" customHeight="1">
+      <c r="A87" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B87" s="3">
+        <v>2.79</v>
+      </c>
+      <c r="C87" s="3">
+        <v>2.2667</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10818,7 +10931,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C86"/>
+  <dimension ref="A1:C87"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11772,6 +11885,17 @@
         <v>3.1733</v>
       </c>
     </row>
+    <row r="87" spans="1:3" ht="16" customHeight="1">
+      <c r="A87" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B87" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C87" s="3">
+        <v>3.19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11780,7 +11904,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C86"/>
+  <dimension ref="A1:C87"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12734,6 +12858,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="87" spans="1:3" ht="16" customHeight="1">
+      <c r="A87" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B87" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C87" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-09-04 14:36:09
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2665" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2687" uniqueCount="91">
   <si>
     <t>Date</t>
   </si>
@@ -295,6 +295,9 @@
   </si>
   <si>
     <t>2026-09-02</t>
+  </si>
+  <si>
+    <t>2026-09-04</t>
   </si>
 </sst>
 </file>
@@ -1201,7 +1204,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C87"/>
+  <dimension ref="A1:C88"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2166,6 +2169,17 @@
         <v>7.89</v>
       </c>
     </row>
+    <row r="88" spans="1:3" ht="16" customHeight="1">
+      <c r="A88" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B88" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C88" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2174,7 +2188,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C87"/>
+  <dimension ref="A1:C88"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3139,6 +3153,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="88" spans="1:3" ht="16" customHeight="1">
+      <c r="A88" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B88" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C88" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3147,7 +3172,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C87"/>
+  <dimension ref="A1:C88"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4112,6 +4137,17 @@
         <v>0.99</v>
       </c>
     </row>
+    <row r="88" spans="1:3" ht="16" customHeight="1">
+      <c r="A88" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B88" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C88" s="3">
+        <v>0.8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4120,7 +4156,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C87"/>
+  <dimension ref="A1:C88"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5085,6 +5121,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="88" spans="1:3" ht="16" customHeight="1">
+      <c r="A88" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B88" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C88" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5093,7 +5140,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C87"/>
+  <dimension ref="A1:C88"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6058,6 +6105,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="88" spans="1:3" ht="16" customHeight="1">
+      <c r="A88" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B88" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C88" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6066,7 +6124,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C87"/>
+  <dimension ref="A1:C88"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7031,6 +7089,17 @@
         <v>6.79</v>
       </c>
     </row>
+    <row r="88" spans="1:3" ht="16" customHeight="1">
+      <c r="A88" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B88" s="3">
+        <v>3.75</v>
+      </c>
+      <c r="C88" s="3">
+        <v>6.625</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7039,7 +7108,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C87"/>
+  <dimension ref="A1:C88"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8004,6 +8073,17 @@
         <v>5.4667</v>
       </c>
     </row>
+    <row r="88" spans="1:3" ht="16" customHeight="1">
+      <c r="A88" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B88" s="3">
+        <v>4.47</v>
+      </c>
+      <c r="C88" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8012,7 +8092,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C87"/>
+  <dimension ref="A1:C88"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8977,6 +9057,17 @@
         <v>4.59</v>
       </c>
     </row>
+    <row r="88" spans="1:3" ht="16" customHeight="1">
+      <c r="A88" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B88" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C88" s="3">
+        <v>4.59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8985,7 +9076,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C87"/>
+  <dimension ref="A1:C88"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9950,6 +10041,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="88" spans="1:3" ht="16" customHeight="1">
+      <c r="A88" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B88" s="3">
+        <v>2.29</v>
+      </c>
+      <c r="C88" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9958,7 +10060,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C87"/>
+  <dimension ref="A1:C88"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10923,6 +11025,17 @@
         <v>2.2667</v>
       </c>
     </row>
+    <row r="88" spans="1:3" ht="16" customHeight="1">
+      <c r="A88" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B88" s="3">
+        <v>2.79</v>
+      </c>
+      <c r="C88" s="3">
+        <v>2.2667</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10931,7 +11044,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C87"/>
+  <dimension ref="A1:C88"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11896,6 +12009,17 @@
         <v>3.19</v>
       </c>
     </row>
+    <row r="88" spans="1:3" ht="16" customHeight="1">
+      <c r="A88" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B88" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C88" s="3">
+        <v>3.19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11904,7 +12028,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C87"/>
+  <dimension ref="A1:C88"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12869,6 +12993,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="88" spans="1:3" ht="16" customHeight="1">
+      <c r="A88" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B88" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C88" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-09-05 13:35:28
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2687" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2707" uniqueCount="92">
   <si>
     <t>Date</t>
   </si>
@@ -298,6 +298,9 @@
   </si>
   <si>
     <t>2026-09-04</t>
+  </si>
+  <si>
+    <t>2026-09-05</t>
   </si>
 </sst>
 </file>
@@ -1204,7 +1207,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C88"/>
+  <dimension ref="A1:C89"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2180,6 +2183,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="89" spans="1:3" ht="16" customHeight="1">
+      <c r="A89" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B89" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C89" s="3">
+        <v>7.89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2188,7 +2202,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C88"/>
+  <dimension ref="A1:C89"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3164,6 +3178,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="89" spans="1:3" ht="16" customHeight="1">
+      <c r="A89" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B89" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C89" s="3">
+        <v>2.39</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3172,7 +3197,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C88"/>
+  <dimension ref="A1:C89"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4148,6 +4173,17 @@
         <v>0.8</v>
       </c>
     </row>
+    <row r="89" spans="1:3" ht="16" customHeight="1">
+      <c r="A89" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B89" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C89" s="3">
+        <v>1.09</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4156,7 +4192,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C88"/>
+  <dimension ref="A1:C89"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5132,6 +5168,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="89" spans="1:3" ht="16" customHeight="1">
+      <c r="A89" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B89" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C89" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5140,7 +5187,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C88"/>
+  <dimension ref="A1:C89"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6116,6 +6163,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="89" spans="1:3" ht="16" customHeight="1">
+      <c r="A89" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B89" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C89" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6124,7 +6182,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C88"/>
+  <dimension ref="A1:C89"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7100,6 +7158,17 @@
         <v>6.625</v>
       </c>
     </row>
+    <row r="89" spans="1:3" ht="16" customHeight="1">
+      <c r="A89" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B89" s="3">
+        <v>3.75</v>
+      </c>
+      <c r="C89" s="3">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7108,7 +7177,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C88"/>
+  <dimension ref="A1:C89"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8084,6 +8153,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="89" spans="1:3" ht="16" customHeight="1">
+      <c r="A89" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B89" s="3">
+        <v>4.47</v>
+      </c>
+      <c r="C89" s="3">
+        <v>3.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8092,7 +8172,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C88"/>
+  <dimension ref="A1:C89"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9068,6 +9148,17 @@
         <v>4.59</v>
       </c>
     </row>
+    <row r="89" spans="1:3" ht="16" customHeight="1">
+      <c r="A89" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B89" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C89" s="3">
+        <v>4.59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9076,7 +9167,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C88"/>
+  <dimension ref="A1:C89"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10052,6 +10143,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="89" spans="1:3" ht="16" customHeight="1">
+      <c r="A89" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B89" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C89" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10060,7 +10162,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C88"/>
+  <dimension ref="A1:C89"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11036,6 +11138,17 @@
         <v>2.2667</v>
       </c>
     </row>
+    <row r="89" spans="1:3" ht="16" customHeight="1">
+      <c r="A89" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B89" s="3">
+        <v>2.79</v>
+      </c>
+      <c r="C89" s="3">
+        <v>3.172</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11044,7 +11157,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C88"/>
+  <dimension ref="A1:C89"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12020,6 +12133,17 @@
         <v>3.19</v>
       </c>
     </row>
+    <row r="89" spans="1:3" ht="16" customHeight="1">
+      <c r="A89" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B89" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C89" s="3">
+        <v>3.0933</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12028,7 +12152,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C88"/>
+  <dimension ref="A1:C89"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13004,6 +13128,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="89" spans="1:3" ht="16" customHeight="1">
+      <c r="A89" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B89" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C89" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-09-06 13:50:26
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2707" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2727" uniqueCount="93">
   <si>
     <t>Date</t>
   </si>
@@ -301,6 +301,9 @@
   </si>
   <si>
     <t>2026-09-05</t>
+  </si>
+  <si>
+    <t>2026-09-06</t>
   </si>
 </sst>
 </file>
@@ -1207,7 +1210,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C89"/>
+  <dimension ref="A1:C90"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2194,6 +2197,17 @@
         <v>7.89</v>
       </c>
     </row>
+    <row r="90" spans="1:3" ht="16" customHeight="1">
+      <c r="A90" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B90" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C90" s="3">
+        <v>7.89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2202,7 +2216,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C89"/>
+  <dimension ref="A1:C90"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3189,6 +3203,17 @@
         <v>2.39</v>
       </c>
     </row>
+    <row r="90" spans="1:3" ht="16" customHeight="1">
+      <c r="A90" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B90" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C90" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3197,7 +3222,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C89"/>
+  <dimension ref="A1:C90"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4184,6 +4209,17 @@
         <v>1.09</v>
       </c>
     </row>
+    <row r="90" spans="1:3" ht="16" customHeight="1">
+      <c r="A90" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B90" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C90" s="3">
+        <v>0.8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4192,7 +4228,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C89"/>
+  <dimension ref="A1:C90"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5179,6 +5215,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="90" spans="1:3" ht="16" customHeight="1">
+      <c r="A90" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B90" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C90" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5187,7 +5234,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C89"/>
+  <dimension ref="A1:C90"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6174,6 +6221,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="90" spans="1:3" ht="16" customHeight="1">
+      <c r="A90" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B90" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C90" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6182,7 +6240,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C89"/>
+  <dimension ref="A1:C90"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7169,6 +7227,17 @@
         <v>6</v>
       </c>
     </row>
+    <row r="90" spans="1:3" ht="16" customHeight="1">
+      <c r="A90" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B90" s="3">
+        <v>3.75</v>
+      </c>
+      <c r="C90" s="3">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7177,7 +7246,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C89"/>
+  <dimension ref="A1:C90"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8164,6 +8233,17 @@
         <v>3.79</v>
       </c>
     </row>
+    <row r="90" spans="1:3" ht="16" customHeight="1">
+      <c r="A90" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B90" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C90" s="3">
+        <v>4.476</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8172,7 +8252,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C89"/>
+  <dimension ref="A1:C90"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9159,6 +9239,17 @@
         <v>4.59</v>
       </c>
     </row>
+    <row r="90" spans="1:3" ht="16" customHeight="1">
+      <c r="A90" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B90" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C90" s="3">
+        <v>4.59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9167,7 +9258,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C89"/>
+  <dimension ref="A1:C90"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10154,6 +10245,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="90" spans="1:3" ht="16" customHeight="1">
+      <c r="A90" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B90" s="3">
+        <v>2.29</v>
+      </c>
+      <c r="C90" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10162,7 +10264,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C89"/>
+  <dimension ref="A1:C90"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11149,6 +11251,17 @@
         <v>3.172</v>
       </c>
     </row>
+    <row r="90" spans="1:3" ht="16" customHeight="1">
+      <c r="A90" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B90" s="3">
+        <v>2.79</v>
+      </c>
+      <c r="C90" s="3">
+        <v>2.2667</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11157,7 +11270,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C89"/>
+  <dimension ref="A1:C90"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12144,6 +12257,17 @@
         <v>3.0933</v>
       </c>
     </row>
+    <row r="90" spans="1:3" ht="16" customHeight="1">
+      <c r="A90" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B90" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C90" s="3">
+        <v>3.1867</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12152,7 +12276,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C89"/>
+  <dimension ref="A1:C90"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13139,6 +13263,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="90" spans="1:3" ht="16" customHeight="1">
+      <c r="A90" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B90" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C90" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-09-07 16:08:55
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2727" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2746" uniqueCount="94">
   <si>
     <t>Date</t>
   </si>
@@ -305,6 +305,9 @@
   <si>
     <t>2026-09-06</t>
   </si>
+  <si>
+    <t>2026-09-07</t>
+  </si>
 </sst>
 </file>
 
@@ -420,7 +423,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -440,7 +443,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -463,7 +466,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -483,7 +486,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -506,7 +509,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -526,7 +529,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -549,7 +552,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -569,7 +572,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -635,7 +638,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -655,7 +658,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -678,7 +681,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -698,7 +701,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -721,7 +724,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -741,7 +744,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -764,7 +767,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -784,7 +787,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -807,7 +810,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -827,7 +830,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -850,7 +853,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>86923</xdr:colOff>
+      <xdr:colOff>79889</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -870,7 +873,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8011723" cy="4368113"/>
+          <a:ext cx="8004689" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1210,7 +1213,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C90"/>
+  <dimension ref="A1:C91"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2208,6 +2211,17 @@
         <v>7.89</v>
       </c>
     </row>
+    <row r="91" spans="1:3" ht="16" customHeight="1">
+      <c r="A91" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B91" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C91" s="3">
+        <v>7.89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2216,7 +2230,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C90"/>
+  <dimension ref="A1:C91"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3214,6 +3228,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="91" spans="1:3" ht="16" customHeight="1">
+      <c r="A91" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B91" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C91" s="3">
+        <v>2.39</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3222,7 +3247,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C90"/>
+  <dimension ref="A1:C91"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4220,6 +4245,17 @@
         <v>0.8</v>
       </c>
     </row>
+    <row r="91" spans="1:3" ht="16" customHeight="1">
+      <c r="A91" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B91" s="3">
+        <v>0.92</v>
+      </c>
+      <c r="C91" s="3">
+        <v>1.09</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4228,7 +4264,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C90"/>
+  <dimension ref="A1:C91"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5226,6 +5262,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="91" spans="1:3" ht="16" customHeight="1">
+      <c r="A91" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B91" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C91" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5234,7 +5281,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C90"/>
+  <dimension ref="A1:C91"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6232,6 +6279,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="91" spans="1:3" ht="16" customHeight="1">
+      <c r="A91" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B91" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C91" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6240,7 +6298,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C90"/>
+  <dimension ref="A1:C91"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7238,6 +7296,17 @@
         <v>6</v>
       </c>
     </row>
+    <row r="91" spans="1:3" ht="16" customHeight="1">
+      <c r="A91" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B91" s="3">
+        <v>3.75</v>
+      </c>
+      <c r="C91" s="3">
+        <v>6.625</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7246,7 +7315,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C90"/>
+  <dimension ref="A1:C91"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8244,6 +8313,17 @@
         <v>4.476</v>
       </c>
     </row>
+    <row r="91" spans="1:3" ht="16" customHeight="1">
+      <c r="A91" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B91" s="3">
+        <v>4.47</v>
+      </c>
+      <c r="C91" s="3">
+        <v>5.3333</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8252,7 +8332,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C90"/>
+  <dimension ref="A1:C91"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9250,6 +9330,17 @@
         <v>4.59</v>
       </c>
     </row>
+    <row r="91" spans="1:3" ht="16" customHeight="1">
+      <c r="A91" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B91" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C91" s="3">
+        <v>4.59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9258,7 +9349,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C90"/>
+  <dimension ref="A1:C91"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10256,6 +10347,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="91" spans="1:3" ht="16" customHeight="1">
+      <c r="A91" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B91" s="3">
+        <v>2.29</v>
+      </c>
+      <c r="C91" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10264,7 +10366,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C90"/>
+  <dimension ref="A1:C91"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11262,6 +11364,17 @@
         <v>2.2667</v>
       </c>
     </row>
+    <row r="91" spans="1:3" ht="16" customHeight="1">
+      <c r="A91" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B91" s="3">
+        <v>2.79</v>
+      </c>
+      <c r="C91" s="3">
+        <v>2.9853</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11270,7 +11383,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C90"/>
+  <dimension ref="A1:C91"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12268,6 +12381,17 @@
         <v>3.1867</v>
       </c>
     </row>
+    <row r="91" spans="1:3" ht="16" customHeight="1">
+      <c r="A91" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B91" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C91" s="3">
+        <v>3.19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12276,7 +12400,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C90"/>
+  <dimension ref="A1:C91"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13274,6 +13398,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="91" spans="1:3" ht="16" customHeight="1">
+      <c r="A91" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B91" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C91" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-09-08 14:48:30
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2746" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2766" uniqueCount="95">
   <si>
     <t>Date</t>
   </si>
@@ -308,6 +308,9 @@
   <si>
     <t>2026-09-07</t>
   </si>
+  <si>
+    <t>2026-09-08</t>
+  </si>
 </sst>
 </file>
 
@@ -423,7 +426,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -443,7 +446,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -466,7 +469,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -486,7 +489,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -509,7 +512,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -529,7 +532,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -552,7 +555,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -572,7 +575,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -638,7 +641,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -658,7 +661,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -681,7 +684,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -701,7 +704,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -724,7 +727,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -744,7 +747,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -767,7 +770,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -787,7 +790,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -810,7 +813,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -830,7 +833,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -853,7 +856,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>79889</xdr:colOff>
+      <xdr:colOff>86923</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>139013</xdr:rowOff>
     </xdr:to>
@@ -873,7 +876,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="3952875" y="0"/>
-          <a:ext cx="8004689" cy="4368113"/>
+          <a:ext cx="8011723" cy="4368113"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1213,7 +1216,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C91"/>
+  <dimension ref="A1:C92"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2222,6 +2225,17 @@
         <v>7.89</v>
       </c>
     </row>
+    <row r="92" spans="1:3" ht="16" customHeight="1">
+      <c r="A92" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B92" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C92" s="3">
+        <v>7.89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2230,7 +2244,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C91"/>
+  <dimension ref="A1:C92"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3239,6 +3253,17 @@
         <v>2.39</v>
       </c>
     </row>
+    <row r="92" spans="1:3" ht="16" customHeight="1">
+      <c r="A92" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B92" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C92" s="3">
+        <v>2.39</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3247,7 +3272,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C91"/>
+  <dimension ref="A1:C92"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4256,6 +4281,17 @@
         <v>1.09</v>
       </c>
     </row>
+    <row r="92" spans="1:3" ht="16" customHeight="1">
+      <c r="A92" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B92" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C92" s="3">
+        <v>1.09</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4264,7 +4300,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C91"/>
+  <dimension ref="A1:C92"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5273,6 +5309,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="92" spans="1:3" ht="16" customHeight="1">
+      <c r="A92" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B92" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C92" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5281,7 +5328,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C91"/>
+  <dimension ref="A1:C92"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6290,6 +6337,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="92" spans="1:3" ht="16" customHeight="1">
+      <c r="A92" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B92" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C92" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6298,7 +6356,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C91"/>
+  <dimension ref="A1:C92"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7307,6 +7365,17 @@
         <v>6.625</v>
       </c>
     </row>
+    <row r="92" spans="1:3" ht="16" customHeight="1">
+      <c r="A92" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B92" s="3">
+        <v>3.75</v>
+      </c>
+      <c r="C92" s="3">
+        <v>6.625</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7315,7 +7384,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C91"/>
+  <dimension ref="A1:C92"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8324,6 +8393,17 @@
         <v>5.3333</v>
       </c>
     </row>
+    <row r="92" spans="1:3" ht="16" customHeight="1">
+      <c r="A92" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B92" s="3">
+        <v>4.47</v>
+      </c>
+      <c r="C92" s="3">
+        <v>5.96</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8332,7 +8412,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C91"/>
+  <dimension ref="A1:C92"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9341,6 +9421,17 @@
         <v>4.59</v>
       </c>
     </row>
+    <row r="92" spans="1:3" ht="16" customHeight="1">
+      <c r="A92" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B92" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C92" s="3">
+        <v>4.59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9349,7 +9440,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C91"/>
+  <dimension ref="A1:C92"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10358,6 +10449,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="92" spans="1:3" ht="16" customHeight="1">
+      <c r="A92" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B92" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C92" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10366,7 +10468,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C91"/>
+  <dimension ref="A1:C92"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11375,6 +11477,17 @@
         <v>2.9853</v>
       </c>
     </row>
+    <row r="92" spans="1:3" ht="16" customHeight="1">
+      <c r="A92" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B92" s="3">
+        <v>2.79</v>
+      </c>
+      <c r="C92" s="3">
+        <v>3.49</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11383,7 +11496,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C91"/>
+  <dimension ref="A1:C92"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12392,6 +12505,17 @@
         <v>3.19</v>
       </c>
     </row>
+    <row r="92" spans="1:3" ht="16" customHeight="1">
+      <c r="A92" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B92" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C92" s="3">
+        <v>3.19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12400,7 +12524,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C91"/>
+  <dimension ref="A1:C92"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13409,6 +13533,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="92" spans="1:3" ht="16" customHeight="1">
+      <c r="A92" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B92" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C92" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-09-09 14:51:09
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2766" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2787" uniqueCount="96">
   <si>
     <t>Date</t>
   </si>
@@ -310,6 +310,9 @@
   </si>
   <si>
     <t>2026-09-08</t>
+  </si>
+  <si>
+    <t>2026-09-09</t>
   </si>
 </sst>
 </file>
@@ -1216,7 +1219,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C92"/>
+  <dimension ref="A1:C93"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2236,6 +2239,17 @@
         <v>7.89</v>
       </c>
     </row>
+    <row r="93" spans="1:3" ht="16" customHeight="1">
+      <c r="A93" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B93" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C93" s="3">
+        <v>7.89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2244,7 +2258,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C92"/>
+  <dimension ref="A1:C93"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3264,6 +3278,17 @@
         <v>2.39</v>
       </c>
     </row>
+    <row r="93" spans="1:3" ht="16" customHeight="1">
+      <c r="A93" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B93" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C93" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3272,7 +3297,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C92"/>
+  <dimension ref="A1:C93"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4292,6 +4317,17 @@
         <v>1.09</v>
       </c>
     </row>
+    <row r="93" spans="1:3" ht="16" customHeight="1">
+      <c r="A93" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B93" s="3">
+        <v>0.92</v>
+      </c>
+      <c r="C93" s="3">
+        <v>1.09</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4300,7 +4336,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C92"/>
+  <dimension ref="A1:C93"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5320,6 +5356,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="93" spans="1:3" ht="16" customHeight="1">
+      <c r="A93" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B93" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C93" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5328,7 +5375,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C92"/>
+  <dimension ref="A1:C93"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6348,6 +6395,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="93" spans="1:3" ht="16" customHeight="1">
+      <c r="A93" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B93" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C93" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6356,7 +6414,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C92"/>
+  <dimension ref="A1:C93"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7376,6 +7434,17 @@
         <v>6.625</v>
       </c>
     </row>
+    <row r="93" spans="1:3" ht="16" customHeight="1">
+      <c r="A93" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B93" s="3">
+        <v>3.75</v>
+      </c>
+      <c r="C93" s="3">
+        <v>6.625</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7384,7 +7453,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C92"/>
+  <dimension ref="A1:C93"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8404,6 +8473,17 @@
         <v>5.96</v>
       </c>
     </row>
+    <row r="93" spans="1:3" ht="16" customHeight="1">
+      <c r="A93" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B93" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C93" s="3">
+        <v>3.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8412,7 +8492,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C92"/>
+  <dimension ref="A1:C93"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9432,6 +9512,17 @@
         <v>4.59</v>
       </c>
     </row>
+    <row r="93" spans="1:3" ht="16" customHeight="1">
+      <c r="A93" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B93" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C93" s="3">
+        <v>3.6842</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9440,7 +9531,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C92"/>
+  <dimension ref="A1:C93"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10460,6 +10551,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="93" spans="1:3" ht="16" customHeight="1">
+      <c r="A93" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B93" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C93" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10468,7 +10570,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C92"/>
+  <dimension ref="A1:C93"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11488,6 +11590,17 @@
         <v>3.49</v>
       </c>
     </row>
+    <row r="93" spans="1:3" ht="16" customHeight="1">
+      <c r="A93" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B93" s="3">
+        <v>2.79</v>
+      </c>
+      <c r="C93" s="3">
+        <v>3.49</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11496,7 +11609,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C92"/>
+  <dimension ref="A1:C93"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12516,6 +12629,17 @@
         <v>3.19</v>
       </c>
     </row>
+    <row r="93" spans="1:3" ht="16" customHeight="1">
+      <c r="A93" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B93" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C93" s="3">
+        <v>3.19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12524,7 +12648,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C92"/>
+  <dimension ref="A1:C93"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13544,6 +13668,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="93" spans="1:3" ht="16" customHeight="1">
+      <c r="A93" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B93" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C93" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-09-10 14:41:03
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2787" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2808" uniqueCount="97">
   <si>
     <t>Date</t>
   </si>
@@ -313,6 +313,9 @@
   </si>
   <si>
     <t>2026-09-09</t>
+  </si>
+  <si>
+    <t>2026-09-10</t>
   </si>
 </sst>
 </file>
@@ -1219,7 +1222,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C93"/>
+  <dimension ref="A1:C94"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2250,6 +2253,17 @@
         <v>7.89</v>
       </c>
     </row>
+    <row r="94" spans="1:3" ht="16" customHeight="1">
+      <c r="A94" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B94" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C94" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2258,7 +2272,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C93"/>
+  <dimension ref="A1:C94"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3289,6 +3303,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="94" spans="1:3" ht="16" customHeight="1">
+      <c r="A94" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B94" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C94" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3297,7 +3322,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C93"/>
+  <dimension ref="A1:C94"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4328,6 +4353,17 @@
         <v>1.09</v>
       </c>
     </row>
+    <row r="94" spans="1:3" ht="16" customHeight="1">
+      <c r="A94" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B94" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C94" s="3">
+        <v>1.09</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4336,7 +4372,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C93"/>
+  <dimension ref="A1:C94"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5367,6 +5403,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="94" spans="1:3" ht="16" customHeight="1">
+      <c r="A94" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B94" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C94" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5375,7 +5422,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C93"/>
+  <dimension ref="A1:C94"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6406,6 +6453,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="94" spans="1:3" ht="16" customHeight="1">
+      <c r="A94" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B94" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C94" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6414,7 +6472,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C93"/>
+  <dimension ref="A1:C94"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7445,6 +7503,17 @@
         <v>6.625</v>
       </c>
     </row>
+    <row r="94" spans="1:3" ht="16" customHeight="1">
+      <c r="A94" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B94" s="3">
+        <v>3.75</v>
+      </c>
+      <c r="C94" s="3">
+        <v>6.625</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7453,7 +7522,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C93"/>
+  <dimension ref="A1:C94"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8484,6 +8553,17 @@
         <v>3.79</v>
       </c>
     </row>
+    <row r="94" spans="1:3" ht="16" customHeight="1">
+      <c r="A94" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B94" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C94" s="3">
+        <v>5.0653</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8492,7 +8572,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C93"/>
+  <dimension ref="A1:C94"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9523,6 +9603,17 @@
         <v>3.6842</v>
       </c>
     </row>
+    <row r="94" spans="1:3" ht="16" customHeight="1">
+      <c r="A94" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B94" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C94" s="3">
+        <v>4.59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9531,7 +9622,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C93"/>
+  <dimension ref="A1:C94"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10562,6 +10653,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="94" spans="1:3" ht="16" customHeight="1">
+      <c r="A94" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B94" s="3">
+        <v>1.99</v>
+      </c>
+      <c r="C94" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10570,7 +10672,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C93"/>
+  <dimension ref="A1:C94"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11601,6 +11703,17 @@
         <v>3.49</v>
       </c>
     </row>
+    <row r="94" spans="1:3" ht="16" customHeight="1">
+      <c r="A94" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B94" s="3">
+        <v>2.79</v>
+      </c>
+      <c r="C94" s="3">
+        <v>3.49</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11609,7 +11722,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C93"/>
+  <dimension ref="A1:C94"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12640,6 +12753,17 @@
         <v>3.19</v>
       </c>
     </row>
+    <row r="94" spans="1:3" ht="16" customHeight="1">
+      <c r="A94" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B94" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C94" s="3">
+        <v>3.9333</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12648,7 +12772,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C93"/>
+  <dimension ref="A1:C94"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13679,6 +13803,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="94" spans="1:3" ht="16" customHeight="1">
+      <c r="A94" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B94" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C94" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-09-11 14:39:43
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2808" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2827" uniqueCount="98">
   <si>
     <t>Date</t>
   </si>
@@ -316,6 +316,9 @@
   </si>
   <si>
     <t>2026-09-10</t>
+  </si>
+  <si>
+    <t>2026-09-11</t>
   </si>
 </sst>
 </file>
@@ -1222,7 +1225,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C94"/>
+  <dimension ref="A1:C95"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2264,6 +2267,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="95" spans="1:3" ht="16" customHeight="1">
+      <c r="A95" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B95" s="3">
+        <v>7.5</v>
+      </c>
+      <c r="C95" s="3">
+        <v>7.89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2272,7 +2286,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C94"/>
+  <dimension ref="A1:C95"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3314,6 +3328,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="95" spans="1:3" ht="16" customHeight="1">
+      <c r="A95" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B95" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C95" s="3">
+        <v>2.39</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3322,7 +3347,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C94"/>
+  <dimension ref="A1:C95"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4364,6 +4389,17 @@
         <v>1.09</v>
       </c>
     </row>
+    <row r="95" spans="1:3" ht="16" customHeight="1">
+      <c r="A95" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B95" s="3">
+        <v>0.92</v>
+      </c>
+      <c r="C95" s="3">
+        <v>1.09</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4372,7 +4408,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C94"/>
+  <dimension ref="A1:C95"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5414,6 +5450,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="95" spans="1:3" ht="16" customHeight="1">
+      <c r="A95" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C95" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5422,7 +5469,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C94"/>
+  <dimension ref="A1:C95"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6464,6 +6511,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="95" spans="1:3" ht="16" customHeight="1">
+      <c r="A95" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C95" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6472,7 +6530,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C94"/>
+  <dimension ref="A1:C95"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7514,6 +7572,17 @@
         <v>6.625</v>
       </c>
     </row>
+    <row r="95" spans="1:3" ht="16" customHeight="1">
+      <c r="A95" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B95" s="3">
+        <v>3.75</v>
+      </c>
+      <c r="C95" s="3">
+        <v>6.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7522,7 +7591,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C94"/>
+  <dimension ref="A1:C95"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8564,6 +8633,17 @@
         <v>5.0653</v>
       </c>
     </row>
+    <row r="95" spans="1:3" ht="16" customHeight="1">
+      <c r="A95" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B95" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C95" s="3">
+        <v>3.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8572,7 +8652,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C94"/>
+  <dimension ref="A1:C95"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9614,6 +9694,17 @@
         <v>4.59</v>
       </c>
     </row>
+    <row r="95" spans="1:3" ht="16" customHeight="1">
+      <c r="A95" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B95" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C95" s="3">
+        <v>3.6842</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9622,7 +9713,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C94"/>
+  <dimension ref="A1:C95"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10664,6 +10755,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="95" spans="1:3" ht="16" customHeight="1">
+      <c r="A95" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C95" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10672,7 +10774,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C94"/>
+  <dimension ref="A1:C95"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11714,6 +11816,17 @@
         <v>3.49</v>
       </c>
     </row>
+    <row r="95" spans="1:3" ht="16" customHeight="1">
+      <c r="A95" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B95" s="3">
+        <v>2.79</v>
+      </c>
+      <c r="C95" s="3">
+        <v>2.2667</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11722,7 +11835,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C94"/>
+  <dimension ref="A1:C95"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12764,6 +12877,17 @@
         <v>3.9333</v>
       </c>
     </row>
+    <row r="95" spans="1:3" ht="16" customHeight="1">
+      <c r="A95" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B95" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C95" s="3">
+        <v>3.19</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12772,7 +12896,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C94"/>
+  <dimension ref="A1:C95"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13814,6 +13938,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="95" spans="1:3" ht="16" customHeight="1">
+      <c r="A95" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C95" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Update GPU prices and charts - 2026-09-12 13:47:45
</commit_message>
<xml_diff>
--- a/output/GPU_Price_Trends.xlsx
+++ b/output/GPU_Price_Trends.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2827" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2845" uniqueCount="99">
   <si>
     <t>Date</t>
   </si>
@@ -319,6 +319,9 @@
   </si>
   <si>
     <t>2026-09-11</t>
+  </si>
+  <si>
+    <t>2026-09-12</t>
   </si>
 </sst>
 </file>
@@ -1225,7 +1228,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C95"/>
+  <dimension ref="A1:C96"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2278,6 +2281,17 @@
         <v>7.89</v>
       </c>
     </row>
+    <row r="96" spans="1:3" ht="16" customHeight="1">
+      <c r="A96" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B96" s="3">
+        <v>7.5</v>
+      </c>
+      <c r="C96" s="3">
+        <v>7.89</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2286,7 +2300,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C95"/>
+  <dimension ref="A1:C96"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -3339,6 +3353,17 @@
         <v>2.39</v>
       </c>
     </row>
+    <row r="96" spans="1:3" ht="16" customHeight="1">
+      <c r="A96" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B96" s="3">
+        <v>2.99</v>
+      </c>
+      <c r="C96" s="3">
+        <v>2.39</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3347,7 +3372,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C95"/>
+  <dimension ref="A1:C96"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -4400,6 +4425,17 @@
         <v>1.09</v>
       </c>
     </row>
+    <row r="96" spans="1:3" ht="16" customHeight="1">
+      <c r="A96" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B96" s="3">
+        <v>0.97</v>
+      </c>
+      <c r="C96" s="3">
+        <v>1.09</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4408,7 +4444,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C95"/>
+  <dimension ref="A1:C96"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -5461,6 +5497,17 @@
         <v>0.9115</v>
       </c>
     </row>
+    <row r="96" spans="1:3" ht="16" customHeight="1">
+      <c r="A96" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B96" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C96" s="3">
+        <v>0.9115</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -5469,7 +5516,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C95"/>
+  <dimension ref="A1:C96"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -6522,6 +6569,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="96" spans="1:3" ht="16" customHeight="1">
+      <c r="A96" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B96" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C96" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -6530,7 +6588,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C95"/>
+  <dimension ref="A1:C96"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -7583,6 +7641,17 @@
         <v>6.79</v>
       </c>
     </row>
+    <row r="96" spans="1:3" ht="16" customHeight="1">
+      <c r="A96" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B96" s="3">
+        <v>6</v>
+      </c>
+      <c r="C96" s="3">
+        <v>6.79</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -7591,7 +7660,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C95"/>
+  <dimension ref="A1:C96"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -8644,6 +8713,17 @@
         <v>3.79</v>
       </c>
     </row>
+    <row r="96" spans="1:3" ht="16" customHeight="1">
+      <c r="A96" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B96" s="3">
+        <v>3.43</v>
+      </c>
+      <c r="C96" s="3">
+        <v>4.1973</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -8652,7 +8732,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C95"/>
+  <dimension ref="A1:C96"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -9705,6 +9785,17 @@
         <v>3.6842</v>
       </c>
     </row>
+    <row r="96" spans="1:3" ht="16" customHeight="1">
+      <c r="A96" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B96" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C96" s="3">
+        <v>3.6842</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -9713,7 +9804,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C95"/>
+  <dimension ref="A1:C96"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -10766,6 +10857,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="96" spans="1:3" ht="16" customHeight="1">
+      <c r="A96" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B96" s="3">
+        <v>2.29</v>
+      </c>
+      <c r="C96" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -10774,7 +10876,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C95"/>
+  <dimension ref="A1:C96"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -11827,6 +11929,17 @@
         <v>2.2667</v>
       </c>
     </row>
+    <row r="96" spans="1:3" ht="16" customHeight="1">
+      <c r="A96" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B96" s="3">
+        <v>2.79</v>
+      </c>
+      <c r="C96" s="3">
+        <v>3.49</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -11835,7 +11948,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C95"/>
+  <dimension ref="A1:C96"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -12888,6 +13001,17 @@
         <v>3.19</v>
       </c>
     </row>
+    <row r="96" spans="1:3" ht="16" customHeight="1">
+      <c r="A96" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B96" s="3">
+        <v>3.11</v>
+      </c>
+      <c r="C96" s="3">
+        <v>3.1467</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -12896,7 +13020,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C95"/>
+  <dimension ref="A1:C96"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -13949,6 +14073,17 @@
         <v>4</v>
       </c>
     </row>
+    <row r="96" spans="1:3" ht="16" customHeight="1">
+      <c r="A96" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B96" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C96" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>